<commit_message>
added to where to collect page
</commit_message>
<xml_diff>
--- a/Power BI V2/Data/DuckDataBI.xlsx
+++ b/Power BI V2/Data/DuckDataBI.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\allan\Documents\DS_Projects\Analyducks\Power BI V2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31A87CF4-9E73-484D-B6EB-5B3AF44AEF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51FE7DB0-B1FE-4512-8A0E-C41683856723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{C5D2797D-B188-49E6-A37E-A541A2C853B5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C5D2797D-B188-49E6-A37E-A541A2C853B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1906" uniqueCount="654">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2022" uniqueCount="708">
   <si>
     <t>Duck</t>
   </si>
@@ -2001,13 +2002,175 @@
   </si>
   <si>
     <t>30th bday</t>
+  </si>
+  <si>
+    <t>Shop Name</t>
+  </si>
+  <si>
+    <t>Link</t>
+  </si>
+  <si>
+    <t>City</t>
+  </si>
+  <si>
+    <t>State</t>
+  </si>
+  <si>
+    <t>Country</t>
+  </si>
+  <si>
+    <t>Address</t>
+  </si>
+  <si>
+    <t>2222 Michelson Dr ste 200, Irvine, CA 92612</t>
+  </si>
+  <si>
+    <t>Irvine</t>
+  </si>
+  <si>
+    <t>https://www.duckdonuts.com/menu/2222-michelson-dr-ste-200-irvine-ca-92612</t>
+  </si>
+  <si>
+    <t>Ammon</t>
+  </si>
+  <si>
+    <t>ID</t>
+  </si>
+  <si>
+    <t>2675 E Sunnyside Rd, Ammon, ID 83406</t>
+  </si>
+  <si>
+    <t>https://www.duckdonuts.com/menu/2675-e-sunnyside-rd-ammon-id-83406</t>
+  </si>
+  <si>
+    <t>The Pretty Duckling</t>
+  </si>
+  <si>
+    <t>Traders Village San Antonio, 9333 SW Loop 410, San Antonio, TX 78242</t>
+  </si>
+  <si>
+    <t>San Antonio</t>
+  </si>
+  <si>
+    <t>https://the-pretty-duckling-5879.myshopify.com/</t>
+  </si>
+  <si>
+    <t>Air Force Museum Store</t>
+  </si>
+  <si>
+    <t>1100 Spaatz St, Dayton, OH 45431</t>
+  </si>
+  <si>
+    <t>https://shop.airforcemuseumfoundation.org/</t>
+  </si>
+  <si>
+    <t>Duck Yeah!</t>
+  </si>
+  <si>
+    <t>131 The Island Dr #9102, Pigeon Forge, TN 37863</t>
+  </si>
+  <si>
+    <t>https://islandinpigeonforge.com/poi/duck-yeah</t>
+  </si>
+  <si>
+    <t>The Tipsy Duck Parlor</t>
+  </si>
+  <si>
+    <t>58 Hypolita St side entrance, St. Augustine, FL 32084</t>
+  </si>
+  <si>
+    <t>St. Augustine</t>
+  </si>
+  <si>
+    <t>http://thetipsyduckparlor.com/</t>
+  </si>
+  <si>
+    <t>Munchies &amp; Memories</t>
+  </si>
+  <si>
+    <t>1312 Boardwalk, Ocean City, NJ 08226</t>
+  </si>
+  <si>
+    <t>http://my.matterport.com/show/?m=77ZfU3QVQH7&amp;play=1</t>
+  </si>
+  <si>
+    <t>507 Main St, Chatham, MA 02633</t>
+  </si>
+  <si>
+    <t>http://www.ducksinthewindow.com/</t>
+  </si>
+  <si>
+    <t>51 Main St, Essex, CT 06426</t>
+  </si>
+  <si>
+    <t>http://www.essexduck.com/</t>
+  </si>
+  <si>
+    <t>Le Petit Duck Shoppe</t>
+  </si>
+  <si>
+    <t>24 Saint-Paul St W, Montreal, Quebec H2Y 1Y7, Canada</t>
+  </si>
+  <si>
+    <t>https://www.lepetitduckshoppe.com/en/</t>
+  </si>
+  <si>
+    <t>Rubber Ducky Café</t>
+  </si>
+  <si>
+    <t>20 Windmill St, Millers Point NSW 2000, Australia</t>
+  </si>
+  <si>
+    <t>https://www.rubberduckycatering.com.au/</t>
+  </si>
+  <si>
+    <t>Cafe Pamplemousse</t>
+  </si>
+  <si>
+    <t>Miyagi</t>
+  </si>
+  <si>
+    <t>Japan, 〒980-0021 Miyagi, Sendai, Aoba Ward, Central, 1 Chome−7−18 日吉第一ビル 3F</t>
+  </si>
+  <si>
+    <t>https://akashia-mitsubachi-youhoujou.com/pamplemousse-sendai/</t>
+  </si>
+  <si>
+    <t>Ducks</t>
+  </si>
+  <si>
+    <t>Kamajura</t>
+  </si>
+  <si>
+    <t>2 Chome-12-36 Komachi, Kamakura, Kanagawa 248-0006, Japan</t>
+  </si>
+  <si>
+    <t>https://duuucks.com/</t>
+  </si>
+  <si>
+    <t>466-4 Zaimokucho, Shimogyo Ward, Kyoto, 600-8146, Japan</t>
+  </si>
+  <si>
+    <t>Ducks Kyoto</t>
+  </si>
+  <si>
+    <t>Myoraku-49 Uji, Kyoto 611-0021, Japan</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/ducks_kyoto_uji?igsh=MWhrdHUzb2o2dWJxbA==</t>
+  </si>
+  <si>
+    <t>Mayya</t>
+  </si>
+  <si>
+    <t>AUS</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2036,6 +2199,12 @@
       <color rgb="FF1F1F1F"/>
       <name val="Google Sans"/>
     </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Roboto"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -2063,7 +2232,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="16">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -2260,11 +2429,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF356854"/>
+      </right>
+      <top style="medium">
+        <color rgb="FF284E3F"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FF284E3F"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FF356854"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="49">
+  <cellXfs count="51">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2399,18 +2594,50 @@
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="16" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="22">
+  <dxfs count="23">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Roboto"/>
+        <scheme val="none"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FF356854"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -3180,30 +3407,48 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{02C6EB19-C16E-4C45-82D8-19820ABC0444}" name="Table1" displayName="Table1" ref="A1:R213" totalsRowShown="0" headerRowDxfId="21" dataDxfId="19" headerRowBorderDxfId="20" tableBorderDxfId="18" totalsRowBorderDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{02C6EB19-C16E-4C45-82D8-19820ABC0444}" name="Table1" displayName="Table1" ref="A1:R213" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19" totalsRowBorderDxfId="18">
   <autoFilter ref="A1:R213" xr:uid="{02C6EB19-C16E-4C45-82D8-19820ABC0444}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R210">
     <sortCondition descending="1" ref="O1:O210"/>
   </sortState>
   <tableColumns count="18">
-    <tableColumn id="1" xr3:uid="{DAB72840-701E-4BFE-934E-006A0ACCCC07}" name="Duck" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{95778B1D-6921-4D32-BBED-0B7F6DA673E5}" name="Name" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{5CB584A0-AB21-47EC-BB26-A11CDCBA20B8}" name="Purchase_Method" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{2884C836-2B85-4AEC-953E-9A14BE8936FE}" name="Purchase_Retailer" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{C904F914-DD34-45E9-850D-B2E396106458}" name="Purchase_City" dataDxfId="12"/>
-    <tableColumn id="6" xr3:uid="{FEBDDC27-D50D-4BCA-B9B7-17F1FDD0B1D7}" name="Purchase_State" dataDxfId="11"/>
-    <tableColumn id="7" xr3:uid="{4BBE096A-92FC-440B-8588-F38EF87162C5}" name="Purchase_Country" dataDxfId="10"/>
-    <tableColumn id="8" xr3:uid="{0D0B4DAC-55B0-4274-A3A3-0CD059EA68D4}" name="ISO_Code" dataDxfId="9"/>
+    <tableColumn id="1" xr3:uid="{DAB72840-701E-4BFE-934E-006A0ACCCC07}" name="Duck" dataDxfId="17"/>
+    <tableColumn id="2" xr3:uid="{95778B1D-6921-4D32-BBED-0B7F6DA673E5}" name="Name" dataDxfId="16"/>
+    <tableColumn id="3" xr3:uid="{5CB584A0-AB21-47EC-BB26-A11CDCBA20B8}" name="Purchase_Method" dataDxfId="15"/>
+    <tableColumn id="4" xr3:uid="{2884C836-2B85-4AEC-953E-9A14BE8936FE}" name="Purchase_Retailer" dataDxfId="14"/>
+    <tableColumn id="5" xr3:uid="{C904F914-DD34-45E9-850D-B2E396106458}" name="Purchase_City" dataDxfId="13"/>
+    <tableColumn id="6" xr3:uid="{FEBDDC27-D50D-4BCA-B9B7-17F1FDD0B1D7}" name="Purchase_State" dataDxfId="12"/>
+    <tableColumn id="7" xr3:uid="{4BBE096A-92FC-440B-8588-F38EF87162C5}" name="Purchase_Country" dataDxfId="11"/>
+    <tableColumn id="8" xr3:uid="{0D0B4DAC-55B0-4274-A3A3-0CD059EA68D4}" name="ISO_Code" dataDxfId="10"/>
     <tableColumn id="9" xr3:uid="{8BFACE2C-57C0-4357-8182-3CE92E40FAC3}" name="Date_Bought"/>
-    <tableColumn id="10" xr3:uid="{924D7501-EE54-48E6-BEE2-5AE397C7A9C0}" name="Latitude" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{F329274D-D590-4D27-86A0-3E8011EF0C8C}" name="Longitude" dataDxfId="7"/>
-    <tableColumn id="12" xr3:uid="{05DCF6FC-1B42-45B5-86A3-DDAB58638C63}" name="About Me" dataDxfId="6"/>
-    <tableColumn id="13" xr3:uid="{EE9A6E60-CA0E-4A9C-8BBF-097878C7AF60}" name="Buyer" dataDxfId="5"/>
-    <tableColumn id="14" xr3:uid="{540CA30D-4816-4B0D-82BB-4F8C99387E34}" name="Quantity" dataDxfId="4"/>
-    <tableColumn id="15" xr3:uid="{9F16EC51-0EC3-458C-8E55-786DA138218A}" name="Total_Weight" dataDxfId="3"/>
-    <tableColumn id="16" xr3:uid="{C9172612-09C9-4AC2-8A2F-560BA19CD352}" name="Height" dataDxfId="2"/>
-    <tableColumn id="17" xr3:uid="{33C2FD9D-E982-4BA4-8A22-F0BF9B0962EB}" name="Width" dataDxfId="1"/>
-    <tableColumn id="18" xr3:uid="{8CA455AB-F612-49A5-887B-A3A90BE4297E}" name="Length" dataDxfId="0"/>
+    <tableColumn id="10" xr3:uid="{924D7501-EE54-48E6-BEE2-5AE397C7A9C0}" name="Latitude" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{F329274D-D590-4D27-86A0-3E8011EF0C8C}" name="Longitude" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{05DCF6FC-1B42-45B5-86A3-DDAB58638C63}" name="About Me" dataDxfId="7"/>
+    <tableColumn id="13" xr3:uid="{EE9A6E60-CA0E-4A9C-8BBF-097878C7AF60}" name="Buyer" dataDxfId="6"/>
+    <tableColumn id="14" xr3:uid="{540CA30D-4816-4B0D-82BB-4F8C99387E34}" name="Quantity" dataDxfId="5"/>
+    <tableColumn id="15" xr3:uid="{9F16EC51-0EC3-458C-8E55-786DA138218A}" name="Total_Weight" dataDxfId="4"/>
+    <tableColumn id="16" xr3:uid="{C9172612-09C9-4AC2-8A2F-560BA19CD352}" name="Height" dataDxfId="3"/>
+    <tableColumn id="17" xr3:uid="{33C2FD9D-E982-4BA4-8A22-F0BF9B0962EB}" name="Width" dataDxfId="2"/>
+    <tableColumn id="18" xr3:uid="{8CA455AB-F612-49A5-887B-A3A90BE4297E}" name="Length" dataDxfId="1"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}" name="Locations" displayName="Locations" ref="A1:I16" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:I16" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{63C32DA5-9104-488A-B085-36DB395683F0}" name="Shop Name"/>
+    <tableColumn id="2" xr3:uid="{9DB5CA49-9344-4EA7-9D0B-03CF697CEB1E}" name="City"/>
+    <tableColumn id="3" xr3:uid="{286EA7E5-4452-4F0D-8C78-04BAE27F1F3A}" name="State"/>
+    <tableColumn id="4" xr3:uid="{88EF38A1-9615-4274-861E-67CCBFC84894}" name="Country"/>
+    <tableColumn id="5" xr3:uid="{B4761F6B-E138-4A60-B88D-220C59CAF85D}" name="ISO_Code"/>
+    <tableColumn id="6" xr3:uid="{B7DA27AC-1D08-4160-81AC-A2AF96AF118C}" name="Latitude"/>
+    <tableColumn id="7" xr3:uid="{CB3D8E42-6E43-4860-B22A-448900D42EA4}" name="Longitude"/>
+    <tableColumn id="8" xr3:uid="{55805FF1-912D-4EA1-BC97-A9AC858273FB}" name="Link"/>
+    <tableColumn id="9" xr3:uid="{05CD9E28-5179-4E3C-9FE0-67152446D074}" name="Address"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -9658,7 +9903,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="53.4" thickBot="1">
+    <row r="111" spans="1:18" ht="40.200000000000003" thickBot="1">
       <c r="A111" s="13" t="s">
         <v>586</v>
       </c>
@@ -12160,7 +12405,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="156" spans="1:18" ht="53.4" thickBot="1">
+    <row r="156" spans="1:18" ht="40.200000000000003" thickBot="1">
       <c r="A156" s="12" t="s">
         <v>18</v>
       </c>
@@ -15259,16 +15504,24 @@
       <c r="J212" s="40"/>
       <c r="K212" s="40"/>
       <c r="L212" s="43"/>
-      <c r="M212" s="41"/>
+      <c r="M212" s="41" t="s">
+        <v>129</v>
+      </c>
       <c r="N212" s="40">
         <v>1</v>
       </c>
       <c r="O212" s="40">
         <v>110</v>
       </c>
-      <c r="P212" s="40"/>
-      <c r="Q212" s="40"/>
-      <c r="R212" s="44"/>
+      <c r="P212" s="40">
+        <v>0</v>
+      </c>
+      <c r="Q212" s="40">
+        <v>0</v>
+      </c>
+      <c r="R212" s="44">
+        <v>0</v>
+      </c>
     </row>
     <row r="213" spans="1:18" ht="26.4">
       <c r="A213" s="39" t="s">
@@ -15283,20 +15536,515 @@
       <c r="F213" s="41"/>
       <c r="G213" s="41"/>
       <c r="H213" s="41"/>
-      <c r="I213" s="46"/>
       <c r="J213" s="40"/>
       <c r="K213" s="40"/>
       <c r="L213" s="43"/>
-      <c r="M213" s="41"/>
+      <c r="M213" s="41" t="s">
+        <v>706</v>
+      </c>
       <c r="N213" s="40">
         <v>1</v>
       </c>
       <c r="O213" s="40">
         <v>20</v>
       </c>
-      <c r="P213" s="47"/>
-      <c r="Q213" s="47"/>
-      <c r="R213" s="48"/>
+      <c r="P213" s="46">
+        <v>0</v>
+      </c>
+      <c r="Q213" s="46">
+        <v>0</v>
+      </c>
+      <c r="R213" s="47">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E690491F-A75A-44CD-AF5E-964C98F48B1D}">
+  <dimension ref="A1:I16"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.44140625" customWidth="1"/>
+    <col min="3" max="3" width="16.33203125" customWidth="1"/>
+    <col min="4" max="4" width="18.77734375" customWidth="1"/>
+    <col min="5" max="5" width="15.6640625" customWidth="1"/>
+    <col min="6" max="6" width="10" customWidth="1"/>
+    <col min="7" max="7" width="15.21875" customWidth="1"/>
+    <col min="9" max="9" width="36.33203125" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="15" thickBot="1">
+      <c r="A1" s="48" t="s">
+        <v>654</v>
+      </c>
+      <c r="B1" s="48" t="s">
+        <v>656</v>
+      </c>
+      <c r="C1" s="48" t="s">
+        <v>657</v>
+      </c>
+      <c r="D1" s="48" t="s">
+        <v>658</v>
+      </c>
+      <c r="E1" s="48" t="s">
+        <v>7</v>
+      </c>
+      <c r="F1" s="48" t="s">
+        <v>9</v>
+      </c>
+      <c r="G1" s="48" t="s">
+        <v>10</v>
+      </c>
+      <c r="H1" s="49" t="s">
+        <v>655</v>
+      </c>
+      <c r="I1" s="50" t="s">
+        <v>659</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9">
+      <c r="A2" t="s">
+        <v>358</v>
+      </c>
+      <c r="B2" t="s">
+        <v>661</v>
+      </c>
+      <c r="C2" t="s">
+        <v>425</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2">
+        <v>33.800500368778202</v>
+      </c>
+      <c r="G2">
+        <v>-117.910289903156</v>
+      </c>
+      <c r="H2" t="s">
+        <v>662</v>
+      </c>
+      <c r="I2" t="s">
+        <v>660</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" t="s">
+        <v>358</v>
+      </c>
+      <c r="B3" t="s">
+        <v>663</v>
+      </c>
+      <c r="C3" t="s">
+        <v>664</v>
+      </c>
+      <c r="D3" t="s">
+        <v>24</v>
+      </c>
+      <c r="E3" t="s">
+        <v>24</v>
+      </c>
+      <c r="F3">
+        <v>44.035644759071097</v>
+      </c>
+      <c r="G3">
+        <v>-112.211925491803</v>
+      </c>
+      <c r="H3" t="s">
+        <v>666</v>
+      </c>
+      <c r="I3" t="s">
+        <v>665</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9">
+      <c r="A4" t="s">
+        <v>667</v>
+      </c>
+      <c r="B4" t="s">
+        <v>669</v>
+      </c>
+      <c r="C4" t="s">
+        <v>248</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4">
+        <v>29.463383242077299</v>
+      </c>
+      <c r="G4">
+        <v>-98.335771519372102</v>
+      </c>
+      <c r="H4" t="s">
+        <v>670</v>
+      </c>
+      <c r="I4" t="s">
+        <v>668</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" t="s">
+        <v>671</v>
+      </c>
+      <c r="B5" t="s">
+        <v>641</v>
+      </c>
+      <c r="C5" t="s">
+        <v>642</v>
+      </c>
+      <c r="D5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E5" t="s">
+        <v>24</v>
+      </c>
+      <c r="F5">
+        <v>41.094637674232096</v>
+      </c>
+      <c r="G5">
+        <v>-83.661265806926806</v>
+      </c>
+      <c r="H5" t="s">
+        <v>673</v>
+      </c>
+      <c r="I5" t="s">
+        <v>672</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" t="s">
+        <v>674</v>
+      </c>
+      <c r="B6" t="s">
+        <v>406</v>
+      </c>
+      <c r="C6" t="s">
+        <v>407</v>
+      </c>
+      <c r="D6" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" t="s">
+        <v>24</v>
+      </c>
+      <c r="F6">
+        <v>36.756490311024898</v>
+      </c>
+      <c r="G6">
+        <v>-83.490698324576201</v>
+      </c>
+      <c r="H6" t="s">
+        <v>676</v>
+      </c>
+      <c r="I6" t="s">
+        <v>675</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" t="s">
+        <v>677</v>
+      </c>
+      <c r="B7" t="s">
+        <v>679</v>
+      </c>
+      <c r="C7" t="s">
+        <v>43</v>
+      </c>
+      <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7">
+        <v>30.237048753086999</v>
+      </c>
+      <c r="G7">
+        <v>-81.302681827847593</v>
+      </c>
+      <c r="H7" t="s">
+        <v>680</v>
+      </c>
+      <c r="I7" t="s">
+        <v>678</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" t="s">
+        <v>681</v>
+      </c>
+      <c r="B8" t="s">
+        <v>636</v>
+      </c>
+      <c r="C8" t="s">
+        <v>266</v>
+      </c>
+      <c r="D8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" t="s">
+        <v>24</v>
+      </c>
+      <c r="F8">
+        <v>39.382735466011901</v>
+      </c>
+      <c r="G8">
+        <v>-74.075276886054397</v>
+      </c>
+      <c r="H8" t="s">
+        <v>683</v>
+      </c>
+      <c r="I8" t="s">
+        <v>682</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" t="s">
+        <v>334</v>
+      </c>
+      <c r="B9" t="s">
+        <v>335</v>
+      </c>
+      <c r="C9" t="s">
+        <v>102</v>
+      </c>
+      <c r="D9" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" t="s">
+        <v>24</v>
+      </c>
+      <c r="F9">
+        <v>41.762380767075598</v>
+      </c>
+      <c r="G9">
+        <v>-69.964720011453906</v>
+      </c>
+      <c r="H9" t="s">
+        <v>685</v>
+      </c>
+      <c r="I9" t="s">
+        <v>684</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" t="s">
+        <v>227</v>
+      </c>
+      <c r="B10" t="s">
+        <v>228</v>
+      </c>
+      <c r="C10" t="s">
+        <v>221</v>
+      </c>
+      <c r="D10" t="s">
+        <v>24</v>
+      </c>
+      <c r="E10" t="s">
+        <v>24</v>
+      </c>
+      <c r="F10">
+        <v>41.424445068117102</v>
+      </c>
+      <c r="G10">
+        <v>-72.242355034482003</v>
+      </c>
+      <c r="H10" t="s">
+        <v>687</v>
+      </c>
+      <c r="I10" t="s">
+        <v>686</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" t="s">
+        <v>688</v>
+      </c>
+      <c r="B11" t="s">
+        <v>175</v>
+      </c>
+      <c r="C11" t="s">
+        <v>88</v>
+      </c>
+      <c r="D11" t="s">
+        <v>177</v>
+      </c>
+      <c r="E11" t="s">
+        <v>177</v>
+      </c>
+      <c r="F11">
+        <v>46.059205916812402</v>
+      </c>
+      <c r="G11">
+        <v>-73.751381735450806</v>
+      </c>
+      <c r="H11" t="s">
+        <v>690</v>
+      </c>
+      <c r="I11" t="s">
+        <v>689</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" t="s">
+        <v>691</v>
+      </c>
+      <c r="B12" t="s">
+        <v>416</v>
+      </c>
+      <c r="C12" t="s">
+        <v>88</v>
+      </c>
+      <c r="D12" t="s">
+        <v>707</v>
+      </c>
+      <c r="E12" t="s">
+        <v>707</v>
+      </c>
+      <c r="F12">
+        <v>-31.301920080120301</v>
+      </c>
+      <c r="G12">
+        <v>150.92525148123801</v>
+      </c>
+      <c r="H12" t="s">
+        <v>693</v>
+      </c>
+      <c r="I12" t="s">
+        <v>692</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" t="s">
+        <v>694</v>
+      </c>
+      <c r="B13" t="s">
+        <v>695</v>
+      </c>
+      <c r="C13" t="s">
+        <v>88</v>
+      </c>
+      <c r="D13" t="s">
+        <v>593</v>
+      </c>
+      <c r="E13" t="s">
+        <v>593</v>
+      </c>
+      <c r="F13">
+        <v>38.266755018307997</v>
+      </c>
+      <c r="G13">
+        <v>140.87937309661501</v>
+      </c>
+      <c r="H13" t="s">
+        <v>697</v>
+      </c>
+      <c r="I13" t="s">
+        <v>696</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" t="s">
+        <v>698</v>
+      </c>
+      <c r="B14" t="s">
+        <v>699</v>
+      </c>
+      <c r="C14" t="s">
+        <v>88</v>
+      </c>
+      <c r="D14" t="s">
+        <v>593</v>
+      </c>
+      <c r="E14" t="s">
+        <v>593</v>
+      </c>
+      <c r="F14">
+        <v>35.339815509095899</v>
+      </c>
+      <c r="G14">
+        <v>139.596898521875</v>
+      </c>
+      <c r="H14" t="s">
+        <v>701</v>
+      </c>
+      <c r="I14" t="s">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" t="s">
+        <v>698</v>
+      </c>
+      <c r="B15" t="s">
+        <v>591</v>
+      </c>
+      <c r="C15" t="s">
+        <v>88</v>
+      </c>
+      <c r="D15" t="s">
+        <v>593</v>
+      </c>
+      <c r="E15" t="s">
+        <v>593</v>
+      </c>
+      <c r="F15">
+        <v>35.012908784767497</v>
+      </c>
+      <c r="G15">
+        <v>135.81056759424601</v>
+      </c>
+      <c r="H15" t="s">
+        <v>701</v>
+      </c>
+      <c r="I15" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" t="s">
+        <v>703</v>
+      </c>
+      <c r="B16" t="s">
+        <v>591</v>
+      </c>
+      <c r="C16" t="s">
+        <v>88</v>
+      </c>
+      <c r="D16" t="s">
+        <v>593</v>
+      </c>
+      <c r="E16" t="s">
+        <v>593</v>
+      </c>
+      <c r="F16">
+        <v>34.905430873998398</v>
+      </c>
+      <c r="G16">
+        <v>135.820807959506</v>
+      </c>
+      <c r="H16" t="s">
+        <v>705</v>
+      </c>
+      <c r="I16" t="s">
+        <v>704</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
added charts to locations page
</commit_message>
<xml_diff>
--- a/Power BI V2/Data/DuckDataBI.xlsx
+++ b/Power BI V2/Data/DuckDataBI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\allan\Documents\DS_Projects\Analyducks\Power BI V2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51FE7DB0-B1FE-4512-8A0E-C41683856723}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3464A9F1-1664-4BAA-867F-9400654F9461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C5D2797D-B188-49E6-A37E-A541A2C853B5}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2022" uniqueCount="708">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2022" uniqueCount="709">
   <si>
     <t>Duck</t>
   </si>
@@ -2164,6 +2164,9 @@
   </si>
   <si>
     <t>AUS</t>
+  </si>
+  <si>
+    <t>Australia</t>
   </si>
 </sst>
 </file>
@@ -14001,7 +14004,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="185" spans="1:18" ht="53.4" thickBot="1">
+    <row r="185" spans="1:18" ht="40.200000000000003" thickBot="1">
       <c r="A185" s="13" t="s">
         <v>204</v>
       </c>
@@ -15883,7 +15886,7 @@
         <v>88</v>
       </c>
       <c r="D11" t="s">
-        <v>177</v>
+        <v>172</v>
       </c>
       <c r="E11" t="s">
         <v>177</v>
@@ -15912,7 +15915,7 @@
         <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>707</v>
+        <v>708</v>
       </c>
       <c r="E12" t="s">
         <v>707</v>
@@ -15941,7 +15944,7 @@
         <v>88</v>
       </c>
       <c r="D13" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E13" t="s">
         <v>593</v>
@@ -15970,7 +15973,7 @@
         <v>88</v>
       </c>
       <c r="D14" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E14" t="s">
         <v>593</v>
@@ -15999,7 +16002,7 @@
         <v>88</v>
       </c>
       <c r="D15" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E15" t="s">
         <v>593</v>
@@ -16028,7 +16031,7 @@
         <v>88</v>
       </c>
       <c r="D16" t="s">
-        <v>593</v>
+        <v>592</v>
       </c>
       <c r="E16" t="s">
         <v>593</v>

</xml_diff>

<commit_message>
added stores to list
</commit_message>
<xml_diff>
--- a/Power BI V2/Data/DuckDataBI.xlsx
+++ b/Power BI V2/Data/DuckDataBI.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\allan\Documents\DS_Projects\Analyducks\Power BI V2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3464A9F1-1664-4BAA-867F-9400654F9461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8D2EF2-4EF3-43CD-B1CB-B5E89A60D41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C5D2797D-B188-49E6-A37E-A541A2C853B5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
+    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2022" uniqueCount="709">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2458" uniqueCount="954">
   <si>
     <t>Duck</t>
   </si>
@@ -2022,27 +2023,6 @@
     <t>Address</t>
   </si>
   <si>
-    <t>2222 Michelson Dr ste 200, Irvine, CA 92612</t>
-  </si>
-  <si>
-    <t>Irvine</t>
-  </si>
-  <si>
-    <t>https://www.duckdonuts.com/menu/2222-michelson-dr-ste-200-irvine-ca-92612</t>
-  </si>
-  <si>
-    <t>Ammon</t>
-  </si>
-  <si>
-    <t>ID</t>
-  </si>
-  <si>
-    <t>2675 E Sunnyside Rd, Ammon, ID 83406</t>
-  </si>
-  <si>
-    <t>https://www.duckdonuts.com/menu/2675-e-sunnyside-rd-ammon-id-83406</t>
-  </si>
-  <si>
     <t>The Pretty Duckling</t>
   </si>
   <si>
@@ -2167,6 +2147,762 @@
   </si>
   <si>
     <t>Australia</t>
+  </si>
+  <si>
+    <t>Store Name</t>
+  </si>
+  <si>
+    <t>Walmart</t>
+  </si>
+  <si>
+    <t>Duck House</t>
+  </si>
+  <si>
+    <t>San Pedro 251, 5550000 Puerto Varas, Los Lagos, Chile</t>
+  </si>
+  <si>
+    <t>Los Lagos</t>
+  </si>
+  <si>
+    <t>Chile</t>
+  </si>
+  <si>
+    <t>http://www.duckhouse.cl/</t>
+  </si>
+  <si>
+    <t>Geronimo de Alderete 324, 4920551 Pucon, Pucón, Araucanía, Chile</t>
+  </si>
+  <si>
+    <t>Araucanía</t>
+  </si>
+  <si>
+    <t>Av. Italia 1300, 7501451 Providencia, Región Metropolitana, Chile</t>
+  </si>
+  <si>
+    <t>Región Metropolitana</t>
+  </si>
+  <si>
+    <t>1480 Gulf Rd, Point Roberts, WA 98281</t>
+  </si>
+  <si>
+    <t>The Rubber Duck Museum</t>
+  </si>
+  <si>
+    <t>https://www.therubberduckmuseum.com/</t>
+  </si>
+  <si>
+    <t>Point Roberts</t>
+  </si>
+  <si>
+    <t>Quacker Gift Shop Grand Lake</t>
+  </si>
+  <si>
+    <t>http://www.quackergiftshop.com/</t>
+  </si>
+  <si>
+    <t>1034 Grand Ave, Grand Lake, CO 80447</t>
+  </si>
+  <si>
+    <t>Grand Lake</t>
+  </si>
+  <si>
+    <t>CO</t>
+  </si>
+  <si>
+    <t>CHL</t>
+  </si>
+  <si>
+    <t>45 Central Square, Santa Rosa Beach, FL 32459</t>
+  </si>
+  <si>
+    <t>Santa Rosa Beach</t>
+  </si>
+  <si>
+    <t>Duckies Shop of Fun</t>
+  </si>
+  <si>
+    <t>http://www.shopduckies.com/</t>
+  </si>
+  <si>
+    <t>460 Main St, Bethlehem, PA 18018</t>
+  </si>
+  <si>
+    <t>Foo Foo Shoppe</t>
+  </si>
+  <si>
+    <t>Bethlehem</t>
+  </si>
+  <si>
+    <t>https://www.thefoofooshoppe.com/</t>
+  </si>
+  <si>
+    <t>14260 Frazee Rd, Divernon, IL 62530</t>
+  </si>
+  <si>
+    <t>World of Ducks</t>
+  </si>
+  <si>
+    <t>Divernon</t>
+  </si>
+  <si>
+    <t>IL</t>
+  </si>
+  <si>
+    <t>https://worldofducks.com/</t>
+  </si>
+  <si>
+    <t>Duck Duck Scoop</t>
+  </si>
+  <si>
+    <t>5801 Golden Triangle Blvd Suite 106, Fort Worth, TX 76244</t>
+  </si>
+  <si>
+    <t>Fort Worth</t>
+  </si>
+  <si>
+    <t>https://www.duckduckscoop.com/</t>
+  </si>
+  <si>
+    <t>King's Bowling</t>
+  </si>
+  <si>
+    <t>Connie's Bath Shack</t>
+  </si>
+  <si>
+    <t>211 Midway St, Spring, TX 77373</t>
+  </si>
+  <si>
+    <t>Spring</t>
+  </si>
+  <si>
+    <t>https://conniesbathshack.square.site/</t>
+  </si>
+  <si>
+    <t>24 Main St N, New London, MN 56273</t>
+  </si>
+  <si>
+    <t>Lucky Duck</t>
+  </si>
+  <si>
+    <t>New London</t>
+  </si>
+  <si>
+    <t>http://www.luckyduckmn.com/</t>
+  </si>
+  <si>
+    <t>Pier 39 Level, Beach St, San Francisco, CA 94133</t>
+  </si>
+  <si>
+    <t>KWAK</t>
+  </si>
+  <si>
+    <t>San Francisco</t>
+  </si>
+  <si>
+    <t>https://kwaksf.com/</t>
+  </si>
+  <si>
+    <t>DUCK!</t>
+  </si>
+  <si>
+    <t>Eagan</t>
+  </si>
+  <si>
+    <t>1004 Diffley Rd #500, Eagan, MN 55123</t>
+  </si>
+  <si>
+    <t>https://www.duck-us.com/</t>
+  </si>
+  <si>
+    <t>Snap Quack Pop</t>
+  </si>
+  <si>
+    <t>Portsmouth</t>
+  </si>
+  <si>
+    <t>https://www.snapquackpop.com/</t>
+  </si>
+  <si>
+    <t>123 Market St, Portsmouth, NH 03801</t>
+  </si>
+  <si>
+    <t>Wicked Ducks, LLC</t>
+  </si>
+  <si>
+    <t>27 Atlantic Ave, Marblehead, MA 01945</t>
+  </si>
+  <si>
+    <t>https://wicked-ducks.com/</t>
+  </si>
+  <si>
+    <t>The Lucky Duck Shop, LLC</t>
+  </si>
+  <si>
+    <t>2626 Central Ave Unit A, St. Petersburg, FL 33712</t>
+  </si>
+  <si>
+    <t>St. Petersburg</t>
+  </si>
+  <si>
+    <t>https://luckyduckshop.com/</t>
+  </si>
+  <si>
+    <t>Madeira Duck Store</t>
+  </si>
+  <si>
+    <t>Funchal</t>
+  </si>
+  <si>
+    <t>Portugal</t>
+  </si>
+  <si>
+    <t>Rua de Santa Maria 85, 9060-291 Funchal, Portugal</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/Madeira-Duck-Store-375771529713427/https://www.instagram.com/madeiraduckstore/?hl=pt</t>
+  </si>
+  <si>
+    <t>Largo Dr. António de Sousa Macedo 6B, 1100-321 Lisboa, Portugal</t>
+  </si>
+  <si>
+    <t>Lisbon Duck Store</t>
+  </si>
+  <si>
+    <t>Lisbon</t>
+  </si>
+  <si>
+    <t>http://lisbonduckstore.com/</t>
+  </si>
+  <si>
+    <t>Porto Duck Store</t>
+  </si>
+  <si>
+    <t>Porto</t>
+  </si>
+  <si>
+    <t>Rua do Choupelo 132, 4400-088 Vila Nova de Gaia, Portugal</t>
+  </si>
+  <si>
+    <t>https://portoduckstore.pt/</t>
+  </si>
+  <si>
+    <t>Segovia Duck Store</t>
+  </si>
+  <si>
+    <t>C. Juan Bravo, 42, 40001 Segovia, Spain</t>
+  </si>
+  <si>
+    <t>Segovia</t>
+  </si>
+  <si>
+    <t>https://www.duckstore.es/es/</t>
+  </si>
+  <si>
+    <t>Pl. Mayor, 10, Centro, Centro, 28012 Madrid, Spain</t>
+  </si>
+  <si>
+    <t>https://www.duckstore.es/</t>
+  </si>
+  <si>
+    <t>Royal Ducks</t>
+  </si>
+  <si>
+    <t>C. del Comercio, 17, 45001 Toledo, Spain</t>
+  </si>
+  <si>
+    <t>Toledo</t>
+  </si>
+  <si>
+    <t>PATURROS - Patitos de Goma - Regalos Originales</t>
+  </si>
+  <si>
+    <t>C. de Don Jaime I, 48-52, Casco Antiguo, 50001 Zaragoza, Spain</t>
+  </si>
+  <si>
+    <t>Zaragoza</t>
+  </si>
+  <si>
+    <t>https://www.paturros.es/?utm_source=google&amp;utm_medium=organic&amp;utm_campaign=gbp_profile&amp;utm_content=website_link</t>
+  </si>
+  <si>
+    <t>San Sebastian Duck Store</t>
+  </si>
+  <si>
+    <t>San Sebastian</t>
+  </si>
+  <si>
+    <t>C. Mayor, 21, 20003 Donostia / San Sebastián, Gipuzkoa, Spain</t>
+  </si>
+  <si>
+    <t>http://duckland.store/</t>
+  </si>
+  <si>
+    <t>Duckland</t>
+  </si>
+  <si>
+    <t>C/ del Trench, 18, Ciutat Vella, 46001 València, Valencia, Spain</t>
+  </si>
+  <si>
+    <t>Valencia</t>
+  </si>
+  <si>
+    <t>Av. de Martínez Alejos, 3, 03501 Benidorm, Alicante, Spain</t>
+  </si>
+  <si>
+    <t>Alicante</t>
+  </si>
+  <si>
+    <t>Av. de Jaume III, 8, Centre, 07012 Palma, Illes Balears, Spain</t>
+  </si>
+  <si>
+    <t>Illes Balears</t>
+  </si>
+  <si>
+    <t>Carrer de la Palla, 11, Ciutat Vella, 08002 Barcelona, Spain</t>
+  </si>
+  <si>
+    <t>https://www.duckstore.es/en/</t>
+  </si>
+  <si>
+    <t>6 Rue Yvonne le Tac, 75018 Paris, France</t>
+  </si>
+  <si>
+    <t>https://parisduckstore.fr/</t>
+  </si>
+  <si>
+    <t>Duck Shop Nice</t>
+  </si>
+  <si>
+    <t>Nice</t>
+  </si>
+  <si>
+    <t>3 Rue Cassini, 06300 Nice, France</t>
+  </si>
+  <si>
+    <t>http://www.duck-shop.fr/</t>
+  </si>
+  <si>
+    <t>SU24, 25 Darwin Centre, Shrewsbury SY1 1BW, United Kingdom</t>
+  </si>
+  <si>
+    <t>Shrewsbury</t>
+  </si>
+  <si>
+    <t>http://www.shop4ducks.co.uk/</t>
+  </si>
+  <si>
+    <t>Shrewsbury Duck Store</t>
+  </si>
+  <si>
+    <t>JustDucks</t>
+  </si>
+  <si>
+    <t>Dutch Barn, 16 Orwell Rd, Barrington, Cambridge CB22 7SE, United Kingdom</t>
+  </si>
+  <si>
+    <t>https://justducks.co.uk/</t>
+  </si>
+  <si>
+    <t>The Duck House</t>
+  </si>
+  <si>
+    <t>Brighton</t>
+  </si>
+  <si>
+    <t>4 Union St, Brighton and Hove, Brighton BN1 1HA, United Kingdom</t>
+  </si>
+  <si>
+    <t>http://www.theduckhousebrighton.online/</t>
+  </si>
+  <si>
+    <t>12B Paddock Ln, Chalk Farm Rd, London NW1 8AH, United Kingdom</t>
+  </si>
+  <si>
+    <t>https://duck-world.com/</t>
+  </si>
+  <si>
+    <t>60 Charing Cross Rd, London WC2H 7JD, United Kingdom</t>
+  </si>
+  <si>
+    <t>Victoria station, Victoria Station, Main Hall, next to Leon, Victoria St, London SW1V 1JU, United Kingdom</t>
+  </si>
+  <si>
+    <t>UK</t>
+  </si>
+  <si>
+    <t>The Rubber Duck Store and More</t>
+  </si>
+  <si>
+    <t>Kerkstraat 8, 2042 JE Zandvoort, Netherlands</t>
+  </si>
+  <si>
+    <t>Zandvoort</t>
+  </si>
+  <si>
+    <t>https://www.visitzandvoort.com/shops/zandvoort/tea-chocolate-more</t>
+  </si>
+  <si>
+    <t>Oude Leliestraat 16, 1015 BJ Amsterdam, Netherlands</t>
+  </si>
+  <si>
+    <t>https://www.amsterdamduckstore.com/%20%20%20%20%20https://www.originalduckstore.com/</t>
+  </si>
+  <si>
+    <t>The Rubber Duck Store</t>
+  </si>
+  <si>
+    <t>Rokin 82, 1012 KW Amsterdam, Netherlands</t>
+  </si>
+  <si>
+    <t>Oude Doelenstraat 2, 1012 ED Amsterdam, Netherlands</t>
+  </si>
+  <si>
+    <t>The Rubber Duck Store Amsterdam</t>
+  </si>
+  <si>
+    <t>Geldersekade 17, 1011 EH Amsterdam, Netherlands</t>
+  </si>
+  <si>
+    <t>The Rubber Duck Store Maastricht</t>
+  </si>
+  <si>
+    <t>Nieuwstraat 22, 6211 CS Maastricht, Netherlands</t>
+  </si>
+  <si>
+    <t>Maastricht</t>
+  </si>
+  <si>
+    <t>http://www.budduck.com/</t>
+  </si>
+  <si>
+    <t>DUCKSHOP</t>
+  </si>
+  <si>
+    <t>Paßkamp 16, 46414 Rhede, Germany</t>
+  </si>
+  <si>
+    <t>Rhede</t>
+  </si>
+  <si>
+    <t>https://www.duckshop.de/</t>
+  </si>
+  <si>
+    <t>DUCKS &amp; SOUVENIRS MÜNCHEN Sabine Bretting</t>
+  </si>
+  <si>
+    <t>Orlandostraße 4, 80331 München, Germany</t>
+  </si>
+  <si>
+    <t>Rubber Ducky Comics</t>
+  </si>
+  <si>
+    <t>Zimmerstraße 99, 10117 Berlin, Germany</t>
+  </si>
+  <si>
+    <t>Berlin</t>
+  </si>
+  <si>
+    <t>Duck Haven</t>
+  </si>
+  <si>
+    <t>Denmark</t>
+  </si>
+  <si>
+    <t>https://www.duckhaven.dk/</t>
+  </si>
+  <si>
+    <t>Vimmelskaftet 47, 1161 København, Denmark</t>
+  </si>
+  <si>
+    <t>København</t>
+  </si>
+  <si>
+    <t>Tallinn Duck Store</t>
+  </si>
+  <si>
+    <t>Tallinn</t>
+  </si>
+  <si>
+    <t>Estonia</t>
+  </si>
+  <si>
+    <t>Pikk tn 12, 10123 Tallinn, Estonia</t>
+  </si>
+  <si>
+    <t>https://tallinnduckstore.com/</t>
+  </si>
+  <si>
+    <t>Duck Land</t>
+  </si>
+  <si>
+    <t>Powstańców Śląskich 8/8, 72-600 Świnoujście, Poland</t>
+  </si>
+  <si>
+    <t>Świnoujście</t>
+  </si>
+  <si>
+    <t>Poland</t>
+  </si>
+  <si>
+    <t>Krakow Duck Store</t>
+  </si>
+  <si>
+    <t>Krakow</t>
+  </si>
+  <si>
+    <t>https://www.krakowduckstore.pl/</t>
+  </si>
+  <si>
+    <t>Szpitalna 32, 31-024 Kraków, Poland</t>
+  </si>
+  <si>
+    <t>Zakopane Duck Store</t>
+  </si>
+  <si>
+    <t>Zakopane</t>
+  </si>
+  <si>
+    <t>Józefa Piłsudskiego 2c, 34-500 Zakopane, Poland</t>
+  </si>
+  <si>
+    <t>http://zakopaneduckstore.pl/</t>
+  </si>
+  <si>
+    <t>Ducksy</t>
+  </si>
+  <si>
+    <t>Budapest</t>
+  </si>
+  <si>
+    <t>Hungary</t>
+  </si>
+  <si>
+    <t>Budapest, Ferenciek tere 10, 1052 Hungary</t>
+  </si>
+  <si>
+    <t>http://www.gumi-kacsa.hu/</t>
+  </si>
+  <si>
+    <t>Bucharest Duck Store</t>
+  </si>
+  <si>
+    <t>Bucharest</t>
+  </si>
+  <si>
+    <t>Romania</t>
+  </si>
+  <si>
+    <t>Strada Frumoasă 56, București 010988, Romania</t>
+  </si>
+  <si>
+    <t>http://bucharestduckstore.ro/</t>
+  </si>
+  <si>
+    <t>Ducklin</t>
+  </si>
+  <si>
+    <t>Athens</t>
+  </si>
+  <si>
+    <t>Greece</t>
+  </si>
+  <si>
+    <t>Miaouli 18, Athina 105 54, Greece</t>
+  </si>
+  <si>
+    <t>http://www.ducklin.gr/</t>
+  </si>
+  <si>
+    <t>Duck Boutique Dubrovnik</t>
+  </si>
+  <si>
+    <t>Dubrovnik</t>
+  </si>
+  <si>
+    <t>Croatia</t>
+  </si>
+  <si>
+    <t>Ul. od Puča 9, 20000, Dubrovnik, Croatia</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/duckboutique.croatia/</t>
+  </si>
+  <si>
+    <t>Duck Shop Split</t>
+  </si>
+  <si>
+    <t>Split</t>
+  </si>
+  <si>
+    <t>Bosanska ul. 6, 21000, Split, Croatia</t>
+  </si>
+  <si>
+    <t>https://splitcurated.com/listings/duck-boutique/</t>
+  </si>
+  <si>
+    <t>Duck Shop Zadar</t>
+  </si>
+  <si>
+    <t>Zadar</t>
+  </si>
+  <si>
+    <t>Ul. Mihovila Klaića 4, 23000, Zadar, Croatia</t>
+  </si>
+  <si>
+    <t>Duck Boutique Split</t>
+  </si>
+  <si>
+    <t>Marulićeva ul. 3, 21000, Split, Croatia</t>
+  </si>
+  <si>
+    <t>Stradun 22, 20000, Dubrovnik, Croatia</t>
+  </si>
+  <si>
+    <t>Ducks Ducks Zagreb</t>
+  </si>
+  <si>
+    <t>Zagreb</t>
+  </si>
+  <si>
+    <t>Ul. Ivana Tkalčića 32, 10000, Zagreb, Croatia</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/ducksduckszagreb?igsh=MXFxdmF5eGFxbXd2dQ==</t>
+  </si>
+  <si>
+    <t>The Rubber Duck Store Ljubljana</t>
+  </si>
+  <si>
+    <t>Ljubljana</t>
+  </si>
+  <si>
+    <t>Slovenia</t>
+  </si>
+  <si>
+    <t>Kongresni trg 5, 1000 Ljubljana, Slovenia</t>
+  </si>
+  <si>
+    <t>Milan Duck Store</t>
+  </si>
+  <si>
+    <t>Milan</t>
+  </si>
+  <si>
+    <t>Via Torino, 77, 20123 Milano MI, Italy</t>
+  </si>
+  <si>
+    <t>https://milanduckstore.com/</t>
+  </si>
+  <si>
+    <t>5414/A, Sotoportego de la Bissa, 30124 Venezia VE, Italy</t>
+  </si>
+  <si>
+    <t>https://www.veniceduckstore.it/</t>
+  </si>
+  <si>
+    <t>S. Marco, 707, 30124 Venezia VE, Italy</t>
+  </si>
+  <si>
+    <t>30121 Venice, Metropolitan City of Venice, Italy</t>
+  </si>
+  <si>
+    <t>Draem Duck</t>
+  </si>
+  <si>
+    <t>Florence</t>
+  </si>
+  <si>
+    <t>Via dei Calzaiuoli, 42, 50122 Firenze FI, Italy</t>
+  </si>
+  <si>
+    <t>https://www.facebook.com/florenceduckstore/</t>
+  </si>
+  <si>
+    <t>San Marino Duck Store</t>
+  </si>
+  <si>
+    <t>San Marino</t>
+  </si>
+  <si>
+    <t>Via Basilicius, 21, 47890 Città di San Marino, San Marino</t>
+  </si>
+  <si>
+    <t>http://www.sanmarinoduckstore.net/</t>
+  </si>
+  <si>
+    <t>Dream Duck Roma</t>
+  </si>
+  <si>
+    <t>00187 Rome, Metropolitan City of Rome Capital, Italy</t>
+  </si>
+  <si>
+    <t>https://www.instagram.com/dream_duck_official?igsh=MWwwamMxdjNrbTFnNQ==</t>
+  </si>
+  <si>
+    <t>V. dei Coronari, 108, 00186 Roma RM, Italy</t>
+  </si>
+  <si>
+    <t>https://www.romeduckstore.it/</t>
+  </si>
+  <si>
+    <t>Old, Old Akko 13/174, Acre, Israel</t>
+  </si>
+  <si>
+    <t>Duck You Akko</t>
+  </si>
+  <si>
+    <t>Acre</t>
+  </si>
+  <si>
+    <t>Duck You TLV</t>
+  </si>
+  <si>
+    <t>https://duckyou.shop/</t>
+  </si>
+  <si>
+    <t>King George St 12, Tel Aviv-Yafo, Israel</t>
+  </si>
+  <si>
+    <t>תחנה רכבת, Yitshak Ben Zvi St 12, Be'er Sheva, 8427712, Israel</t>
+  </si>
+  <si>
+    <t>Duck You  Be'er Sheva</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Be'er Sheva</t>
+  </si>
+  <si>
+    <t>https://www.duckyoubs.co.il/</t>
+  </si>
+  <si>
+    <t>Yellow Duck World</t>
+  </si>
+  <si>
+    <t>Arkan Plaza, First Al Sheikh Zayed, Second Al Sheikh Zayed, Giza Governorate 3242304, Egypt</t>
+  </si>
+  <si>
+    <t>https://yellowduckworld.com/</t>
+  </si>
+  <si>
+    <t>Egypt</t>
+  </si>
+  <si>
+    <t>Giza</t>
+  </si>
+  <si>
+    <t>Five Little Ducks</t>
+  </si>
+  <si>
+    <t>Dubai</t>
+  </si>
+  <si>
+    <t>UAE</t>
+  </si>
+  <si>
+    <t>185 Jumeira St - Jumeirah - Jumeira First - Dubai - United Arab Emirates</t>
+  </si>
+  <si>
+    <t>https://fivelittleducksme.com/</t>
   </si>
 </sst>
 </file>
@@ -2462,7 +3198,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="51">
+  <cellXfs count="52">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2611,6 +3347,9 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -3440,8 +4179,8 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}" name="Locations" displayName="Locations" ref="A1:I16" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:I16" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}" name="Locations" displayName="Locations" ref="A1:I87" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:I87" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{63C32DA5-9104-488A-B085-36DB395683F0}" name="Shop Name"/>
     <tableColumn id="2" xr3:uid="{9DB5CA49-9344-4EA7-9D0B-03CF697CEB1E}" name="City"/>
@@ -3454,6 +4193,16 @@
     <tableColumn id="9" xr3:uid="{05CD9E28-5179-4E3C-9FE0-67152446D074}" name="Address"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E618F2B7-E85B-4339-9336-15CEB340032D}" name="Chains" displayName="Chains" ref="A1:A7" totalsRowShown="0">
+  <autoFilter ref="A1:A7" xr:uid="{E618F2B7-E85B-4339-9336-15CEB340032D}"/>
+  <tableColumns count="1">
+    <tableColumn id="1" xr3:uid="{5AFB1E65-00FF-4DE8-A836-37B2BBE3CF06}" name="Store Name"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -14004,7 +14753,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="185" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="185" spans="1:18" ht="53.4" thickBot="1">
       <c r="A185" s="13" t="s">
         <v>204</v>
       </c>
@@ -15543,7 +16292,7 @@
       <c r="K213" s="40"/>
       <c r="L213" s="43"/>
       <c r="M213" s="41" t="s">
-        <v>706</v>
+        <v>699</v>
       </c>
       <c r="N213" s="40">
         <v>1</v>
@@ -15572,7 +16321,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E690491F-A75A-44CD-AF5E-964C98F48B1D}">
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I87"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
@@ -15582,7 +16331,7 @@
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
     <col min="7" max="7" width="15.21875" customWidth="1"/>
-    <col min="9" max="9" width="36.33203125" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="75.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" thickBot="1">
@@ -15616,42 +16365,42 @@
     </row>
     <row r="2" spans="1:9">
       <c r="A2" t="s">
-        <v>358</v>
+        <v>660</v>
       </c>
       <c r="B2" t="s">
+        <v>662</v>
+      </c>
+      <c r="C2" t="s">
+        <v>248</v>
+      </c>
+      <c r="D2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" t="s">
+        <v>24</v>
+      </c>
+      <c r="F2">
+        <v>29.463383242077299</v>
+      </c>
+      <c r="G2">
+        <v>-98.335771519372102</v>
+      </c>
+      <c r="H2" t="s">
+        <v>663</v>
+      </c>
+      <c r="I2" t="s">
         <v>661</v>
-      </c>
-      <c r="C2" t="s">
-        <v>425</v>
-      </c>
-      <c r="D2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" t="s">
-        <v>24</v>
-      </c>
-      <c r="F2">
-        <v>33.800500368778202</v>
-      </c>
-      <c r="G2">
-        <v>-117.910289903156</v>
-      </c>
-      <c r="H2" t="s">
-        <v>662</v>
-      </c>
-      <c r="I2" t="s">
-        <v>660</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" t="s">
-        <v>358</v>
+        <v>664</v>
       </c>
       <c r="B3" t="s">
-        <v>663</v>
+        <v>641</v>
       </c>
       <c r="C3" t="s">
-        <v>664</v>
+        <v>642</v>
       </c>
       <c r="D3" t="s">
         <v>24</v>
@@ -15660,10 +16409,10 @@
         <v>24</v>
       </c>
       <c r="F3">
-        <v>44.035644759071097</v>
+        <v>41.094637674232096</v>
       </c>
       <c r="G3">
-        <v>-112.211925491803</v>
+        <v>-83.661265806926806</v>
       </c>
       <c r="H3" t="s">
         <v>666</v>
@@ -15677,25 +16426,25 @@
         <v>667</v>
       </c>
       <c r="B4" t="s">
+        <v>406</v>
+      </c>
+      <c r="C4" t="s">
+        <v>407</v>
+      </c>
+      <c r="D4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E4" t="s">
+        <v>24</v>
+      </c>
+      <c r="F4">
+        <v>36.756490311024898</v>
+      </c>
+      <c r="G4">
+        <v>-83.490698324576201</v>
+      </c>
+      <c r="H4" t="s">
         <v>669</v>
-      </c>
-      <c r="C4" t="s">
-        <v>248</v>
-      </c>
-      <c r="D4" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" t="s">
-        <v>24</v>
-      </c>
-      <c r="F4">
-        <v>29.463383242077299</v>
-      </c>
-      <c r="G4">
-        <v>-98.335771519372102</v>
-      </c>
-      <c r="H4" t="s">
-        <v>670</v>
       </c>
       <c r="I4" t="s">
         <v>668</v>
@@ -15703,13 +16452,13 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>671</v>
+        <v>670</v>
       </c>
       <c r="B5" t="s">
-        <v>641</v>
+        <v>672</v>
       </c>
       <c r="C5" t="s">
-        <v>642</v>
+        <v>43</v>
       </c>
       <c r="D5" t="s">
         <v>24</v>
@@ -15718,16 +16467,16 @@
         <v>24</v>
       </c>
       <c r="F5">
-        <v>41.094637674232096</v>
+        <v>30.237048753086999</v>
       </c>
       <c r="G5">
-        <v>-83.661265806926806</v>
+        <v>-81.302681827847593</v>
       </c>
       <c r="H5" t="s">
         <v>673</v>
       </c>
       <c r="I5" t="s">
-        <v>672</v>
+        <v>671</v>
       </c>
     </row>
     <row r="6" spans="1:9">
@@ -15735,10 +16484,10 @@
         <v>674</v>
       </c>
       <c r="B6" t="s">
-        <v>406</v>
+        <v>636</v>
       </c>
       <c r="C6" t="s">
-        <v>407</v>
+        <v>266</v>
       </c>
       <c r="D6" t="s">
         <v>24</v>
@@ -15747,10 +16496,10 @@
         <v>24</v>
       </c>
       <c r="F6">
-        <v>36.756490311024898</v>
+        <v>39.382735466011901</v>
       </c>
       <c r="G6">
-        <v>-83.490698324576201</v>
+        <v>-74.075276886054397</v>
       </c>
       <c r="H6" t="s">
         <v>676</v>
@@ -15761,42 +16510,42 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
+        <v>334</v>
+      </c>
+      <c r="B7" t="s">
+        <v>335</v>
+      </c>
+      <c r="C7" t="s">
+        <v>102</v>
+      </c>
+      <c r="D7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" t="s">
+        <v>24</v>
+      </c>
+      <c r="F7">
+        <v>41.762380767075598</v>
+      </c>
+      <c r="G7">
+        <v>-69.964720011453906</v>
+      </c>
+      <c r="H7" t="s">
+        <v>678</v>
+      </c>
+      <c r="I7" t="s">
         <v>677</v>
-      </c>
-      <c r="B7" t="s">
-        <v>679</v>
-      </c>
-      <c r="C7" t="s">
-        <v>43</v>
-      </c>
-      <c r="D7" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" t="s">
-        <v>24</v>
-      </c>
-      <c r="F7">
-        <v>30.237048753086999</v>
-      </c>
-      <c r="G7">
-        <v>-81.302681827847593</v>
-      </c>
-      <c r="H7" t="s">
-        <v>680</v>
-      </c>
-      <c r="I7" t="s">
-        <v>678</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>681</v>
+        <v>227</v>
       </c>
       <c r="B8" t="s">
-        <v>636</v>
+        <v>228</v>
       </c>
       <c r="C8" t="s">
-        <v>266</v>
+        <v>221</v>
       </c>
       <c r="D8" t="s">
         <v>24</v>
@@ -15805,97 +16554,97 @@
         <v>24</v>
       </c>
       <c r="F8">
-        <v>39.382735466011901</v>
+        <v>41.424445068117102</v>
       </c>
       <c r="G8">
-        <v>-74.075276886054397</v>
+        <v>-72.242355034482003</v>
       </c>
       <c r="H8" t="s">
-        <v>683</v>
+        <v>680</v>
       </c>
       <c r="I8" t="s">
-        <v>682</v>
+        <v>679</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>334</v>
+        <v>681</v>
       </c>
       <c r="B9" t="s">
-        <v>335</v>
+        <v>175</v>
       </c>
       <c r="C9" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="D9" t="s">
-        <v>24</v>
+        <v>172</v>
       </c>
       <c r="E9" t="s">
-        <v>24</v>
+        <v>177</v>
       </c>
       <c r="F9">
-        <v>41.762380767075598</v>
+        <v>46.059205916812402</v>
       </c>
       <c r="G9">
-        <v>-69.964720011453906</v>
+        <v>-73.751381735450806</v>
       </c>
       <c r="H9" t="s">
-        <v>685</v>
+        <v>683</v>
       </c>
       <c r="I9" t="s">
-        <v>684</v>
+        <v>682</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>227</v>
+        <v>684</v>
       </c>
       <c r="B10" t="s">
-        <v>228</v>
+        <v>416</v>
       </c>
       <c r="C10" t="s">
-        <v>221</v>
+        <v>88</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>701</v>
       </c>
       <c r="E10" t="s">
-        <v>24</v>
+        <v>700</v>
       </c>
       <c r="F10">
-        <v>41.424445068117102</v>
+        <v>-31.301920080120301</v>
       </c>
       <c r="G10">
-        <v>-72.242355034482003</v>
+        <v>150.92525148123801</v>
       </c>
       <c r="H10" t="s">
-        <v>687</v>
+        <v>686</v>
       </c>
       <c r="I10" t="s">
-        <v>686</v>
+        <v>685</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
+        <v>687</v>
+      </c>
+      <c r="B11" t="s">
         <v>688</v>
-      </c>
-      <c r="B11" t="s">
-        <v>175</v>
       </c>
       <c r="C11" t="s">
         <v>88</v>
       </c>
       <c r="D11" t="s">
-        <v>172</v>
+        <v>592</v>
       </c>
       <c r="E11" t="s">
-        <v>177</v>
+        <v>593</v>
       </c>
       <c r="F11">
-        <v>46.059205916812402</v>
+        <v>38.266755018307997</v>
       </c>
       <c r="G11">
-        <v>-73.751381735450806</v>
+        <v>140.87937309661501</v>
       </c>
       <c r="H11" t="s">
         <v>690</v>
@@ -15909,36 +16658,36 @@
         <v>691</v>
       </c>
       <c r="B12" t="s">
-        <v>416</v>
+        <v>692</v>
       </c>
       <c r="C12" t="s">
         <v>88</v>
       </c>
       <c r="D12" t="s">
-        <v>708</v>
+        <v>592</v>
       </c>
       <c r="E12" t="s">
-        <v>707</v>
+        <v>593</v>
       </c>
       <c r="F12">
-        <v>-31.301920080120301</v>
+        <v>35.339815509095899</v>
       </c>
       <c r="G12">
-        <v>150.92525148123801</v>
+        <v>139.596898521875</v>
       </c>
       <c r="H12" t="s">
+        <v>694</v>
+      </c>
+      <c r="I12" t="s">
         <v>693</v>
-      </c>
-      <c r="I12" t="s">
-        <v>692</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>694</v>
+        <v>691</v>
       </c>
       <c r="B13" t="s">
-        <v>695</v>
+        <v>591</v>
       </c>
       <c r="C13" t="s">
         <v>88</v>
@@ -15950,24 +16699,24 @@
         <v>593</v>
       </c>
       <c r="F13">
-        <v>38.266755018307997</v>
+        <v>35.012908784767497</v>
       </c>
       <c r="G13">
-        <v>140.87937309661501</v>
+        <v>135.81056759424601</v>
       </c>
       <c r="H13" t="s">
-        <v>697</v>
+        <v>694</v>
       </c>
       <c r="I13" t="s">
-        <v>696</v>
+        <v>695</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>698</v>
+        <v>696</v>
       </c>
       <c r="B14" t="s">
-        <v>699</v>
+        <v>591</v>
       </c>
       <c r="C14" t="s">
         <v>88</v>
@@ -15979,74 +16728,1929 @@
         <v>593</v>
       </c>
       <c r="F14">
-        <v>35.339815509095899</v>
+        <v>34.905430873998398</v>
       </c>
       <c r="G14">
-        <v>139.596898521875</v>
+        <v>135.820807959506</v>
       </c>
       <c r="H14" t="s">
-        <v>701</v>
+        <v>698</v>
       </c>
       <c r="I14" t="s">
-        <v>700</v>
+        <v>697</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>698</v>
+        <v>704</v>
       </c>
       <c r="B15" t="s">
-        <v>591</v>
+        <v>706</v>
       </c>
       <c r="C15" t="s">
         <v>88</v>
       </c>
       <c r="D15" t="s">
-        <v>592</v>
+        <v>707</v>
       </c>
       <c r="E15" t="s">
-        <v>593</v>
+        <v>722</v>
       </c>
       <c r="F15">
-        <v>35.012908784767497</v>
+        <v>-40.786415636732201</v>
       </c>
       <c r="G15">
-        <v>135.81056759424601</v>
+        <v>-71.580962813109593</v>
       </c>
       <c r="H15" t="s">
-        <v>701</v>
+        <v>708</v>
       </c>
       <c r="I15" t="s">
-        <v>702</v>
+        <v>705</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>703</v>
+        <v>704</v>
       </c>
       <c r="B16" t="s">
-        <v>591</v>
+        <v>710</v>
       </c>
       <c r="C16" t="s">
         <v>88</v>
       </c>
       <c r="D16" t="s">
-        <v>592</v>
+        <v>707</v>
       </c>
       <c r="E16" t="s">
-        <v>593</v>
+        <v>722</v>
       </c>
       <c r="F16">
-        <v>34.905430873998398</v>
+        <v>-38.725857404054402</v>
       </c>
       <c r="G16">
-        <v>135.820807959506</v>
+        <v>-71.756744063156802</v>
       </c>
       <c r="H16" t="s">
-        <v>705</v>
+        <v>708</v>
       </c>
       <c r="I16" t="s">
+        <v>709</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" t="s">
         <v>704</v>
+      </c>
+      <c r="B17" t="s">
+        <v>712</v>
+      </c>
+      <c r="C17" t="s">
+        <v>88</v>
+      </c>
+      <c r="D17" t="s">
+        <v>707</v>
+      </c>
+      <c r="E17" t="s">
+        <v>722</v>
+      </c>
+      <c r="F17">
+        <v>-32.013300460726299</v>
+      </c>
+      <c r="G17">
+        <v>-67.307104194756405</v>
+      </c>
+      <c r="H17" t="s">
+        <v>708</v>
+      </c>
+      <c r="I17" t="s">
+        <v>711</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" t="s">
+        <v>714</v>
+      </c>
+      <c r="B18" t="s">
+        <v>716</v>
+      </c>
+      <c r="C18" t="s">
+        <v>633</v>
+      </c>
+      <c r="D18" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" t="s">
+        <v>24</v>
+      </c>
+      <c r="F18">
+        <v>52.433531012009098</v>
+      </c>
+      <c r="G18">
+        <v>-123.22178013617</v>
+      </c>
+      <c r="H18" t="s">
+        <v>715</v>
+      </c>
+      <c r="I18" t="s">
+        <v>713</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" t="s">
+        <v>717</v>
+      </c>
+      <c r="B19" t="s">
+        <v>720</v>
+      </c>
+      <c r="C19" t="s">
+        <v>721</v>
+      </c>
+      <c r="D19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19" t="s">
+        <v>24</v>
+      </c>
+      <c r="F19">
+        <v>41.013755634792503</v>
+      </c>
+      <c r="G19">
+        <v>-104.67981369292001</v>
+      </c>
+      <c r="H19" t="s">
+        <v>718</v>
+      </c>
+      <c r="I19" t="s">
+        <v>719</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" t="s">
+        <v>725</v>
+      </c>
+      <c r="B20" t="s">
+        <v>724</v>
+      </c>
+      <c r="C20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D20" t="s">
+        <v>24</v>
+      </c>
+      <c r="E20" t="s">
+        <v>24</v>
+      </c>
+      <c r="F20">
+        <v>31.630322255398099</v>
+      </c>
+      <c r="G20">
+        <v>-85.5425843592501</v>
+      </c>
+      <c r="H20" t="s">
+        <v>726</v>
+      </c>
+      <c r="I20" t="s">
+        <v>723</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
+        <v>728</v>
+      </c>
+      <c r="B21" t="s">
+        <v>729</v>
+      </c>
+      <c r="C21" t="s">
+        <v>23</v>
+      </c>
+      <c r="D21" t="s">
+        <v>24</v>
+      </c>
+      <c r="E21" t="s">
+        <v>24</v>
+      </c>
+      <c r="F21">
+        <v>40.747527963989199</v>
+      </c>
+      <c r="G21">
+        <v>-75.217366002108193</v>
+      </c>
+      <c r="H21" t="s">
+        <v>730</v>
+      </c>
+      <c r="I21" t="s">
+        <v>727</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>732</v>
+      </c>
+      <c r="B22" t="s">
+        <v>733</v>
+      </c>
+      <c r="C22" t="s">
+        <v>734</v>
+      </c>
+      <c r="D22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22" t="s">
+        <v>24</v>
+      </c>
+      <c r="F22">
+        <v>39.864495027195801</v>
+      </c>
+      <c r="G22">
+        <v>-88.989360409703806</v>
+      </c>
+      <c r="H22" t="s">
+        <v>735</v>
+      </c>
+      <c r="I22" t="s">
+        <v>731</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>736</v>
+      </c>
+      <c r="B23" t="s">
+        <v>738</v>
+      </c>
+      <c r="C23" t="s">
+        <v>248</v>
+      </c>
+      <c r="D23" t="s">
+        <v>24</v>
+      </c>
+      <c r="E23" t="s">
+        <v>24</v>
+      </c>
+      <c r="F23">
+        <v>32.981457350907903</v>
+      </c>
+      <c r="G23">
+        <v>-97.248080019994205</v>
+      </c>
+      <c r="H23" t="s">
+        <v>739</v>
+      </c>
+      <c r="I23" t="s">
+        <v>737</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>741</v>
+      </c>
+      <c r="B24" t="s">
+        <v>743</v>
+      </c>
+      <c r="C24" t="s">
+        <v>248</v>
+      </c>
+      <c r="D24" t="s">
+        <v>24</v>
+      </c>
+      <c r="E24" t="s">
+        <v>24</v>
+      </c>
+      <c r="F24">
+        <v>30.419982573452302</v>
+      </c>
+      <c r="G24">
+        <v>-95.488375549339693</v>
+      </c>
+      <c r="H24" t="s">
+        <v>744</v>
+      </c>
+      <c r="I24" t="s">
+        <v>742</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>746</v>
+      </c>
+      <c r="B25" t="s">
+        <v>747</v>
+      </c>
+      <c r="C25" t="s">
+        <v>376</v>
+      </c>
+      <c r="D25" t="s">
+        <v>24</v>
+      </c>
+      <c r="E25" t="s">
+        <v>24</v>
+      </c>
+      <c r="F25">
+        <v>45.652471967540798</v>
+      </c>
+      <c r="G25">
+        <v>-94.631015820070601</v>
+      </c>
+      <c r="H25" t="s">
+        <v>748</v>
+      </c>
+      <c r="I25" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
+        <v>750</v>
+      </c>
+      <c r="B26" t="s">
+        <v>751</v>
+      </c>
+      <c r="C26" t="s">
+        <v>425</v>
+      </c>
+      <c r="D26" t="s">
+        <v>24</v>
+      </c>
+      <c r="E26" t="s">
+        <v>24</v>
+      </c>
+      <c r="F26">
+        <v>38.6044143871462</v>
+      </c>
+      <c r="G26">
+        <v>-121.970852569643</v>
+      </c>
+      <c r="H26" t="s">
+        <v>752</v>
+      </c>
+      <c r="I26" t="s">
+        <v>749</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>753</v>
+      </c>
+      <c r="B27" t="s">
+        <v>754</v>
+      </c>
+      <c r="C27" t="s">
+        <v>376</v>
+      </c>
+      <c r="D27" t="s">
+        <v>24</v>
+      </c>
+      <c r="E27" t="s">
+        <v>24</v>
+      </c>
+      <c r="F27">
+        <v>44.912860602563299</v>
+      </c>
+      <c r="G27">
+        <v>-93.159409454946299</v>
+      </c>
+      <c r="H27" t="s">
+        <v>756</v>
+      </c>
+      <c r="I27" t="s">
+        <v>755</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" t="s">
+        <v>757</v>
+      </c>
+      <c r="B28" t="s">
+        <v>758</v>
+      </c>
+      <c r="C28" t="s">
+        <v>199</v>
+      </c>
+      <c r="D28" t="s">
+        <v>24</v>
+      </c>
+      <c r="E28" t="s">
+        <v>24</v>
+      </c>
+      <c r="F28">
+        <v>43.087409565957998</v>
+      </c>
+      <c r="G28">
+        <v>-70.765013104871798</v>
+      </c>
+      <c r="H28" t="s">
+        <v>759</v>
+      </c>
+      <c r="I28" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" t="s">
+        <v>761</v>
+      </c>
+      <c r="B29" t="s">
+        <v>118</v>
+      </c>
+      <c r="C29" t="s">
+        <v>102</v>
+      </c>
+      <c r="D29" t="s">
+        <v>24</v>
+      </c>
+      <c r="E29" t="s">
+        <v>24</v>
+      </c>
+      <c r="F29">
+        <v>42.513539232803197</v>
+      </c>
+      <c r="G29">
+        <v>-70.858736422377703</v>
+      </c>
+      <c r="H29" t="s">
+        <v>763</v>
+      </c>
+      <c r="I29" t="s">
+        <v>762</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="28.8">
+      <c r="A30" s="51" t="s">
+        <v>764</v>
+      </c>
+      <c r="B30" t="s">
+        <v>766</v>
+      </c>
+      <c r="C30" t="s">
+        <v>43</v>
+      </c>
+      <c r="D30" t="s">
+        <v>24</v>
+      </c>
+      <c r="E30" t="s">
+        <v>24</v>
+      </c>
+      <c r="F30">
+        <v>28.3912216062288</v>
+      </c>
+      <c r="G30">
+        <v>-82.575119545015397</v>
+      </c>
+      <c r="H30" t="s">
+        <v>767</v>
+      </c>
+      <c r="I30" t="s">
+        <v>765</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" t="s">
+        <v>768</v>
+      </c>
+      <c r="B31" t="s">
+        <v>769</v>
+      </c>
+      <c r="C31" t="s">
+        <v>88</v>
+      </c>
+      <c r="D31" t="s">
+        <v>770</v>
+      </c>
+      <c r="F31">
+        <v>32.698968976301302</v>
+      </c>
+      <c r="G31">
+        <v>-16.861378151127099</v>
+      </c>
+      <c r="H31" t="s">
+        <v>772</v>
+      </c>
+      <c r="I31" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" t="s">
+        <v>774</v>
+      </c>
+      <c r="B32" t="s">
+        <v>775</v>
+      </c>
+      <c r="C32" t="s">
+        <v>88</v>
+      </c>
+      <c r="D32" t="s">
+        <v>770</v>
+      </c>
+      <c r="F32">
+        <v>39.036139407971199</v>
+      </c>
+      <c r="G32">
+        <v>-9.2255342942693908</v>
+      </c>
+      <c r="H32" t="s">
+        <v>776</v>
+      </c>
+      <c r="I32" t="s">
+        <v>773</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" t="s">
+        <v>777</v>
+      </c>
+      <c r="B33" t="s">
+        <v>778</v>
+      </c>
+      <c r="C33" t="s">
+        <v>88</v>
+      </c>
+      <c r="D33" t="s">
+        <v>770</v>
+      </c>
+      <c r="F33">
+        <v>41.351962361722599</v>
+      </c>
+      <c r="G33">
+        <v>-7.3798311687738796</v>
+      </c>
+      <c r="H33" t="s">
+        <v>780</v>
+      </c>
+      <c r="I33" t="s">
+        <v>779</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" t="s">
+        <v>781</v>
+      </c>
+      <c r="B34" t="s">
+        <v>783</v>
+      </c>
+      <c r="C34" t="s">
+        <v>88</v>
+      </c>
+      <c r="D34" t="s">
+        <v>68</v>
+      </c>
+      <c r="F34">
+        <v>41.294194149250401</v>
+      </c>
+      <c r="G34">
+        <v>-4.1820650812680196</v>
+      </c>
+      <c r="H34" t="s">
+        <v>784</v>
+      </c>
+      <c r="I34" t="s">
+        <v>782</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" t="s">
+        <v>491</v>
+      </c>
+      <c r="B35" t="s">
+        <v>492</v>
+      </c>
+      <c r="C35" t="s">
+        <v>88</v>
+      </c>
+      <c r="D35" t="s">
+        <v>68</v>
+      </c>
+      <c r="F35">
+        <v>40.721797077446197</v>
+      </c>
+      <c r="G35">
+        <v>-3.4235315612319299</v>
+      </c>
+      <c r="H35" t="s">
+        <v>786</v>
+      </c>
+      <c r="I35" t="s">
+        <v>785</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" t="s">
+        <v>787</v>
+      </c>
+      <c r="B36" t="s">
+        <v>789</v>
+      </c>
+      <c r="C36" t="s">
+        <v>88</v>
+      </c>
+      <c r="D36" t="s">
+        <v>68</v>
+      </c>
+      <c r="F36">
+        <v>40.052125191398602</v>
+      </c>
+      <c r="G36">
+        <v>-3.3718133666840102</v>
+      </c>
+      <c r="I36" t="s">
+        <v>788</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" t="s">
+        <v>790</v>
+      </c>
+      <c r="B37" t="s">
+        <v>792</v>
+      </c>
+      <c r="C37" t="s">
+        <v>88</v>
+      </c>
+      <c r="D37" t="s">
+        <v>68</v>
+      </c>
+      <c r="F37">
+        <v>41.810234875948503</v>
+      </c>
+      <c r="G37">
+        <v>-6.1848916288551999E-2</v>
+      </c>
+      <c r="H37" t="s">
+        <v>793</v>
+      </c>
+      <c r="I37" t="s">
+        <v>791</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" t="s">
+        <v>794</v>
+      </c>
+      <c r="B38" t="s">
+        <v>795</v>
+      </c>
+      <c r="C38" t="s">
+        <v>88</v>
+      </c>
+      <c r="D38" t="s">
+        <v>68</v>
+      </c>
+      <c r="F38">
+        <v>43.458849891467899</v>
+      </c>
+      <c r="G38">
+        <v>-2.0443797072919598</v>
+      </c>
+      <c r="H38" t="s">
+        <v>786</v>
+      </c>
+      <c r="I38" t="s">
+        <v>796</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" t="s">
+        <v>798</v>
+      </c>
+      <c r="B39" t="s">
+        <v>800</v>
+      </c>
+      <c r="C39" t="s">
+        <v>88</v>
+      </c>
+      <c r="D39" t="s">
+        <v>68</v>
+      </c>
+      <c r="F39">
+        <v>39.612507832099098</v>
+      </c>
+      <c r="G39">
+        <v>-0.17264615686895099</v>
+      </c>
+      <c r="H39" t="s">
+        <v>797</v>
+      </c>
+      <c r="I39" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" t="s">
+        <v>458</v>
+      </c>
+      <c r="B40" t="s">
+        <v>802</v>
+      </c>
+      <c r="C40" t="s">
+        <v>88</v>
+      </c>
+      <c r="D40" t="s">
+        <v>68</v>
+      </c>
+      <c r="F40">
+        <v>38.649531481995503</v>
+      </c>
+      <c r="G40">
+        <v>-0.161659828717404</v>
+      </c>
+      <c r="I40" t="s">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" t="s">
+        <v>798</v>
+      </c>
+      <c r="B41" t="s">
+        <v>804</v>
+      </c>
+      <c r="C41" t="s">
+        <v>88</v>
+      </c>
+      <c r="D41" t="s">
+        <v>68</v>
+      </c>
+      <c r="F41">
+        <v>41.523431604823699</v>
+      </c>
+      <c r="G41">
+        <v>2.1674417340687002</v>
+      </c>
+      <c r="H41" t="s">
+        <v>797</v>
+      </c>
+      <c r="I41" t="s">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" t="s">
+        <v>66</v>
+      </c>
+      <c r="B42" t="s">
+        <v>67</v>
+      </c>
+      <c r="C42" t="s">
+        <v>88</v>
+      </c>
+      <c r="D42" t="s">
+        <v>68</v>
+      </c>
+      <c r="F42">
+        <v>41.523431613458399</v>
+      </c>
+      <c r="G42">
+        <v>2.5409768902508598</v>
+      </c>
+      <c r="H42" t="s">
+        <v>806</v>
+      </c>
+      <c r="I42" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" t="s">
+        <v>156</v>
+      </c>
+      <c r="B43" t="s">
+        <v>157</v>
+      </c>
+      <c r="C43" t="s">
+        <v>88</v>
+      </c>
+      <c r="D43" t="s">
+        <v>158</v>
+      </c>
+      <c r="F43">
+        <v>48.973399886181802</v>
+      </c>
+      <c r="G43">
+        <v>2.30468277539183</v>
+      </c>
+      <c r="H43" t="s">
+        <v>808</v>
+      </c>
+      <c r="I43" t="s">
+        <v>807</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" t="s">
+        <v>809</v>
+      </c>
+      <c r="B44" t="s">
+        <v>810</v>
+      </c>
+      <c r="C44" t="s">
+        <v>88</v>
+      </c>
+      <c r="D44" t="s">
+        <v>158</v>
+      </c>
+      <c r="F44">
+        <v>43.771369444886702</v>
+      </c>
+      <c r="G44">
+        <v>7.2646827520436696</v>
+      </c>
+      <c r="H44" t="s">
+        <v>812</v>
+      </c>
+      <c r="I44" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" t="s">
+        <v>816</v>
+      </c>
+      <c r="B45" t="s">
+        <v>814</v>
+      </c>
+      <c r="C45" t="s">
+        <v>88</v>
+      </c>
+      <c r="D45" t="s">
+        <v>828</v>
+      </c>
+      <c r="F45">
+        <v>52.711779660655402</v>
+      </c>
+      <c r="G45">
+        <v>-2.7544210462605099</v>
+      </c>
+      <c r="H45" t="s">
+        <v>815</v>
+      </c>
+      <c r="I45" t="s">
+        <v>813</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" t="s">
+        <v>817</v>
+      </c>
+      <c r="B46" t="s">
+        <v>101</v>
+      </c>
+      <c r="C46" t="s">
+        <v>88</v>
+      </c>
+      <c r="D46" t="s">
+        <v>828</v>
+      </c>
+      <c r="F46">
+        <v>52.131304915221598</v>
+      </c>
+      <c r="G46">
+        <v>2.3116018557096701E-2</v>
+      </c>
+      <c r="H46" t="s">
+        <v>819</v>
+      </c>
+      <c r="I46" t="s">
+        <v>818</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" t="s">
+        <v>820</v>
+      </c>
+      <c r="B47" t="s">
+        <v>821</v>
+      </c>
+      <c r="C47" t="s">
+        <v>88</v>
+      </c>
+      <c r="D47" t="s">
+        <v>828</v>
+      </c>
+      <c r="F47">
+        <v>50.824919945324702</v>
+      </c>
+      <c r="G47">
+        <v>-0.14456399091611599</v>
+      </c>
+      <c r="H47" t="s">
+        <v>823</v>
+      </c>
+      <c r="I47" t="s">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" t="s">
+        <v>458</v>
+      </c>
+      <c r="B48" t="s">
+        <v>94</v>
+      </c>
+      <c r="C48" t="s">
+        <v>88</v>
+      </c>
+      <c r="D48" t="s">
+        <v>828</v>
+      </c>
+      <c r="F48">
+        <v>51.544533375625001</v>
+      </c>
+      <c r="G48">
+        <v>-0.14992233319881601</v>
+      </c>
+      <c r="H48" t="s">
+        <v>825</v>
+      </c>
+      <c r="I48" t="s">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" t="s">
+        <v>458</v>
+      </c>
+      <c r="B49" t="s">
+        <v>94</v>
+      </c>
+      <c r="C49" t="s">
+        <v>88</v>
+      </c>
+      <c r="D49" t="s">
+        <v>828</v>
+      </c>
+      <c r="F49">
+        <v>51.513388843156498</v>
+      </c>
+      <c r="G49">
+        <v>-0.13013037045387099</v>
+      </c>
+      <c r="H49" t="s">
+        <v>825</v>
+      </c>
+      <c r="I49" t="s">
+        <v>826</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" t="s">
+        <v>458</v>
+      </c>
+      <c r="B50" t="s">
+        <v>94</v>
+      </c>
+      <c r="C50" t="s">
+        <v>88</v>
+      </c>
+      <c r="D50" t="s">
+        <v>828</v>
+      </c>
+      <c r="F50">
+        <v>51.495996583316597</v>
+      </c>
+      <c r="G50">
+        <v>-0.14526540078824099</v>
+      </c>
+      <c r="H50" t="s">
+        <v>825</v>
+      </c>
+      <c r="I50" t="s">
+        <v>827</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" t="s">
+        <v>829</v>
+      </c>
+      <c r="B51" t="s">
+        <v>831</v>
+      </c>
+      <c r="C51" t="s">
+        <v>88</v>
+      </c>
+      <c r="D51" t="s">
+        <v>649</v>
+      </c>
+      <c r="F51">
+        <v>52.378198062539497</v>
+      </c>
+      <c r="G51">
+        <v>4.5170594911307704</v>
+      </c>
+      <c r="H51" t="s">
+        <v>832</v>
+      </c>
+      <c r="I51" t="s">
+        <v>830</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" t="s">
+        <v>526</v>
+      </c>
+      <c r="B52" t="s">
+        <v>524</v>
+      </c>
+      <c r="C52" t="s">
+        <v>88</v>
+      </c>
+      <c r="D52" t="s">
+        <v>649</v>
+      </c>
+      <c r="F52">
+        <v>52.375070075125102</v>
+      </c>
+      <c r="G52">
+        <v>4.8883119454223003</v>
+      </c>
+      <c r="H52" t="s">
+        <v>834</v>
+      </c>
+      <c r="I52" t="s">
+        <v>833</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" t="s">
+        <v>835</v>
+      </c>
+      <c r="B53" t="s">
+        <v>524</v>
+      </c>
+      <c r="C53" t="s">
+        <v>88</v>
+      </c>
+      <c r="D53" t="s">
+        <v>649</v>
+      </c>
+      <c r="F53">
+        <v>52.370196721388403</v>
+      </c>
+      <c r="G53">
+        <v>4.8920884957162798</v>
+      </c>
+      <c r="I53" t="s">
+        <v>836</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" t="s">
+        <v>838</v>
+      </c>
+      <c r="B54" t="s">
+        <v>524</v>
+      </c>
+      <c r="C54" t="s">
+        <v>88</v>
+      </c>
+      <c r="D54" t="s">
+        <v>649</v>
+      </c>
+      <c r="F54">
+        <v>52.371873634966299</v>
+      </c>
+      <c r="G54">
+        <v>4.89612253807576</v>
+      </c>
+      <c r="I54" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" t="s">
+        <v>835</v>
+      </c>
+      <c r="B55" t="s">
+        <v>524</v>
+      </c>
+      <c r="C55" t="s">
+        <v>88</v>
+      </c>
+      <c r="D55" t="s">
+        <v>649</v>
+      </c>
+      <c r="F55">
+        <v>52.375594059638097</v>
+      </c>
+      <c r="G55">
+        <v>4.9023881783362304</v>
+      </c>
+      <c r="I55" t="s">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" t="s">
+        <v>840</v>
+      </c>
+      <c r="B56" t="s">
+        <v>842</v>
+      </c>
+      <c r="C56" t="s">
+        <v>88</v>
+      </c>
+      <c r="D56" t="s">
+        <v>649</v>
+      </c>
+      <c r="F56">
+        <v>50.853174792217501</v>
+      </c>
+      <c r="G56">
+        <v>5.69135731114772</v>
+      </c>
+      <c r="H56" t="s">
+        <v>843</v>
+      </c>
+      <c r="I56" t="s">
+        <v>841</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" t="s">
+        <v>844</v>
+      </c>
+      <c r="B57" t="s">
+        <v>846</v>
+      </c>
+      <c r="C57" t="s">
+        <v>88</v>
+      </c>
+      <c r="D57" t="s">
+        <v>571</v>
+      </c>
+      <c r="F57">
+        <v>51.878187806059799</v>
+      </c>
+      <c r="G57">
+        <v>6.6960724324398102</v>
+      </c>
+      <c r="H57" t="s">
+        <v>847</v>
+      </c>
+      <c r="I57" t="s">
+        <v>845</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" t="s">
+        <v>848</v>
+      </c>
+      <c r="B58" t="s">
+        <v>570</v>
+      </c>
+      <c r="C58" t="s">
+        <v>88</v>
+      </c>
+      <c r="D58" t="s">
+        <v>571</v>
+      </c>
+      <c r="F58">
+        <v>48.137221333880603</v>
+      </c>
+      <c r="G58">
+        <v>11.4690853303973</v>
+      </c>
+      <c r="I58" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" t="s">
+        <v>850</v>
+      </c>
+      <c r="B59" t="s">
+        <v>852</v>
+      </c>
+      <c r="C59" t="s">
+        <v>88</v>
+      </c>
+      <c r="D59" t="s">
+        <v>571</v>
+      </c>
+      <c r="F59">
+        <v>52.545502086676898</v>
+      </c>
+      <c r="G59">
+        <v>13.355599788077599</v>
+      </c>
+      <c r="I59" t="s">
+        <v>851</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" t="s">
+        <v>853</v>
+      </c>
+      <c r="B60" t="s">
+        <v>857</v>
+      </c>
+      <c r="C60" t="s">
+        <v>88</v>
+      </c>
+      <c r="D60" t="s">
+        <v>854</v>
+      </c>
+      <c r="F60">
+        <v>55.6774230496355</v>
+      </c>
+      <c r="G60">
+        <v>12.568158381159201</v>
+      </c>
+      <c r="H60" t="s">
+        <v>855</v>
+      </c>
+      <c r="I60" t="s">
+        <v>856</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9">
+      <c r="A61" t="s">
+        <v>858</v>
+      </c>
+      <c r="B61" t="s">
+        <v>859</v>
+      </c>
+      <c r="C61" t="s">
+        <v>88</v>
+      </c>
+      <c r="D61" t="s">
+        <v>860</v>
+      </c>
+      <c r="F61">
+        <v>59.442348826981799</v>
+      </c>
+      <c r="G61">
+        <v>24.7429114165996</v>
+      </c>
+      <c r="H61" t="s">
+        <v>862</v>
+      </c>
+      <c r="I61" t="s">
+        <v>861</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9">
+      <c r="A62" t="s">
+        <v>863</v>
+      </c>
+      <c r="B62" t="s">
+        <v>865</v>
+      </c>
+      <c r="C62" t="s">
+        <v>88</v>
+      </c>
+      <c r="D62" t="s">
+        <v>866</v>
+      </c>
+      <c r="F62">
+        <v>53.918879037622801</v>
+      </c>
+      <c r="G62">
+        <v>14.2528957989717</v>
+      </c>
+      <c r="I62" t="s">
+        <v>864</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9">
+      <c r="A63" t="s">
+        <v>867</v>
+      </c>
+      <c r="B63" t="s">
+        <v>868</v>
+      </c>
+      <c r="C63" t="s">
+        <v>88</v>
+      </c>
+      <c r="D63" t="s">
+        <v>866</v>
+      </c>
+      <c r="F63">
+        <v>50.062293158228499</v>
+      </c>
+      <c r="G63">
+        <v>19.9349083318201</v>
+      </c>
+      <c r="H63" t="s">
+        <v>869</v>
+      </c>
+      <c r="I63" t="s">
+        <v>870</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9">
+      <c r="A64" t="s">
+        <v>871</v>
+      </c>
+      <c r="B64" t="s">
+        <v>872</v>
+      </c>
+      <c r="C64" t="s">
+        <v>88</v>
+      </c>
+      <c r="D64" t="s">
+        <v>866</v>
+      </c>
+      <c r="F64">
+        <v>49.299704517398801</v>
+      </c>
+      <c r="G64">
+        <v>19.955287727156101</v>
+      </c>
+      <c r="H64" t="s">
+        <v>874</v>
+      </c>
+      <c r="I64" t="s">
+        <v>873</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9">
+      <c r="A65" t="s">
+        <v>875</v>
+      </c>
+      <c r="B65" t="s">
+        <v>876</v>
+      </c>
+      <c r="C65" t="s">
+        <v>88</v>
+      </c>
+      <c r="D65" t="s">
+        <v>877</v>
+      </c>
+      <c r="F65">
+        <v>47.493781030775899</v>
+      </c>
+      <c r="G65">
+        <v>19.056194687097499</v>
+      </c>
+      <c r="H65" t="s">
+        <v>879</v>
+      </c>
+      <c r="I65" t="s">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9">
+      <c r="A66" t="s">
+        <v>880</v>
+      </c>
+      <c r="B66" t="s">
+        <v>881</v>
+      </c>
+      <c r="C66" t="s">
+        <v>88</v>
+      </c>
+      <c r="D66" t="s">
+        <v>882</v>
+      </c>
+      <c r="F66">
+        <v>44.450794263639096</v>
+      </c>
+      <c r="G66">
+        <v>26.086394058725201</v>
+      </c>
+      <c r="H66" t="s">
+        <v>884</v>
+      </c>
+      <c r="I66" t="s">
+        <v>883</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9">
+      <c r="A67" t="s">
+        <v>885</v>
+      </c>
+      <c r="B67" t="s">
+        <v>886</v>
+      </c>
+      <c r="C67" t="s">
+        <v>88</v>
+      </c>
+      <c r="D67" t="s">
+        <v>887</v>
+      </c>
+      <c r="F67">
+        <v>37.977628330785301</v>
+      </c>
+      <c r="G67">
+        <v>23.724571665283101</v>
+      </c>
+      <c r="H67" t="s">
+        <v>889</v>
+      </c>
+      <c r="I67" t="s">
+        <v>888</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9">
+      <c r="A68" t="s">
+        <v>890</v>
+      </c>
+      <c r="B68" t="s">
+        <v>891</v>
+      </c>
+      <c r="C68" t="s">
+        <v>88</v>
+      </c>
+      <c r="D68" t="s">
+        <v>892</v>
+      </c>
+      <c r="F68">
+        <v>42.640669732898502</v>
+      </c>
+      <c r="G68">
+        <v>18.1088954965102</v>
+      </c>
+      <c r="H68" t="s">
+        <v>894</v>
+      </c>
+      <c r="I68" t="s">
+        <v>893</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9">
+      <c r="A69" t="s">
+        <v>895</v>
+      </c>
+      <c r="B69" t="s">
+        <v>896</v>
+      </c>
+      <c r="C69" t="s">
+        <v>88</v>
+      </c>
+      <c r="D69" t="s">
+        <v>892</v>
+      </c>
+      <c r="F69">
+        <v>43.509153771859999</v>
+      </c>
+      <c r="G69">
+        <v>16.439297745722001</v>
+      </c>
+      <c r="H69" t="s">
+        <v>898</v>
+      </c>
+      <c r="I69" t="s">
+        <v>897</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9">
+      <c r="A70" t="s">
+        <v>899</v>
+      </c>
+      <c r="B70" t="s">
+        <v>900</v>
+      </c>
+      <c r="C70" t="s">
+        <v>88</v>
+      </c>
+      <c r="D70" t="s">
+        <v>892</v>
+      </c>
+      <c r="F70">
+        <v>44.113881823968498</v>
+      </c>
+      <c r="G70">
+        <v>15.226994459353801</v>
+      </c>
+      <c r="I70" t="s">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9">
+      <c r="A71" t="s">
+        <v>902</v>
+      </c>
+      <c r="B71" t="s">
+        <v>896</v>
+      </c>
+      <c r="C71" t="s">
+        <v>88</v>
+      </c>
+      <c r="D71" t="s">
+        <v>892</v>
+      </c>
+      <c r="F71">
+        <v>43.508491462566703</v>
+      </c>
+      <c r="G71">
+        <v>16.438738703728799</v>
+      </c>
+      <c r="H71" t="s">
+        <v>894</v>
+      </c>
+      <c r="I71" t="s">
+        <v>903</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9">
+      <c r="A72" t="s">
+        <v>890</v>
+      </c>
+      <c r="B72" t="s">
+        <v>891</v>
+      </c>
+      <c r="C72" t="s">
+        <v>88</v>
+      </c>
+      <c r="D72" t="s">
+        <v>892</v>
+      </c>
+      <c r="F72">
+        <v>42.641448880157299</v>
+      </c>
+      <c r="G72">
+        <v>18.108708858081901</v>
+      </c>
+      <c r="H72" t="s">
+        <v>894</v>
+      </c>
+      <c r="I72" t="s">
+        <v>904</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9">
+      <c r="A73" t="s">
+        <v>905</v>
+      </c>
+      <c r="B73" t="s">
+        <v>906</v>
+      </c>
+      <c r="C73" t="s">
+        <v>88</v>
+      </c>
+      <c r="D73" t="s">
+        <v>892</v>
+      </c>
+      <c r="F73">
+        <v>45.815999034471403</v>
+      </c>
+      <c r="G73">
+        <v>15.9757907599175</v>
+      </c>
+      <c r="H73" t="s">
+        <v>908</v>
+      </c>
+      <c r="I73" t="s">
+        <v>907</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9">
+      <c r="A74" t="s">
+        <v>909</v>
+      </c>
+      <c r="B74" t="s">
+        <v>910</v>
+      </c>
+      <c r="C74" t="s">
+        <v>88</v>
+      </c>
+      <c r="D74" t="s">
+        <v>911</v>
+      </c>
+      <c r="F74">
+        <v>46.052500560187703</v>
+      </c>
+      <c r="G74">
+        <v>14.5051018908164</v>
+      </c>
+      <c r="I74" t="s">
+        <v>912</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9">
+      <c r="A75" t="s">
+        <v>913</v>
+      </c>
+      <c r="B75" t="s">
+        <v>914</v>
+      </c>
+      <c r="C75" t="s">
+        <v>88</v>
+      </c>
+      <c r="D75" t="s">
+        <v>314</v>
+      </c>
+      <c r="F75">
+        <v>45.459955873306903</v>
+      </c>
+      <c r="G75">
+        <v>9.1817341590042698</v>
+      </c>
+      <c r="H75" t="s">
+        <v>916</v>
+      </c>
+      <c r="I75" t="s">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9">
+      <c r="A76" t="s">
+        <v>318</v>
+      </c>
+      <c r="B76" t="s">
+        <v>319</v>
+      </c>
+      <c r="C76" t="s">
+        <v>88</v>
+      </c>
+      <c r="D76" t="s">
+        <v>314</v>
+      </c>
+      <c r="F76">
+        <v>45.437711653191698</v>
+      </c>
+      <c r="G76">
+        <v>12.3372600700623</v>
+      </c>
+      <c r="H76" t="s">
+        <v>918</v>
+      </c>
+      <c r="I76" t="s">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9">
+      <c r="A77" t="s">
+        <v>318</v>
+      </c>
+      <c r="B77" t="s">
+        <v>319</v>
+      </c>
+      <c r="C77" t="s">
+        <v>88</v>
+      </c>
+      <c r="D77" t="s">
+        <v>314</v>
+      </c>
+      <c r="F77">
+        <v>45.4357857236336</v>
+      </c>
+      <c r="G77">
+        <v>12.338114341246699</v>
+      </c>
+      <c r="H77" t="s">
+        <v>918</v>
+      </c>
+      <c r="I77" t="s">
+        <v>919</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9">
+      <c r="A78" t="s">
+        <v>318</v>
+      </c>
+      <c r="B78" t="s">
+        <v>319</v>
+      </c>
+      <c r="C78" t="s">
+        <v>88</v>
+      </c>
+      <c r="D78" t="s">
+        <v>314</v>
+      </c>
+      <c r="F78">
+        <v>45.440782321598597</v>
+      </c>
+      <c r="G78">
+        <v>12.3352324126277</v>
+      </c>
+      <c r="H78" t="s">
+        <v>918</v>
+      </c>
+      <c r="I78" t="s">
+        <v>920</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9">
+      <c r="A79" t="s">
+        <v>921</v>
+      </c>
+      <c r="B79" t="s">
+        <v>922</v>
+      </c>
+      <c r="C79" t="s">
+        <v>88</v>
+      </c>
+      <c r="D79" t="s">
+        <v>314</v>
+      </c>
+      <c r="F79">
+        <v>43.770867429289197</v>
+      </c>
+      <c r="G79">
+        <v>11.2554047899725</v>
+      </c>
+      <c r="H79" t="s">
+        <v>924</v>
+      </c>
+      <c r="I79" t="s">
+        <v>923</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9">
+      <c r="A80" t="s">
+        <v>925</v>
+      </c>
+      <c r="B80" t="s">
+        <v>926</v>
+      </c>
+      <c r="C80" t="s">
+        <v>88</v>
+      </c>
+      <c r="D80" t="s">
+        <v>314</v>
+      </c>
+      <c r="F80">
+        <v>43.935609314633197</v>
+      </c>
+      <c r="G80">
+        <v>12.446803482111701</v>
+      </c>
+      <c r="H80" t="s">
+        <v>928</v>
+      </c>
+      <c r="I80" t="s">
+        <v>927</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9">
+      <c r="A81" t="s">
+        <v>929</v>
+      </c>
+      <c r="B81" t="s">
+        <v>325</v>
+      </c>
+      <c r="C81" t="s">
+        <v>88</v>
+      </c>
+      <c r="D81" t="s">
+        <v>314</v>
+      </c>
+      <c r="F81">
+        <v>41.904766191071197</v>
+      </c>
+      <c r="G81">
+        <v>12.478982679078699</v>
+      </c>
+      <c r="H81" t="s">
+        <v>931</v>
+      </c>
+      <c r="I81" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9">
+      <c r="A82" t="s">
+        <v>327</v>
+      </c>
+      <c r="B82" t="s">
+        <v>325</v>
+      </c>
+      <c r="C82" t="s">
+        <v>88</v>
+      </c>
+      <c r="D82" t="s">
+        <v>314</v>
+      </c>
+      <c r="F82">
+        <v>41.900532853153301</v>
+      </c>
+      <c r="G82">
+        <v>12.468392352353</v>
+      </c>
+      <c r="H82" t="s">
+        <v>933</v>
+      </c>
+      <c r="I82" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9">
+      <c r="A83" t="s">
+        <v>935</v>
+      </c>
+      <c r="B83" t="s">
+        <v>936</v>
+      </c>
+      <c r="C83" t="s">
+        <v>88</v>
+      </c>
+      <c r="D83" t="s">
+        <v>134</v>
+      </c>
+      <c r="F83">
+        <v>32.922455623738799</v>
+      </c>
+      <c r="G83">
+        <v>35.070240555908498</v>
+      </c>
+      <c r="I83" t="s">
+        <v>934</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" t="s">
+        <v>937</v>
+      </c>
+      <c r="B84" t="s">
+        <v>133</v>
+      </c>
+      <c r="C84" t="s">
+        <v>88</v>
+      </c>
+      <c r="D84" t="s">
+        <v>134</v>
+      </c>
+      <c r="F84">
+        <v>32.070936261991797</v>
+      </c>
+      <c r="G84">
+        <v>34.772256917509203</v>
+      </c>
+      <c r="H84" t="s">
+        <v>938</v>
+      </c>
+      <c r="I84" t="s">
+        <v>939</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9">
+      <c r="A85" t="s">
+        <v>941</v>
+      </c>
+      <c r="B85" t="s">
+        <v>942</v>
+      </c>
+      <c r="C85" t="s">
+        <v>88</v>
+      </c>
+      <c r="D85" t="s">
+        <v>134</v>
+      </c>
+      <c r="F85">
+        <v>31.241277726774001</v>
+      </c>
+      <c r="G85">
+        <v>34.796193268741902</v>
+      </c>
+      <c r="H85" t="s">
+        <v>943</v>
+      </c>
+      <c r="I85" t="s">
+        <v>940</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9">
+      <c r="A86" t="s">
+        <v>944</v>
+      </c>
+      <c r="B86" t="s">
+        <v>948</v>
+      </c>
+      <c r="C86" t="s">
+        <v>88</v>
+      </c>
+      <c r="D86" t="s">
+        <v>947</v>
+      </c>
+      <c r="F86">
+        <v>30.020802135695298</v>
+      </c>
+      <c r="G86">
+        <v>31.0030222660539</v>
+      </c>
+      <c r="H86" t="s">
+        <v>946</v>
+      </c>
+      <c r="I86" t="s">
+        <v>945</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9">
+      <c r="A87" t="s">
+        <v>949</v>
+      </c>
+      <c r="B87" t="s">
+        <v>950</v>
+      </c>
+      <c r="C87" t="s">
+        <v>88</v>
+      </c>
+      <c r="D87" t="s">
+        <v>951</v>
+      </c>
+      <c r="F87">
+        <v>25.215850937399502</v>
+      </c>
+      <c r="G87">
+        <v>55.250893152761897</v>
+      </c>
+      <c r="H87" t="s">
+        <v>953</v>
+      </c>
+      <c r="I87" t="s">
+        <v>952</v>
       </c>
     </row>
   </sheetData>
@@ -16056,4 +18660,55 @@
     <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54904E20-3C5D-490F-BCF5-E5014AEEFD29}">
+  <dimension ref="A1:A7"/>
+  <sheetFormatPr defaultRowHeight="14.4"/>
+  <cols>
+    <col min="1" max="1" width="12.33203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>702</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>703</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>479</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>740</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId1"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
added duck data, changed slicer settings, played with home page
</commit_message>
<xml_diff>
--- a/Power BI V2/Data/DuckDataBI.xlsx
+++ b/Power BI V2/Data/DuckDataBI.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\allan\Documents\DS_Projects\Analyducks\Power BI V2\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA8D2EF2-4EF3-43CD-B1CB-B5E89A60D41C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD6A4A38-F1A3-4C8E-B305-BB79F60B0E0F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{C5D2797D-B188-49E6-A37E-A541A2C853B5}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C5D2797D-B188-49E6-A37E-A541A2C853B5}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
-    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
-    <sheet name="Sheet3" sheetId="3" r:id="rId3"/>
+    <sheet name="Ducks" sheetId="1" r:id="rId1"/>
+    <sheet name="Stores" sheetId="2" r:id="rId2"/>
+    <sheet name="Chains" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2458" uniqueCount="954">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2517" uniqueCount="983">
   <si>
     <t>Duck</t>
   </si>
@@ -2143,9 +2143,6 @@
     <t>Mayya</t>
   </si>
   <si>
-    <t>AUS</t>
-  </si>
-  <si>
     <t>Australia</t>
   </si>
   <si>
@@ -2209,9 +2206,6 @@
     <t>CO</t>
   </si>
   <si>
-    <t>CHL</t>
-  </si>
-  <si>
     <t>45 Central Square, Santa Rosa Beach, FL 32459</t>
   </si>
   <si>
@@ -2903,6 +2897,99 @@
   </si>
   <si>
     <t>https://fivelittleducksme.com/</t>
+  </si>
+  <si>
+    <t>Mama Duck Store</t>
+  </si>
+  <si>
+    <t>http://www.mamaducksstore.nl/</t>
+  </si>
+  <si>
+    <t>Reguliersbreestraat 47, 1017 CM Amsterdam, Netherlands</t>
+  </si>
+  <si>
+    <t>Chamber of Ducks</t>
+  </si>
+  <si>
+    <t>38 Burgate, Canterbury CT1 2HW, United Kingdom</t>
+  </si>
+  <si>
+    <t>Canterbury</t>
+  </si>
+  <si>
+    <t>Killarney</t>
+  </si>
+  <si>
+    <t>78 High Street, Killarney, Co. Kerry, V93 AP11, Ireland</t>
+  </si>
+  <si>
+    <t>Killarney Duck Store</t>
+  </si>
+  <si>
+    <t>Ireland</t>
+  </si>
+  <si>
+    <t>https://killarneyduckstore.ie/</t>
+  </si>
+  <si>
+    <t>Turkey1</t>
+  </si>
+  <si>
+    <t>Turkey2</t>
+  </si>
+  <si>
+    <t>Turkey3</t>
+  </si>
+  <si>
+    <t>Snowflake green</t>
+  </si>
+  <si>
+    <t>2026 duck</t>
+  </si>
+  <si>
+    <t>Balloon Animal</t>
+  </si>
+  <si>
+    <t>Pirate</t>
+  </si>
+  <si>
+    <t>Marcus Theaters</t>
+  </si>
+  <si>
+    <t>Chesterfield</t>
+  </si>
+  <si>
+    <t>Five Below</t>
+  </si>
+  <si>
+    <t>Michaels</t>
+  </si>
+  <si>
+    <t>Captain Quack Sparrow</t>
+  </si>
+  <si>
+    <t>2026!</t>
+  </si>
+  <si>
+    <t>SnowDrake</t>
+  </si>
+  <si>
+    <t>Laika</t>
+  </si>
+  <si>
+    <t>Eminem</t>
+  </si>
+  <si>
+    <t>Slim Shady</t>
+  </si>
+  <si>
+    <t>Tuxie</t>
+  </si>
+  <si>
+    <t>Ally</t>
+  </si>
+  <si>
+    <t>Voorhees</t>
   </si>
 </sst>
 </file>
@@ -3198,7 +3285,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -3350,6 +3437,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="16" fontId="2" fillId="3" borderId="12" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4149,8 +4239,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{02C6EB19-C16E-4C45-82D8-19820ABC0444}" name="Table1" displayName="Table1" ref="A1:R213" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19" totalsRowBorderDxfId="18">
-  <autoFilter ref="A1:R213" xr:uid="{02C6EB19-C16E-4C45-82D8-19820ABC0444}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{02C6EB19-C16E-4C45-82D8-19820ABC0444}" name="Table1" displayName="Table1" ref="A1:R220" totalsRowShown="0" headerRowDxfId="22" dataDxfId="20" headerRowBorderDxfId="21" tableBorderDxfId="19" totalsRowBorderDxfId="18">
+  <autoFilter ref="A1:R220" xr:uid="{02C6EB19-C16E-4C45-82D8-19820ABC0444}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:R210">
     <sortCondition descending="1" ref="O1:O210"/>
   </sortState>
@@ -4179,14 +4269,13 @@
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}" name="Locations" displayName="Locations" ref="A1:I87" totalsRowShown="0" headerRowDxfId="0">
-  <autoFilter ref="A1:I87" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}" name="Locations" displayName="Locations" ref="A1:H90" totalsRowShown="0" headerRowDxfId="0">
+  <autoFilter ref="A1:H90" xr:uid="{56F15032-C742-40F5-BC53-07A970E7D3F4}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{63C32DA5-9104-488A-B085-36DB395683F0}" name="Shop Name"/>
     <tableColumn id="2" xr3:uid="{9DB5CA49-9344-4EA7-9D0B-03CF697CEB1E}" name="City"/>
     <tableColumn id="3" xr3:uid="{286EA7E5-4452-4F0D-8C78-04BAE27F1F3A}" name="State"/>
     <tableColumn id="4" xr3:uid="{88EF38A1-9615-4274-861E-67CCBFC84894}" name="Country"/>
-    <tableColumn id="5" xr3:uid="{B4761F6B-E138-4A60-B88D-220C59CAF85D}" name="ISO_Code"/>
     <tableColumn id="6" xr3:uid="{B7DA27AC-1D08-4160-81AC-A2AF96AF118C}" name="Latitude"/>
     <tableColumn id="7" xr3:uid="{CB3D8E42-6E43-4860-B22A-448900D42EA4}" name="Longitude"/>
     <tableColumn id="8" xr3:uid="{55805FF1-912D-4EA1-BC97-A9AC858273FB}" name="Link"/>
@@ -4197,8 +4286,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E618F2B7-E85B-4339-9336-15CEB340032D}" name="Chains" displayName="Chains" ref="A1:A7" totalsRowShown="0">
-  <autoFilter ref="A1:A7" xr:uid="{E618F2B7-E85B-4339-9336-15CEB340032D}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{E618F2B7-E85B-4339-9336-15CEB340032D}" name="Chains" displayName="Chains" ref="A1:A8" totalsRowShown="0">
+  <autoFilter ref="A1:A8" xr:uid="{E618F2B7-E85B-4339-9336-15CEB340032D}"/>
   <tableColumns count="1">
     <tableColumn id="1" xr3:uid="{5AFB1E65-00FF-4DE8-A836-37B2BBE3CF06}" name="Store Name"/>
   </tableColumns>
@@ -4523,9 +4612,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9F4260E6-9B1A-4EF4-9E2A-700EF8F18DD3}">
-  <dimension ref="A1:R213"/>
+  <dimension ref="A1:R220"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
+    <col min="1" max="1" width="16.77734375" customWidth="1"/>
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="18.33203125" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
@@ -4534,7 +4624,7 @@
     <col min="7" max="7" width="18.6640625" customWidth="1"/>
     <col min="8" max="8" width="14.109375" customWidth="1"/>
     <col min="9" max="9" width="14.6640625" customWidth="1"/>
-    <col min="10" max="10" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="11" max="11" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="30.33203125" customWidth="1"/>
     <col min="13" max="13" width="8.33203125" bestFit="1" customWidth="1"/>
@@ -4601,7 +4691,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="27" thickBot="1">
+    <row r="2" spans="1:18" ht="15" thickBot="1">
       <c r="A2" s="12" t="s">
         <v>614</v>
       </c>
@@ -4728,7 +4818,7 @@
         <v>175</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>176</v>
+        <v>88</v>
       </c>
       <c r="G4" s="1" t="s">
         <v>172</v>
@@ -4823,7 +4913,7 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="6" spans="1:18" ht="27" thickBot="1">
+    <row r="6" spans="1:18" ht="15" thickBot="1">
       <c r="A6" s="12" t="s">
         <v>310</v>
       </c>
@@ -4879,7 +4969,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="7" spans="1:18" ht="27" thickBot="1">
+    <row r="7" spans="1:18" ht="15" thickBot="1">
       <c r="A7" s="20" t="s">
         <v>299</v>
       </c>
@@ -4991,7 +5081,7 @@
         <v>9.6999999999999993</v>
       </c>
     </row>
-    <row r="9" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="9" spans="1:18" ht="15" thickBot="1">
       <c r="A9" s="13" t="s">
         <v>388</v>
       </c>
@@ -5551,7 +5641,7 @@
         <v>12.5</v>
       </c>
     </row>
-    <row r="19" spans="1:18" ht="27" thickBot="1">
+    <row r="19" spans="1:18" ht="15" thickBot="1">
       <c r="A19" s="13" t="s">
         <v>287</v>
       </c>
@@ -5827,7 +5917,7 @@
         <v>8.3000000000000007</v>
       </c>
     </row>
-    <row r="24" spans="1:18" ht="27" thickBot="1">
+    <row r="24" spans="1:18" ht="15" thickBot="1">
       <c r="A24" s="19" t="s">
         <v>535</v>
       </c>
@@ -5939,7 +6029,7 @@
         <v>8.1999999999999993</v>
       </c>
     </row>
-    <row r="26" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="26" spans="1:18" ht="15" thickBot="1">
       <c r="A26" s="12" t="s">
         <v>409</v>
       </c>
@@ -5995,7 +6085,7 @@
         <v>6.7</v>
       </c>
     </row>
-    <row r="27" spans="1:18" ht="27" thickBot="1">
+    <row r="27" spans="1:18" ht="15" thickBot="1">
       <c r="A27" s="13" t="s">
         <v>422</v>
       </c>
@@ -6051,7 +6141,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="28" spans="1:18" ht="27" thickBot="1">
+    <row r="28" spans="1:18" ht="15" thickBot="1">
       <c r="A28" s="19" t="s">
         <v>551</v>
       </c>
@@ -6157,7 +6247,7 @@
         <v>10.5</v>
       </c>
     </row>
-    <row r="30" spans="1:18" ht="27" thickBot="1">
+    <row r="30" spans="1:18" ht="15" thickBot="1">
       <c r="A30" s="19" t="s">
         <v>330</v>
       </c>
@@ -6213,7 +6303,7 @@
         <v>10.3</v>
       </c>
     </row>
-    <row r="31" spans="1:18" ht="27" thickBot="1">
+    <row r="31" spans="1:18" ht="15" thickBot="1">
       <c r="A31" s="20" t="s">
         <v>345</v>
       </c>
@@ -6437,7 +6527,7 @@
         <v>12.4</v>
       </c>
     </row>
-    <row r="35" spans="1:18" ht="27" thickBot="1">
+    <row r="35" spans="1:18" ht="15" thickBot="1">
       <c r="A35" s="20" t="s">
         <v>555</v>
       </c>
@@ -6711,7 +6801,7 @@
         <v>8.3000000000000007</v>
       </c>
     </row>
-    <row r="40" spans="1:18" ht="27" thickBot="1">
+    <row r="40" spans="1:18" ht="15" thickBot="1">
       <c r="A40" s="19" t="s">
         <v>502</v>
       </c>
@@ -6989,7 +7079,7 @@
         <v>8.8000000000000007</v>
       </c>
     </row>
-    <row r="45" spans="1:18" ht="27" thickBot="1">
+    <row r="45" spans="1:18" ht="15" thickBot="1">
       <c r="A45" s="13" t="s">
         <v>316</v>
       </c>
@@ -7045,7 +7135,7 @@
         <v>8.9</v>
       </c>
     </row>
-    <row r="46" spans="1:18" ht="27" thickBot="1">
+    <row r="46" spans="1:18" ht="15" thickBot="1">
       <c r="A46" s="12" t="s">
         <v>320</v>
       </c>
@@ -7491,7 +7581,7 @@
         <v>8.8000000000000007</v>
       </c>
     </row>
-    <row r="54" spans="1:18" ht="27" thickBot="1">
+    <row r="54" spans="1:18" ht="15" thickBot="1">
       <c r="A54" s="12" t="s">
         <v>534</v>
       </c>
@@ -7883,7 +7973,7 @@
         <v>8.8000000000000007</v>
       </c>
     </row>
-    <row r="61" spans="1:18" ht="27" thickBot="1">
+    <row r="61" spans="1:18" ht="15" thickBot="1">
       <c r="A61" s="13" t="s">
         <v>594</v>
       </c>
@@ -8159,7 +8249,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="66" spans="1:18" ht="27" thickBot="1">
+    <row r="66" spans="1:18" ht="15" thickBot="1">
       <c r="A66" s="19" t="s">
         <v>343</v>
       </c>
@@ -8215,7 +8305,7 @@
         <v>9.1999999999999993</v>
       </c>
     </row>
-    <row r="67" spans="1:18" ht="27" thickBot="1">
+    <row r="67" spans="1:18" ht="15" thickBot="1">
       <c r="A67" s="13" t="s">
         <v>385</v>
       </c>
@@ -8327,7 +8417,7 @@
         <v>7.9</v>
       </c>
     </row>
-    <row r="69" spans="1:18" ht="27" thickBot="1">
+    <row r="69" spans="1:18" ht="15" thickBot="1">
       <c r="A69" s="20" t="s">
         <v>386</v>
       </c>
@@ -8663,7 +8753,7 @@
         <v>8.1999999999999993</v>
       </c>
     </row>
-    <row r="75" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="75" spans="1:18" ht="27" thickBot="1">
       <c r="A75" s="20" t="s">
         <v>382</v>
       </c>
@@ -8779,8 +8869,8 @@
       <c r="A77" s="20" t="s">
         <v>644</v>
       </c>
-      <c r="B77" s="24">
-        <v>113</v>
+      <c r="B77" s="24" t="s">
+        <v>644</v>
       </c>
       <c r="C77" s="22" t="s">
         <v>29</v>
@@ -8829,7 +8919,7 @@
         <v>8.6999999999999993</v>
       </c>
     </row>
-    <row r="78" spans="1:18" ht="27" thickBot="1">
+    <row r="78" spans="1:18" ht="15" thickBot="1">
       <c r="A78" s="19" t="s">
         <v>212</v>
       </c>
@@ -8997,7 +9087,7 @@
         <v>8.4</v>
       </c>
     </row>
-    <row r="81" spans="1:18" ht="27" thickBot="1">
+    <row r="81" spans="1:18" ht="15" thickBot="1">
       <c r="A81" s="20" t="s">
         <v>340</v>
       </c>
@@ -9165,7 +9255,7 @@
         <v>7.6</v>
       </c>
     </row>
-    <row r="84" spans="1:18" ht="27" thickBot="1">
+    <row r="84" spans="1:18" ht="15" thickBot="1">
       <c r="A84" s="12" t="s">
         <v>498</v>
       </c>
@@ -9331,7 +9421,7 @@
         <v>7.8</v>
       </c>
     </row>
-    <row r="87" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="87" spans="1:18" ht="27" thickBot="1">
       <c r="A87" s="13" t="s">
         <v>482</v>
       </c>
@@ -9443,7 +9533,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="89" spans="1:18" ht="27" thickBot="1">
+    <row r="89" spans="1:18" ht="15" thickBot="1">
       <c r="A89" s="13" t="s">
         <v>489</v>
       </c>
@@ -9499,12 +9589,12 @@
         <v>8</v>
       </c>
     </row>
-    <row r="90" spans="1:18" ht="27" thickBot="1">
+    <row r="90" spans="1:18" ht="15" thickBot="1">
       <c r="A90" s="12" t="s">
         <v>604</v>
       </c>
-      <c r="B90" s="3">
-        <v>105</v>
+      <c r="B90" s="3" t="s">
+        <v>981</v>
       </c>
       <c r="C90" s="1" t="s">
         <v>29</v>
@@ -9545,7 +9635,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="91" spans="1:18" ht="27" thickBot="1">
+    <row r="91" spans="1:18" ht="15" thickBot="1">
       <c r="A91" s="13" t="s">
         <v>496</v>
       </c>
@@ -9711,7 +9801,7 @@
         <v>4.5</v>
       </c>
     </row>
-    <row r="94" spans="1:18" ht="27" thickBot="1">
+    <row r="94" spans="1:18" ht="15" thickBot="1">
       <c r="A94" s="12" t="s">
         <v>622</v>
       </c>
@@ -9765,7 +9855,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="95" spans="1:18" ht="27" thickBot="1">
+    <row r="95" spans="1:18" ht="15" thickBot="1">
       <c r="A95" s="13" t="s">
         <v>629</v>
       </c>
@@ -9819,7 +9909,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="96" spans="1:18" ht="27" thickBot="1">
+    <row r="96" spans="1:18" ht="15" thickBot="1">
       <c r="A96" s="12" t="s">
         <v>548</v>
       </c>
@@ -9931,7 +10021,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="98" spans="1:18" ht="27" thickBot="1">
+    <row r="98" spans="1:18" ht="15" thickBot="1">
       <c r="A98" s="19" t="s">
         <v>624</v>
       </c>
@@ -9985,7 +10075,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="99" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="99" spans="1:18" ht="27" thickBot="1">
       <c r="A99" s="13" t="s">
         <v>549</v>
       </c>
@@ -10041,7 +10131,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="100" spans="1:18" ht="27" thickBot="1">
+    <row r="100" spans="1:18" ht="15" thickBot="1">
       <c r="A100" s="12" t="s">
         <v>626</v>
       </c>
@@ -10095,7 +10185,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="101" spans="1:18" ht="53.4" thickBot="1">
+    <row r="101" spans="1:18" ht="27" thickBot="1">
       <c r="A101" s="20" t="s">
         <v>566</v>
       </c>
@@ -10263,7 +10353,7 @@
         <v>5.9</v>
       </c>
     </row>
-    <row r="104" spans="1:18" ht="27" thickBot="1">
+    <row r="104" spans="1:18" ht="15" thickBot="1">
       <c r="A104" s="12" t="s">
         <v>544</v>
       </c>
@@ -10319,7 +10409,7 @@
         <v>6.6</v>
       </c>
     </row>
-    <row r="105" spans="1:18" ht="27" thickBot="1">
+    <row r="105" spans="1:18" ht="15" thickBot="1">
       <c r="A105" s="13" t="s">
         <v>578</v>
       </c>
@@ -10375,7 +10465,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="106" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="106" spans="1:18" ht="15" thickBot="1">
       <c r="A106" s="19" t="s">
         <v>562</v>
       </c>
@@ -10431,7 +10521,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="107" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="107" spans="1:18" ht="27" thickBot="1">
       <c r="A107" s="20" t="s">
         <v>579</v>
       </c>
@@ -10487,7 +10577,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="108" spans="1:18" ht="27" thickBot="1">
+    <row r="108" spans="1:18" ht="15" thickBot="1">
       <c r="A108" s="19" t="s">
         <v>429</v>
       </c>
@@ -10655,7 +10745,7 @@
         <v>7.5</v>
       </c>
     </row>
-    <row r="111" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="111" spans="1:18" ht="27" thickBot="1">
       <c r="A111" s="13" t="s">
         <v>586</v>
       </c>
@@ -10711,7 +10801,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="112" spans="1:18" ht="27" thickBot="1">
+    <row r="112" spans="1:18" ht="15" thickBot="1">
       <c r="A112" s="12" t="s">
         <v>431</v>
       </c>
@@ -10767,7 +10857,7 @@
         <v>7.6</v>
       </c>
     </row>
-    <row r="113" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="113" spans="1:18" ht="27" thickBot="1">
       <c r="A113" s="20" t="s">
         <v>455</v>
       </c>
@@ -10823,7 +10913,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="114" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="114" spans="1:18" ht="15" thickBot="1">
       <c r="A114" s="12" t="s">
         <v>494</v>
       </c>
@@ -10879,7 +10969,7 @@
         <v>6.1</v>
       </c>
     </row>
-    <row r="115" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="115" spans="1:18" ht="27" thickBot="1">
       <c r="A115" s="13" t="s">
         <v>538</v>
       </c>
@@ -10935,7 +11025,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="116" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="116" spans="1:18" ht="15" thickBot="1">
       <c r="A116" s="19" t="s">
         <v>582</v>
       </c>
@@ -10991,7 +11081,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="117" spans="1:18" ht="27" thickBot="1">
+    <row r="117" spans="1:18" ht="15" thickBot="1">
       <c r="A117" s="20" t="s">
         <v>563</v>
       </c>
@@ -11047,7 +11137,7 @@
         <v>6.8</v>
       </c>
     </row>
-    <row r="118" spans="1:18" ht="27" thickBot="1">
+    <row r="118" spans="1:18" ht="15" thickBot="1">
       <c r="A118" s="12" t="s">
         <v>558</v>
       </c>
@@ -11325,7 +11415,7 @@
         <v>6.1</v>
       </c>
     </row>
-    <row r="123" spans="1:18" ht="27" thickBot="1">
+    <row r="123" spans="1:18" ht="15" thickBot="1">
       <c r="A123" s="13" t="s">
         <v>302</v>
       </c>
@@ -11381,7 +11471,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="124" spans="1:18" ht="27" thickBot="1">
+    <row r="124" spans="1:18" ht="15" thickBot="1">
       <c r="A124" s="19" t="s">
         <v>627</v>
       </c>
@@ -11491,7 +11581,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="126" spans="1:18" ht="27" thickBot="1">
+    <row r="126" spans="1:18" ht="15" thickBot="1">
       <c r="A126" s="12" t="s">
         <v>304</v>
       </c>
@@ -11547,7 +11637,7 @@
         <v>7.1</v>
       </c>
     </row>
-    <row r="127" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="127" spans="1:18" ht="27" thickBot="1">
       <c r="A127" s="13" t="s">
         <v>543</v>
       </c>
@@ -11715,7 +11805,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="130" spans="1:18" ht="27" thickBot="1">
+    <row r="130" spans="1:18" ht="15" thickBot="1">
       <c r="A130" s="12" t="s">
         <v>400</v>
       </c>
@@ -11771,7 +11861,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="131" spans="1:18" ht="27" thickBot="1">
+    <row r="131" spans="1:18" ht="15" thickBot="1">
       <c r="A131" s="20" t="s">
         <v>532</v>
       </c>
@@ -11939,7 +12029,7 @@
         <v>6.4</v>
       </c>
     </row>
-    <row r="134" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="134" spans="1:18" ht="15" thickBot="1">
       <c r="A134" s="12" t="s">
         <v>539</v>
       </c>
@@ -11995,7 +12085,7 @@
         <v>6.5</v>
       </c>
     </row>
-    <row r="135" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="135" spans="1:18" ht="15" thickBot="1">
       <c r="A135" s="20" t="s">
         <v>528</v>
       </c>
@@ -12051,7 +12141,7 @@
         <v>6.3</v>
       </c>
     </row>
-    <row r="136" spans="1:18" ht="27" thickBot="1">
+    <row r="136" spans="1:18" ht="15" thickBot="1">
       <c r="A136" s="19" t="s">
         <v>404</v>
       </c>
@@ -12163,7 +12253,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="138" spans="1:18" ht="27" thickBot="1">
+    <row r="138" spans="1:18" ht="15" thickBot="1">
       <c r="A138" s="19" t="s">
         <v>605</v>
       </c>
@@ -12209,7 +12299,7 @@
         <v>4.9000000000000004</v>
       </c>
     </row>
-    <row r="139" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="139" spans="1:18" ht="27" thickBot="1">
       <c r="A139" s="13" t="s">
         <v>639</v>
       </c>
@@ -12263,7 +12353,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="140" spans="1:18" ht="27" thickBot="1">
+    <row r="140" spans="1:18" ht="15" thickBot="1">
       <c r="A140" s="12" t="s">
         <v>393</v>
       </c>
@@ -12599,7 +12689,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="146" spans="1:18" ht="53.4" thickBot="1">
+    <row r="146" spans="1:18" ht="27" thickBot="1">
       <c r="A146" s="12" t="s">
         <v>637</v>
       </c>
@@ -12653,7 +12743,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="147" spans="1:18" ht="27" thickBot="1">
+    <row r="147" spans="1:18" ht="15" thickBot="1">
       <c r="A147" s="20" t="s">
         <v>290</v>
       </c>
@@ -12709,7 +12799,7 @@
         <v>6.2</v>
       </c>
     </row>
-    <row r="148" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="148" spans="1:18" ht="27" thickBot="1">
       <c r="A148" s="12" t="s">
         <v>396</v>
       </c>
@@ -12821,7 +12911,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="150" spans="1:18" ht="27" thickBot="1">
+    <row r="150" spans="1:18" ht="15" thickBot="1">
       <c r="A150" s="19" t="s">
         <v>398</v>
       </c>
@@ -12877,7 +12967,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="151" spans="1:18" ht="27" thickBot="1">
+    <row r="151" spans="1:18" ht="15" thickBot="1">
       <c r="A151" s="13" t="s">
         <v>446</v>
       </c>
@@ -13101,7 +13191,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="155" spans="1:18" ht="27" thickBot="1">
+    <row r="155" spans="1:18" ht="15" thickBot="1">
       <c r="A155" s="13" t="s">
         <v>365</v>
       </c>
@@ -13213,7 +13303,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="157" spans="1:18" ht="27" thickBot="1">
+    <row r="157" spans="1:18" ht="15" thickBot="1">
       <c r="A157" s="20" t="s">
         <v>443</v>
       </c>
@@ -13325,7 +13415,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="159" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="159" spans="1:18" ht="15" thickBot="1">
       <c r="A159" s="20" t="s">
         <v>420</v>
       </c>
@@ -13435,7 +13525,7 @@
         <v>5.7</v>
       </c>
     </row>
-    <row r="161" spans="1:18" ht="27" thickBot="1">
+    <row r="161" spans="1:18" ht="15" thickBot="1">
       <c r="A161" s="20" t="s">
         <v>367</v>
       </c>
@@ -13823,7 +13913,7 @@
         <v>5.8</v>
       </c>
     </row>
-    <row r="168" spans="1:18" ht="27" thickBot="1">
+    <row r="168" spans="1:18" ht="15" thickBot="1">
       <c r="A168" s="12" t="s">
         <v>541</v>
       </c>
@@ -14047,7 +14137,7 @@
         <v>5.4</v>
       </c>
     </row>
-    <row r="172" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="172" spans="1:18" ht="15" thickBot="1">
       <c r="A172" s="12" t="s">
         <v>601</v>
       </c>
@@ -14093,7 +14183,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="173" spans="1:18" ht="27" thickBot="1">
+    <row r="173" spans="1:18" ht="15" thickBot="1">
       <c r="A173" s="13" t="s">
         <v>557</v>
       </c>
@@ -14261,7 +14351,7 @@
         <v>5.2</v>
       </c>
     </row>
-    <row r="176" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="176" spans="1:18" ht="27" thickBot="1">
       <c r="A176" s="19" t="s">
         <v>530</v>
       </c>
@@ -14809,7 +14899,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="186" spans="1:18" ht="66.599999999999994" thickBot="1">
+    <row r="186" spans="1:18" ht="27" thickBot="1">
       <c r="A186" s="19" t="s">
         <v>533</v>
       </c>
@@ -14981,8 +15071,8 @@
       <c r="A189" s="20" t="s">
         <v>225</v>
       </c>
-      <c r="B189" s="24">
-        <v>34</v>
+      <c r="B189" s="24" t="s">
+        <v>980</v>
       </c>
       <c r="C189" s="22" t="s">
         <v>36</v>
@@ -15033,7 +15123,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="190" spans="1:18" ht="27" thickBot="1">
+    <row r="190" spans="1:18" ht="15" thickBot="1">
       <c r="A190" s="12" t="s">
         <v>360</v>
       </c>
@@ -15089,7 +15179,7 @@
         <v>5.0999999999999996</v>
       </c>
     </row>
-    <row r="191" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="191" spans="1:18" ht="27" thickBot="1">
       <c r="A191" s="20" t="s">
         <v>606</v>
       </c>
@@ -15135,7 +15225,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="192" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="192" spans="1:18" ht="27" thickBot="1">
       <c r="A192" s="19" t="s">
         <v>607</v>
       </c>
@@ -15237,7 +15327,7 @@
         <v>4.8</v>
       </c>
     </row>
-    <row r="194" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="194" spans="1:18" ht="15" thickBot="1">
       <c r="A194" s="12" t="s">
         <v>476</v>
       </c>
@@ -15293,7 +15383,7 @@
         <v>4.5999999999999996</v>
       </c>
     </row>
-    <row r="195" spans="1:18" ht="27" thickBot="1">
+    <row r="195" spans="1:18" ht="15" thickBot="1">
       <c r="A195" s="13" t="s">
         <v>477</v>
       </c>
@@ -15461,7 +15551,7 @@
         <v>4.7</v>
       </c>
     </row>
-    <row r="198" spans="1:18" ht="27" thickBot="1">
+    <row r="198" spans="1:18" ht="15" thickBot="1">
       <c r="A198" s="12" t="s">
         <v>448</v>
       </c>
@@ -15517,7 +15607,7 @@
         <v>5.5</v>
       </c>
     </row>
-    <row r="199" spans="1:18" ht="27" thickBot="1">
+    <row r="199" spans="1:18" ht="15" thickBot="1">
       <c r="A199" s="13" t="s">
         <v>507</v>
       </c>
@@ -15577,8 +15667,8 @@
       <c r="A200" s="19" t="s">
         <v>514</v>
       </c>
-      <c r="B200" s="23">
-        <v>100</v>
+      <c r="B200" s="23" t="s">
+        <v>979</v>
       </c>
       <c r="C200" s="21" t="s">
         <v>29</v>
@@ -15687,8 +15777,8 @@
       <c r="A202" s="12" t="s">
         <v>514</v>
       </c>
-      <c r="B202" s="3">
-        <v>61</v>
+      <c r="B202" s="3" t="s">
+        <v>978</v>
       </c>
       <c r="C202" s="1" t="s">
         <v>29</v>
@@ -15851,7 +15941,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="205" spans="1:18" ht="53.4" thickBot="1">
+    <row r="205" spans="1:18" ht="27" thickBot="1">
       <c r="A205" s="20" t="s">
         <v>426</v>
       </c>
@@ -15907,7 +15997,7 @@
         <v>3.5</v>
       </c>
     </row>
-    <row r="206" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="206" spans="1:18" ht="15" thickBot="1">
       <c r="A206" s="12" t="s">
         <v>371</v>
       </c>
@@ -15963,7 +16053,7 @@
         <v>3.3</v>
       </c>
     </row>
-    <row r="207" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="207" spans="1:18" ht="27" thickBot="1">
       <c r="A207" s="20" t="s">
         <v>485</v>
       </c>
@@ -16187,7 +16277,7 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="211" spans="1:18" ht="40.200000000000003" thickBot="1">
+    <row r="211" spans="1:18" ht="27" thickBot="1">
       <c r="A211" s="39" t="s">
         <v>648</v>
       </c>
@@ -16246,13 +16336,27 @@
       <c r="B212" s="40" t="s">
         <v>652</v>
       </c>
-      <c r="C212" s="41"/>
-      <c r="D212" s="42"/>
-      <c r="E212" s="41"/>
-      <c r="F212" s="41"/>
-      <c r="G212" s="41"/>
-      <c r="H212" s="41"/>
-      <c r="I212" s="41"/>
+      <c r="C212" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="D212" s="42" t="s">
+        <v>60</v>
+      </c>
+      <c r="E212" s="41" t="s">
+        <v>424</v>
+      </c>
+      <c r="F212" s="41" t="s">
+        <v>425</v>
+      </c>
+      <c r="G212" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H212" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I212" s="52">
+        <v>45969</v>
+      </c>
       <c r="J212" s="40"/>
       <c r="K212" s="40"/>
       <c r="L212" s="43"/>
@@ -16275,19 +16379,34 @@
         <v>0</v>
       </c>
     </row>
-    <row r="213" spans="1:18" ht="26.4">
+    <row r="213" spans="1:18" ht="15" thickBot="1">
       <c r="A213" s="39" t="s">
         <v>653</v>
       </c>
       <c r="B213" s="40" t="s">
         <v>26</v>
       </c>
-      <c r="C213" s="41"/>
-      <c r="D213" s="42"/>
-      <c r="E213" s="41"/>
-      <c r="F213" s="41"/>
-      <c r="G213" s="41"/>
-      <c r="H213" s="41"/>
+      <c r="C213" s="41" t="s">
+        <v>59</v>
+      </c>
+      <c r="D213" s="42" t="s">
+        <v>60</v>
+      </c>
+      <c r="E213" s="41" t="s">
+        <v>982</v>
+      </c>
+      <c r="F213" s="41" t="s">
+        <v>266</v>
+      </c>
+      <c r="G213" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H213" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I213" s="45">
+        <v>45969</v>
+      </c>
       <c r="J213" s="40"/>
       <c r="K213" s="40"/>
       <c r="L213" s="43"/>
@@ -16307,6 +16426,354 @@
         <v>0</v>
       </c>
       <c r="R213" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="214" spans="1:18" ht="15" thickBot="1">
+      <c r="A214" s="39" t="s">
+        <v>963</v>
+      </c>
+      <c r="B214" s="40"/>
+      <c r="C214" s="41"/>
+      <c r="D214" s="42"/>
+      <c r="E214" s="41" t="s">
+        <v>359</v>
+      </c>
+      <c r="F214" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="G214" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H214" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I214" s="45">
+        <v>45969</v>
+      </c>
+      <c r="J214" s="40"/>
+      <c r="K214" s="40"/>
+      <c r="L214" s="43"/>
+      <c r="M214" s="41" t="s">
+        <v>647</v>
+      </c>
+      <c r="N214" s="40">
+        <v>1</v>
+      </c>
+      <c r="O214" s="40">
+        <v>0</v>
+      </c>
+      <c r="P214" s="46">
+        <v>0</v>
+      </c>
+      <c r="Q214" s="46">
+        <v>0</v>
+      </c>
+      <c r="R214" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="215" spans="1:18" ht="15" thickBot="1">
+      <c r="A215" s="39" t="s">
+        <v>964</v>
+      </c>
+      <c r="B215" s="40"/>
+      <c r="C215" s="41"/>
+      <c r="D215" s="42"/>
+      <c r="E215" s="41" t="s">
+        <v>359</v>
+      </c>
+      <c r="F215" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="G215" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H215" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I215" s="45">
+        <v>45969</v>
+      </c>
+      <c r="J215" s="40"/>
+      <c r="K215" s="40"/>
+      <c r="L215" s="43"/>
+      <c r="M215" s="41" t="s">
+        <v>647</v>
+      </c>
+      <c r="N215" s="40">
+        <v>1</v>
+      </c>
+      <c r="O215" s="40">
+        <v>0</v>
+      </c>
+      <c r="P215" s="46">
+        <v>0</v>
+      </c>
+      <c r="Q215" s="46">
+        <v>0</v>
+      </c>
+      <c r="R215" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="216" spans="1:18" ht="15" thickBot="1">
+      <c r="A216" s="39" t="s">
+        <v>965</v>
+      </c>
+      <c r="B216" s="40"/>
+      <c r="C216" s="41"/>
+      <c r="D216" s="42"/>
+      <c r="E216" s="41" t="s">
+        <v>359</v>
+      </c>
+      <c r="F216" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="G216" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H216" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I216" s="45">
+        <v>45969</v>
+      </c>
+      <c r="J216" s="40"/>
+      <c r="K216" s="40"/>
+      <c r="L216" s="43"/>
+      <c r="M216" s="41" t="s">
+        <v>647</v>
+      </c>
+      <c r="N216" s="40">
+        <v>1</v>
+      </c>
+      <c r="O216" s="40">
+        <v>0</v>
+      </c>
+      <c r="P216" s="46">
+        <v>0</v>
+      </c>
+      <c r="Q216" s="46">
+        <v>0</v>
+      </c>
+      <c r="R216" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="217" spans="1:18" ht="15" thickBot="1">
+      <c r="A217" s="39" t="s">
+        <v>966</v>
+      </c>
+      <c r="B217" s="40" t="s">
+        <v>976</v>
+      </c>
+      <c r="C217" s="41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D217" s="42" t="s">
+        <v>214</v>
+      </c>
+      <c r="E217" s="41" t="s">
+        <v>359</v>
+      </c>
+      <c r="F217" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="G217" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H217" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I217" s="45">
+        <v>45984</v>
+      </c>
+      <c r="J217" s="6">
+        <v>39.056086000000001</v>
+      </c>
+      <c r="K217" s="6">
+        <v>-77.114896999999999</v>
+      </c>
+      <c r="L217" s="43"/>
+      <c r="M217" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="N217" s="40">
+        <v>1</v>
+      </c>
+      <c r="O217" s="40">
+        <v>0</v>
+      </c>
+      <c r="P217" s="46">
+        <v>0</v>
+      </c>
+      <c r="Q217" s="46">
+        <v>0</v>
+      </c>
+      <c r="R217" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="218" spans="1:18" ht="15" thickBot="1">
+      <c r="A218" s="39" t="s">
+        <v>967</v>
+      </c>
+      <c r="B218" s="40" t="s">
+        <v>975</v>
+      </c>
+      <c r="C218" s="41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D218" s="42" t="s">
+        <v>214</v>
+      </c>
+      <c r="E218" s="41" t="s">
+        <v>359</v>
+      </c>
+      <c r="F218" s="41" t="s">
+        <v>62</v>
+      </c>
+      <c r="G218" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H218" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I218" s="45">
+        <v>45984</v>
+      </c>
+      <c r="J218" s="6">
+        <v>39.056086000000001</v>
+      </c>
+      <c r="K218" s="6">
+        <v>-77.114896999999999</v>
+      </c>
+      <c r="L218" s="43"/>
+      <c r="M218" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="N218" s="40">
+        <v>1</v>
+      </c>
+      <c r="O218" s="40">
+        <v>0</v>
+      </c>
+      <c r="P218" s="46">
+        <v>0</v>
+      </c>
+      <c r="Q218" s="46">
+        <v>0</v>
+      </c>
+      <c r="R218" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="219" spans="1:18" ht="15" thickBot="1">
+      <c r="A219" s="39" t="s">
+        <v>968</v>
+      </c>
+      <c r="B219" s="40" t="s">
+        <v>977</v>
+      </c>
+      <c r="C219" s="41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D219" s="42" t="s">
+        <v>970</v>
+      </c>
+      <c r="E219" s="41" t="s">
+        <v>971</v>
+      </c>
+      <c r="F219" s="41" t="s">
+        <v>127</v>
+      </c>
+      <c r="G219" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H219" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I219" s="45">
+        <v>45989</v>
+      </c>
+      <c r="J219" s="40">
+        <v>38.666018932416797</v>
+      </c>
+      <c r="K219" s="40">
+        <v>-90.608585713903693</v>
+      </c>
+      <c r="L219" s="43"/>
+      <c r="M219" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="N219" s="40">
+        <v>1</v>
+      </c>
+      <c r="O219" s="40">
+        <v>0</v>
+      </c>
+      <c r="P219" s="46">
+        <v>0</v>
+      </c>
+      <c r="Q219" s="46">
+        <v>0</v>
+      </c>
+      <c r="R219" s="47">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="220" spans="1:18">
+      <c r="A220" s="39" t="s">
+        <v>969</v>
+      </c>
+      <c r="B220" s="40" t="s">
+        <v>974</v>
+      </c>
+      <c r="C220" s="41" t="s">
+        <v>29</v>
+      </c>
+      <c r="D220" s="42" t="s">
+        <v>970</v>
+      </c>
+      <c r="E220" s="41" t="s">
+        <v>971</v>
+      </c>
+      <c r="F220" s="41" t="s">
+        <v>127</v>
+      </c>
+      <c r="G220" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H220" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="I220" s="45">
+        <v>45989</v>
+      </c>
+      <c r="J220" s="40">
+        <v>38.666018932416797</v>
+      </c>
+      <c r="K220" s="40">
+        <v>-90.608585713903693</v>
+      </c>
+      <c r="L220" s="43"/>
+      <c r="M220" s="41" t="s">
+        <v>26</v>
+      </c>
+      <c r="N220" s="40">
+        <v>1</v>
+      </c>
+      <c r="O220" s="40">
+        <v>0</v>
+      </c>
+      <c r="P220" s="46">
+        <v>0</v>
+      </c>
+      <c r="Q220" s="46">
+        <v>0</v>
+      </c>
+      <c r="R220" s="47">
         <v>0</v>
       </c>
     </row>
@@ -16321,7 +16788,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E690491F-A75A-44CD-AF5E-964C98F48B1D}">
-  <dimension ref="A1:I87"/>
+  <dimension ref="A1:H90"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="20.6640625" bestFit="1" customWidth="1"/>
@@ -16331,10 +16798,11 @@
     <col min="5" max="5" width="15.6640625" customWidth="1"/>
     <col min="6" max="6" width="10" customWidth="1"/>
     <col min="7" max="7" width="15.21875" customWidth="1"/>
+    <col min="8" max="8" width="87.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="75.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="15" thickBot="1">
+    <row r="1" spans="1:8" ht="15" thickBot="1">
       <c r="A1" s="48" t="s">
         <v>654</v>
       </c>
@@ -16348,22 +16816,19 @@
         <v>658</v>
       </c>
       <c r="E1" s="48" t="s">
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="F1" s="48" t="s">
-        <v>9</v>
-      </c>
-      <c r="G1" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="H1" s="49" t="s">
+      <c r="G1" s="49" t="s">
         <v>655</v>
       </c>
-      <c r="I1" s="50" t="s">
+      <c r="H1" s="50" t="s">
         <v>659</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:8">
       <c r="A2" t="s">
         <v>660</v>
       </c>
@@ -16376,23 +16841,20 @@
       <c r="D2" t="s">
         <v>24</v>
       </c>
-      <c r="E2" t="s">
-        <v>24</v>
+      <c r="E2">
+        <v>29.463383242077299</v>
       </c>
       <c r="F2">
-        <v>29.463383242077299</v>
-      </c>
-      <c r="G2">
         <v>-98.335771519372102</v>
       </c>
+      <c r="G2" t="s">
+        <v>663</v>
+      </c>
       <c r="H2" t="s">
-        <v>663</v>
-      </c>
-      <c r="I2" t="s">
         <v>661</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:8">
       <c r="A3" t="s">
         <v>664</v>
       </c>
@@ -16405,23 +16867,20 @@
       <c r="D3" t="s">
         <v>24</v>
       </c>
-      <c r="E3" t="s">
-        <v>24</v>
+      <c r="E3">
+        <v>41.094637674232096</v>
       </c>
       <c r="F3">
-        <v>41.094637674232096</v>
-      </c>
-      <c r="G3">
         <v>-83.661265806926806</v>
       </c>
+      <c r="G3" t="s">
+        <v>666</v>
+      </c>
       <c r="H3" t="s">
-        <v>666</v>
-      </c>
-      <c r="I3" t="s">
         <v>665</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:8">
       <c r="A4" t="s">
         <v>667</v>
       </c>
@@ -16434,23 +16893,20 @@
       <c r="D4" t="s">
         <v>24</v>
       </c>
-      <c r="E4" t="s">
-        <v>24</v>
+      <c r="E4">
+        <v>36.756490311024898</v>
       </c>
       <c r="F4">
-        <v>36.756490311024898</v>
-      </c>
-      <c r="G4">
         <v>-83.490698324576201</v>
       </c>
+      <c r="G4" t="s">
+        <v>669</v>
+      </c>
       <c r="H4" t="s">
-        <v>669</v>
-      </c>
-      <c r="I4" t="s">
         <v>668</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:8">
       <c r="A5" t="s">
         <v>670</v>
       </c>
@@ -16463,23 +16919,20 @@
       <c r="D5" t="s">
         <v>24</v>
       </c>
-      <c r="E5" t="s">
-        <v>24</v>
+      <c r="E5">
+        <v>30.237048753086999</v>
       </c>
       <c r="F5">
-        <v>30.237048753086999</v>
-      </c>
-      <c r="G5">
         <v>-81.302681827847593</v>
       </c>
+      <c r="G5" t="s">
+        <v>673</v>
+      </c>
       <c r="H5" t="s">
-        <v>673</v>
-      </c>
-      <c r="I5" t="s">
         <v>671</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:8">
       <c r="A6" t="s">
         <v>674</v>
       </c>
@@ -16492,23 +16945,20 @@
       <c r="D6" t="s">
         <v>24</v>
       </c>
-      <c r="E6" t="s">
-        <v>24</v>
+      <c r="E6">
+        <v>39.382735466011901</v>
       </c>
       <c r="F6">
-        <v>39.382735466011901</v>
-      </c>
-      <c r="G6">
         <v>-74.075276886054397</v>
       </c>
+      <c r="G6" t="s">
+        <v>676</v>
+      </c>
       <c r="H6" t="s">
-        <v>676</v>
-      </c>
-      <c r="I6" t="s">
         <v>675</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:8">
       <c r="A7" t="s">
         <v>334</v>
       </c>
@@ -16521,23 +16971,20 @@
       <c r="D7" t="s">
         <v>24</v>
       </c>
-      <c r="E7" t="s">
-        <v>24</v>
+      <c r="E7">
+        <v>41.762380767075598</v>
       </c>
       <c r="F7">
-        <v>41.762380767075598</v>
-      </c>
-      <c r="G7">
         <v>-69.964720011453906</v>
       </c>
+      <c r="G7" t="s">
+        <v>678</v>
+      </c>
       <c r="H7" t="s">
-        <v>678</v>
-      </c>
-      <c r="I7" t="s">
         <v>677</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:8">
       <c r="A8" t="s">
         <v>227</v>
       </c>
@@ -16550,23 +16997,20 @@
       <c r="D8" t="s">
         <v>24</v>
       </c>
-      <c r="E8" t="s">
-        <v>24</v>
+      <c r="E8">
+        <v>41.424445068117102</v>
       </c>
       <c r="F8">
-        <v>41.424445068117102</v>
-      </c>
-      <c r="G8">
         <v>-72.242355034482003</v>
       </c>
+      <c r="G8" t="s">
+        <v>680</v>
+      </c>
       <c r="H8" t="s">
-        <v>680</v>
-      </c>
-      <c r="I8" t="s">
         <v>679</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:8">
       <c r="A9" t="s">
         <v>681</v>
       </c>
@@ -16579,23 +17023,20 @@
       <c r="D9" t="s">
         <v>172</v>
       </c>
-      <c r="E9" t="s">
-        <v>177</v>
+      <c r="E9">
+        <v>46.059205916812402</v>
       </c>
       <c r="F9">
-        <v>46.059205916812402</v>
-      </c>
-      <c r="G9">
         <v>-73.751381735450806</v>
       </c>
+      <c r="G9" t="s">
+        <v>683</v>
+      </c>
       <c r="H9" t="s">
-        <v>683</v>
-      </c>
-      <c r="I9" t="s">
         <v>682</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:8">
       <c r="A10" t="s">
         <v>684</v>
       </c>
@@ -16606,25 +17047,22 @@
         <v>88</v>
       </c>
       <c r="D10" t="s">
-        <v>701</v>
-      </c>
-      <c r="E10" t="s">
         <v>700</v>
       </c>
+      <c r="E10">
+        <v>-31.301920080120301</v>
+      </c>
       <c r="F10">
-        <v>-31.301920080120301</v>
-      </c>
-      <c r="G10">
         <v>150.92525148123801</v>
       </c>
+      <c r="G10" t="s">
+        <v>686</v>
+      </c>
       <c r="H10" t="s">
-        <v>686</v>
-      </c>
-      <c r="I10" t="s">
         <v>685</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:8">
       <c r="A11" t="s">
         <v>687</v>
       </c>
@@ -16637,23 +17075,20 @@
       <c r="D11" t="s">
         <v>592</v>
       </c>
-      <c r="E11" t="s">
-        <v>593</v>
+      <c r="E11">
+        <v>38.266755018307997</v>
       </c>
       <c r="F11">
-        <v>38.266755018307997</v>
-      </c>
-      <c r="G11">
         <v>140.87937309661501</v>
       </c>
+      <c r="G11" t="s">
+        <v>690</v>
+      </c>
       <c r="H11" t="s">
-        <v>690</v>
-      </c>
-      <c r="I11" t="s">
         <v>689</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:8">
       <c r="A12" t="s">
         <v>691</v>
       </c>
@@ -16666,23 +17101,20 @@
       <c r="D12" t="s">
         <v>592</v>
       </c>
-      <c r="E12" t="s">
-        <v>593</v>
+      <c r="E12">
+        <v>35.339815509095899</v>
       </c>
       <c r="F12">
-        <v>35.339815509095899</v>
-      </c>
-      <c r="G12">
         <v>139.596898521875</v>
       </c>
+      <c r="G12" t="s">
+        <v>694</v>
+      </c>
       <c r="H12" t="s">
-        <v>694</v>
-      </c>
-      <c r="I12" t="s">
         <v>693</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:8">
       <c r="A13" t="s">
         <v>691</v>
       </c>
@@ -16695,23 +17127,20 @@
       <c r="D13" t="s">
         <v>592</v>
       </c>
-      <c r="E13" t="s">
-        <v>593</v>
+      <c r="E13">
+        <v>35.012908784767497</v>
       </c>
       <c r="F13">
-        <v>35.012908784767497</v>
-      </c>
-      <c r="G13">
         <v>135.81056759424601</v>
       </c>
+      <c r="G13" t="s">
+        <v>694</v>
+      </c>
       <c r="H13" t="s">
-        <v>694</v>
-      </c>
-      <c r="I13" t="s">
         <v>695</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:8">
       <c r="A14" t="s">
         <v>696</v>
       </c>
@@ -16724,115 +17153,103 @@
       <c r="D14" t="s">
         <v>592</v>
       </c>
-      <c r="E14" t="s">
-        <v>593</v>
+      <c r="E14">
+        <v>34.905430873998398</v>
       </c>
       <c r="F14">
-        <v>34.905430873998398</v>
-      </c>
-      <c r="G14">
         <v>135.820807959506</v>
       </c>
+      <c r="G14" t="s">
+        <v>698</v>
+      </c>
       <c r="H14" t="s">
-        <v>698</v>
-      </c>
-      <c r="I14" t="s">
         <v>697</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:8">
       <c r="A15" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B15" t="s">
-        <v>706</v>
+        <v>705</v>
       </c>
       <c r="C15" t="s">
         <v>88</v>
       </c>
       <c r="D15" t="s">
+        <v>706</v>
+      </c>
+      <c r="E15">
+        <v>-40.786415636732201</v>
+      </c>
+      <c r="F15">
+        <v>-71.580962813109593</v>
+      </c>
+      <c r="G15" t="s">
         <v>707</v>
       </c>
-      <c r="E15" t="s">
-        <v>722</v>
-      </c>
-      <c r="F15">
-        <v>-40.786415636732201</v>
-      </c>
-      <c r="G15">
-        <v>-71.580962813109593</v>
-      </c>
       <c r="H15" t="s">
-        <v>708</v>
-      </c>
-      <c r="I15" t="s">
-        <v>705</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9">
+        <v>704</v>
+      </c>
+    </row>
+    <row r="16" spans="1:8">
       <c r="A16" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B16" t="s">
-        <v>710</v>
+        <v>709</v>
       </c>
       <c r="C16" t="s">
         <v>88</v>
       </c>
       <c r="D16" t="s">
+        <v>706</v>
+      </c>
+      <c r="E16">
+        <v>-38.725857404054402</v>
+      </c>
+      <c r="F16">
+        <v>-71.756744063156802</v>
+      </c>
+      <c r="G16" t="s">
         <v>707</v>
-      </c>
-      <c r="E16" t="s">
-        <v>722</v>
-      </c>
-      <c r="F16">
-        <v>-38.725857404054402</v>
-      </c>
-      <c r="G16">
-        <v>-71.756744063156802</v>
       </c>
       <c r="H16" t="s">
         <v>708</v>
       </c>
-      <c r="I16" t="s">
-        <v>709</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9">
+    </row>
+    <row r="17" spans="1:8">
       <c r="A17" t="s">
-        <v>704</v>
+        <v>703</v>
       </c>
       <c r="B17" t="s">
-        <v>712</v>
+        <v>711</v>
       </c>
       <c r="C17" t="s">
         <v>88</v>
       </c>
       <c r="D17" t="s">
+        <v>706</v>
+      </c>
+      <c r="E17">
+        <v>-32.013300460726299</v>
+      </c>
+      <c r="F17">
+        <v>-67.307104194756405</v>
+      </c>
+      <c r="G17" t="s">
         <v>707</v>
       </c>
-      <c r="E17" t="s">
-        <v>722</v>
-      </c>
-      <c r="F17">
-        <v>-32.013300460726299</v>
-      </c>
-      <c r="G17">
-        <v>-67.307104194756405</v>
-      </c>
       <c r="H17" t="s">
-        <v>708</v>
-      </c>
-      <c r="I17" t="s">
-        <v>711</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9">
+        <v>710</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8">
       <c r="A18" t="s">
-        <v>714</v>
+        <v>713</v>
       </c>
       <c r="B18" t="s">
-        <v>716</v>
+        <v>715</v>
       </c>
       <c r="C18" t="s">
         <v>633</v>
@@ -16840,57 +17257,51 @@
       <c r="D18" t="s">
         <v>24</v>
       </c>
-      <c r="E18" t="s">
-        <v>24</v>
+      <c r="E18">
+        <v>52.433531012009098</v>
       </c>
       <c r="F18">
-        <v>52.433531012009098</v>
-      </c>
-      <c r="G18">
         <v>-123.22178013617</v>
       </c>
+      <c r="G18" t="s">
+        <v>714</v>
+      </c>
       <c r="H18" t="s">
-        <v>715</v>
-      </c>
-      <c r="I18" t="s">
-        <v>713</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9">
+        <v>712</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8">
       <c r="A19" t="s">
+        <v>716</v>
+      </c>
+      <c r="B19" t="s">
+        <v>719</v>
+      </c>
+      <c r="C19" t="s">
+        <v>720</v>
+      </c>
+      <c r="D19" t="s">
+        <v>24</v>
+      </c>
+      <c r="E19">
+        <v>41.013755634792503</v>
+      </c>
+      <c r="F19">
+        <v>-104.67981369292001</v>
+      </c>
+      <c r="G19" t="s">
         <v>717</v>
-      </c>
-      <c r="B19" t="s">
-        <v>720</v>
-      </c>
-      <c r="C19" t="s">
-        <v>721</v>
-      </c>
-      <c r="D19" t="s">
-        <v>24</v>
-      </c>
-      <c r="E19" t="s">
-        <v>24</v>
-      </c>
-      <c r="F19">
-        <v>41.013755634792503</v>
-      </c>
-      <c r="G19">
-        <v>-104.67981369292001</v>
       </c>
       <c r="H19" t="s">
         <v>718</v>
       </c>
-      <c r="I19" t="s">
-        <v>719</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9">
+    </row>
+    <row r="20" spans="1:8">
       <c r="A20" t="s">
-        <v>725</v>
+        <v>723</v>
       </c>
       <c r="B20" t="s">
-        <v>724</v>
+        <v>722</v>
       </c>
       <c r="C20" t="s">
         <v>43</v>
@@ -16898,28 +17309,25 @@
       <c r="D20" t="s">
         <v>24</v>
       </c>
-      <c r="E20" t="s">
-        <v>24</v>
+      <c r="E20">
+        <v>31.630322255398099</v>
       </c>
       <c r="F20">
-        <v>31.630322255398099</v>
-      </c>
-      <c r="G20">
         <v>-85.5425843592501</v>
       </c>
+      <c r="G20" t="s">
+        <v>724</v>
+      </c>
       <c r="H20" t="s">
+        <v>721</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8">
+      <c r="A21" t="s">
         <v>726</v>
       </c>
-      <c r="I20" t="s">
-        <v>723</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9">
-      <c r="A21" t="s">
-        <v>728</v>
-      </c>
       <c r="B21" t="s">
-        <v>729</v>
+        <v>727</v>
       </c>
       <c r="C21" t="s">
         <v>23</v>
@@ -16927,57 +17335,51 @@
       <c r="D21" t="s">
         <v>24</v>
       </c>
-      <c r="E21" t="s">
-        <v>24</v>
+      <c r="E21">
+        <v>40.747527963989199</v>
       </c>
       <c r="F21">
-        <v>40.747527963989199</v>
-      </c>
-      <c r="G21">
         <v>-75.217366002108193</v>
       </c>
+      <c r="G21" t="s">
+        <v>728</v>
+      </c>
       <c r="H21" t="s">
+        <v>725</v>
+      </c>
+    </row>
+    <row r="22" spans="1:8">
+      <c r="A22" t="s">
         <v>730</v>
       </c>
-      <c r="I21" t="s">
-        <v>727</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9">
-      <c r="A22" t="s">
+      <c r="B22" t="s">
+        <v>731</v>
+      </c>
+      <c r="C22" t="s">
         <v>732</v>
       </c>
-      <c r="B22" t="s">
+      <c r="D22" t="s">
+        <v>24</v>
+      </c>
+      <c r="E22">
+        <v>39.864495027195801</v>
+      </c>
+      <c r="F22">
+        <v>-88.989360409703806</v>
+      </c>
+      <c r="G22" t="s">
         <v>733</v>
       </c>
-      <c r="C22" t="s">
+      <c r="H22" t="s">
+        <v>729</v>
+      </c>
+    </row>
+    <row r="23" spans="1:8">
+      <c r="A23" t="s">
         <v>734</v>
       </c>
-      <c r="D22" t="s">
-        <v>24</v>
-      </c>
-      <c r="E22" t="s">
-        <v>24</v>
-      </c>
-      <c r="F22">
-        <v>39.864495027195801</v>
-      </c>
-      <c r="G22">
-        <v>-88.989360409703806</v>
-      </c>
-      <c r="H22" t="s">
-        <v>735</v>
-      </c>
-      <c r="I22" t="s">
-        <v>731</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9">
-      <c r="A23" t="s">
+      <c r="B23" t="s">
         <v>736</v>
-      </c>
-      <c r="B23" t="s">
-        <v>738</v>
       </c>
       <c r="C23" t="s">
         <v>248</v>
@@ -16985,28 +17387,25 @@
       <c r="D23" t="s">
         <v>24</v>
       </c>
-      <c r="E23" t="s">
-        <v>24</v>
+      <c r="E23">
+        <v>32.981457350907903</v>
       </c>
       <c r="F23">
-        <v>32.981457350907903</v>
-      </c>
-      <c r="G23">
         <v>-97.248080019994205</v>
       </c>
+      <c r="G23" t="s">
+        <v>737</v>
+      </c>
       <c r="H23" t="s">
+        <v>735</v>
+      </c>
+    </row>
+    <row r="24" spans="1:8">
+      <c r="A24" t="s">
         <v>739</v>
       </c>
-      <c r="I23" t="s">
-        <v>737</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9">
-      <c r="A24" t="s">
+      <c r="B24" t="s">
         <v>741</v>
-      </c>
-      <c r="B24" t="s">
-        <v>743</v>
       </c>
       <c r="C24" t="s">
         <v>248</v>
@@ -17014,28 +17413,25 @@
       <c r="D24" t="s">
         <v>24</v>
       </c>
-      <c r="E24" t="s">
-        <v>24</v>
+      <c r="E24">
+        <v>30.419982573452302</v>
       </c>
       <c r="F24">
-        <v>30.419982573452302</v>
-      </c>
-      <c r="G24">
         <v>-95.488375549339693</v>
       </c>
+      <c r="G24" t="s">
+        <v>742</v>
+      </c>
       <c r="H24" t="s">
+        <v>740</v>
+      </c>
+    </row>
+    <row r="25" spans="1:8">
+      <c r="A25" t="s">
         <v>744</v>
       </c>
-      <c r="I24" t="s">
-        <v>742</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9">
-      <c r="A25" t="s">
-        <v>746</v>
-      </c>
       <c r="B25" t="s">
-        <v>747</v>
+        <v>745</v>
       </c>
       <c r="C25" t="s">
         <v>376</v>
@@ -17043,28 +17439,25 @@
       <c r="D25" t="s">
         <v>24</v>
       </c>
-      <c r="E25" t="s">
-        <v>24</v>
+      <c r="E25">
+        <v>45.652471967540798</v>
       </c>
       <c r="F25">
-        <v>45.652471967540798</v>
-      </c>
-      <c r="G25">
         <v>-94.631015820070601</v>
       </c>
+      <c r="G25" t="s">
+        <v>746</v>
+      </c>
       <c r="H25" t="s">
+        <v>743</v>
+      </c>
+    </row>
+    <row r="26" spans="1:8">
+      <c r="A26" t="s">
         <v>748</v>
       </c>
-      <c r="I25" t="s">
-        <v>745</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9">
-      <c r="A26" t="s">
-        <v>750</v>
-      </c>
       <c r="B26" t="s">
-        <v>751</v>
+        <v>749</v>
       </c>
       <c r="C26" t="s">
         <v>425</v>
@@ -17072,28 +17465,25 @@
       <c r="D26" t="s">
         <v>24</v>
       </c>
-      <c r="E26" t="s">
-        <v>24</v>
+      <c r="E26">
+        <v>38.6044143871462</v>
       </c>
       <c r="F26">
-        <v>38.6044143871462</v>
-      </c>
-      <c r="G26">
         <v>-121.970852569643</v>
       </c>
+      <c r="G26" t="s">
+        <v>750</v>
+      </c>
       <c r="H26" t="s">
+        <v>747</v>
+      </c>
+    </row>
+    <row r="27" spans="1:8">
+      <c r="A27" t="s">
+        <v>751</v>
+      </c>
+      <c r="B27" t="s">
         <v>752</v>
-      </c>
-      <c r="I26" t="s">
-        <v>749</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9">
-      <c r="A27" t="s">
-        <v>753</v>
-      </c>
-      <c r="B27" t="s">
-        <v>754</v>
       </c>
       <c r="C27" t="s">
         <v>376</v>
@@ -17101,28 +17491,25 @@
       <c r="D27" t="s">
         <v>24</v>
       </c>
-      <c r="E27" t="s">
-        <v>24</v>
+      <c r="E27">
+        <v>44.912860602563299</v>
       </c>
       <c r="F27">
-        <v>44.912860602563299</v>
-      </c>
-      <c r="G27">
         <v>-93.159409454946299</v>
       </c>
+      <c r="G27" t="s">
+        <v>754</v>
+      </c>
       <c r="H27" t="s">
+        <v>753</v>
+      </c>
+    </row>
+    <row r="28" spans="1:8">
+      <c r="A28" t="s">
+        <v>755</v>
+      </c>
+      <c r="B28" t="s">
         <v>756</v>
-      </c>
-      <c r="I27" t="s">
-        <v>755</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9">
-      <c r="A28" t="s">
-        <v>757</v>
-      </c>
-      <c r="B28" t="s">
-        <v>758</v>
       </c>
       <c r="C28" t="s">
         <v>199</v>
@@ -17130,25 +17517,22 @@
       <c r="D28" t="s">
         <v>24</v>
       </c>
-      <c r="E28" t="s">
-        <v>24</v>
+      <c r="E28">
+        <v>43.087409565957998</v>
       </c>
       <c r="F28">
-        <v>43.087409565957998</v>
-      </c>
-      <c r="G28">
         <v>-70.765013104871798</v>
       </c>
+      <c r="G28" t="s">
+        <v>757</v>
+      </c>
       <c r="H28" t="s">
+        <v>758</v>
+      </c>
+    </row>
+    <row r="29" spans="1:8">
+      <c r="A29" t="s">
         <v>759</v>
-      </c>
-      <c r="I28" t="s">
-        <v>760</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9">
-      <c r="A29" t="s">
-        <v>761</v>
       </c>
       <c r="B29" t="s">
         <v>118</v>
@@ -17159,28 +17543,25 @@
       <c r="D29" t="s">
         <v>24</v>
       </c>
-      <c r="E29" t="s">
-        <v>24</v>
+      <c r="E29">
+        <v>42.513539232803197</v>
       </c>
       <c r="F29">
-        <v>42.513539232803197</v>
-      </c>
-      <c r="G29">
         <v>-70.858736422377703</v>
       </c>
+      <c r="G29" t="s">
+        <v>761</v>
+      </c>
       <c r="H29" t="s">
-        <v>763</v>
-      </c>
-      <c r="I29" t="s">
+        <v>760</v>
+      </c>
+    </row>
+    <row r="30" spans="1:8" ht="28.8">
+      <c r="A30" s="51" t="s">
         <v>762</v>
       </c>
-    </row>
-    <row r="30" spans="1:9" ht="28.8">
-      <c r="A30" s="51" t="s">
+      <c r="B30" t="s">
         <v>764</v>
-      </c>
-      <c r="B30" t="s">
-        <v>766</v>
       </c>
       <c r="C30" t="s">
         <v>43</v>
@@ -17188,106 +17569,103 @@
       <c r="D30" t="s">
         <v>24</v>
       </c>
-      <c r="E30" t="s">
-        <v>24</v>
+      <c r="E30">
+        <v>28.3912216062288</v>
       </c>
       <c r="F30">
-        <v>28.3912216062288</v>
-      </c>
-      <c r="G30">
         <v>-82.575119545015397</v>
       </c>
+      <c r="G30" t="s">
+        <v>765</v>
+      </c>
       <c r="H30" t="s">
+        <v>763</v>
+      </c>
+    </row>
+    <row r="31" spans="1:8">
+      <c r="A31" t="s">
+        <v>766</v>
+      </c>
+      <c r="B31" t="s">
         <v>767</v>
-      </c>
-      <c r="I30" t="s">
-        <v>765</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9">
-      <c r="A31" t="s">
-        <v>768</v>
-      </c>
-      <c r="B31" t="s">
-        <v>769</v>
       </c>
       <c r="C31" t="s">
         <v>88</v>
       </c>
       <c r="D31" t="s">
+        <v>768</v>
+      </c>
+      <c r="E31">
+        <v>32.698968976301302</v>
+      </c>
+      <c r="F31">
+        <v>-16.861378151127099</v>
+      </c>
+      <c r="G31" t="s">
         <v>770</v>
       </c>
-      <c r="F31">
-        <v>32.698968976301302</v>
-      </c>
-      <c r="G31">
-        <v>-16.861378151127099</v>
-      </c>
       <c r="H31" t="s">
+        <v>769</v>
+      </c>
+    </row>
+    <row r="32" spans="1:8">
+      <c r="A32" t="s">
         <v>772</v>
       </c>
-      <c r="I31" t="s">
-        <v>771</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9">
-      <c r="A32" t="s">
-        <v>774</v>
-      </c>
       <c r="B32" t="s">
-        <v>775</v>
+        <v>773</v>
       </c>
       <c r="C32" t="s">
         <v>88</v>
       </c>
       <c r="D32" t="s">
-        <v>770</v>
+        <v>768</v>
+      </c>
+      <c r="E32">
+        <v>39.036139407971199</v>
       </c>
       <c r="F32">
-        <v>39.036139407971199</v>
-      </c>
-      <c r="G32">
         <v>-9.2255342942693908</v>
       </c>
+      <c r="G32" t="s">
+        <v>774</v>
+      </c>
       <c r="H32" t="s">
+        <v>771</v>
+      </c>
+    </row>
+    <row r="33" spans="1:8">
+      <c r="A33" t="s">
+        <v>775</v>
+      </c>
+      <c r="B33" t="s">
         <v>776</v>
-      </c>
-      <c r="I32" t="s">
-        <v>773</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9">
-      <c r="A33" t="s">
-        <v>777</v>
-      </c>
-      <c r="B33" t="s">
-        <v>778</v>
       </c>
       <c r="C33" t="s">
         <v>88</v>
       </c>
       <c r="D33" t="s">
-        <v>770</v>
+        <v>768</v>
+      </c>
+      <c r="E33">
+        <v>41.351962361722599</v>
       </c>
       <c r="F33">
-        <v>41.351962361722599</v>
-      </c>
-      <c r="G33">
         <v>-7.3798311687738796</v>
       </c>
+      <c r="G33" t="s">
+        <v>778</v>
+      </c>
       <c r="H33" t="s">
-        <v>780</v>
-      </c>
-      <c r="I33" t="s">
+        <v>777</v>
+      </c>
+    </row>
+    <row r="34" spans="1:8">
+      <c r="A34" t="s">
         <v>779</v>
       </c>
-    </row>
-    <row r="34" spans="1:9">
-      <c r="A34" t="s">
+      <c r="B34" t="s">
         <v>781</v>
-      </c>
-      <c r="B34" t="s">
-        <v>783</v>
       </c>
       <c r="C34" t="s">
         <v>88</v>
@@ -17295,20 +17673,20 @@
       <c r="D34" t="s">
         <v>68</v>
       </c>
+      <c r="E34">
+        <v>41.294194149250401</v>
+      </c>
       <c r="F34">
-        <v>41.294194149250401</v>
-      </c>
-      <c r="G34">
         <v>-4.1820650812680196</v>
       </c>
+      <c r="G34" t="s">
+        <v>782</v>
+      </c>
       <c r="H34" t="s">
-        <v>784</v>
-      </c>
-      <c r="I34" t="s">
-        <v>782</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9">
+        <v>780</v>
+      </c>
+    </row>
+    <row r="35" spans="1:8">
       <c r="A35" t="s">
         <v>491</v>
       </c>
@@ -17321,25 +17699,25 @@
       <c r="D35" t="s">
         <v>68</v>
       </c>
+      <c r="E35">
+        <v>40.721797077446197</v>
+      </c>
       <c r="F35">
-        <v>40.721797077446197</v>
-      </c>
-      <c r="G35">
         <v>-3.4235315612319299</v>
       </c>
+      <c r="G35" t="s">
+        <v>784</v>
+      </c>
       <c r="H35" t="s">
-        <v>786</v>
-      </c>
-      <c r="I35" t="s">
+        <v>783</v>
+      </c>
+    </row>
+    <row r="36" spans="1:8">
+      <c r="A36" t="s">
         <v>785</v>
       </c>
-    </row>
-    <row r="36" spans="1:9">
-      <c r="A36" t="s">
+      <c r="B36" t="s">
         <v>787</v>
-      </c>
-      <c r="B36" t="s">
-        <v>789</v>
       </c>
       <c r="C36" t="s">
         <v>88</v>
@@ -17347,22 +17725,22 @@
       <c r="D36" t="s">
         <v>68</v>
       </c>
+      <c r="E36">
+        <v>40.052125191398602</v>
+      </c>
       <c r="F36">
-        <v>40.052125191398602</v>
-      </c>
-      <c r="G36">
         <v>-3.3718133666840102</v>
       </c>
-      <c r="I36" t="s">
+      <c r="H36" t="s">
+        <v>786</v>
+      </c>
+    </row>
+    <row r="37" spans="1:8">
+      <c r="A37" t="s">
         <v>788</v>
       </c>
-    </row>
-    <row r="37" spans="1:9">
-      <c r="A37" t="s">
+      <c r="B37" t="s">
         <v>790</v>
-      </c>
-      <c r="B37" t="s">
-        <v>792</v>
       </c>
       <c r="C37" t="s">
         <v>88</v>
@@ -17370,25 +17748,25 @@
       <c r="D37" t="s">
         <v>68</v>
       </c>
+      <c r="E37">
+        <v>41.810234875948503</v>
+      </c>
       <c r="F37">
-        <v>41.810234875948503</v>
-      </c>
-      <c r="G37">
         <v>-6.1848916288551999E-2</v>
       </c>
+      <c r="G37" t="s">
+        <v>791</v>
+      </c>
       <c r="H37" t="s">
+        <v>789</v>
+      </c>
+    </row>
+    <row r="38" spans="1:8">
+      <c r="A38" t="s">
+        <v>792</v>
+      </c>
+      <c r="B38" t="s">
         <v>793</v>
-      </c>
-      <c r="I37" t="s">
-        <v>791</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9">
-      <c r="A38" t="s">
-        <v>794</v>
-      </c>
-      <c r="B38" t="s">
-        <v>795</v>
       </c>
       <c r="C38" t="s">
         <v>88</v>
@@ -17396,25 +17774,25 @@
       <c r="D38" t="s">
         <v>68</v>
       </c>
+      <c r="E38">
+        <v>43.458849891467899</v>
+      </c>
       <c r="F38">
-        <v>43.458849891467899</v>
-      </c>
-      <c r="G38">
         <v>-2.0443797072919598</v>
       </c>
+      <c r="G38" t="s">
+        <v>784</v>
+      </c>
       <c r="H38" t="s">
-        <v>786</v>
-      </c>
-      <c r="I38" t="s">
+        <v>794</v>
+      </c>
+    </row>
+    <row r="39" spans="1:8">
+      <c r="A39" t="s">
         <v>796</v>
       </c>
-    </row>
-    <row r="39" spans="1:9">
-      <c r="A39" t="s">
+      <c r="B39" t="s">
         <v>798</v>
-      </c>
-      <c r="B39" t="s">
-        <v>800</v>
       </c>
       <c r="C39" t="s">
         <v>88</v>
@@ -17422,25 +17800,25 @@
       <c r="D39" t="s">
         <v>68</v>
       </c>
+      <c r="E39">
+        <v>39.612507832099098</v>
+      </c>
       <c r="F39">
-        <v>39.612507832099098</v>
-      </c>
-      <c r="G39">
         <v>-0.17264615686895099</v>
+      </c>
+      <c r="G39" t="s">
+        <v>795</v>
       </c>
       <c r="H39" t="s">
         <v>797</v>
       </c>
-      <c r="I39" t="s">
-        <v>799</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9">
+    </row>
+    <row r="40" spans="1:8">
       <c r="A40" t="s">
         <v>458</v>
       </c>
       <c r="B40" t="s">
-        <v>802</v>
+        <v>800</v>
       </c>
       <c r="C40" t="s">
         <v>88</v>
@@ -17448,22 +17826,22 @@
       <c r="D40" t="s">
         <v>68</v>
       </c>
+      <c r="E40">
+        <v>38.649531481995503</v>
+      </c>
       <c r="F40">
-        <v>38.649531481995503</v>
-      </c>
-      <c r="G40">
         <v>-0.161659828717404</v>
       </c>
-      <c r="I40" t="s">
-        <v>801</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9">
+      <c r="H40" t="s">
+        <v>799</v>
+      </c>
+    </row>
+    <row r="41" spans="1:8">
       <c r="A41" t="s">
-        <v>798</v>
+        <v>796</v>
       </c>
       <c r="B41" t="s">
-        <v>804</v>
+        <v>802</v>
       </c>
       <c r="C41" t="s">
         <v>88</v>
@@ -17471,20 +17849,20 @@
       <c r="D41" t="s">
         <v>68</v>
       </c>
+      <c r="E41">
+        <v>41.523431604823699</v>
+      </c>
       <c r="F41">
-        <v>41.523431604823699</v>
-      </c>
-      <c r="G41">
         <v>2.1674417340687002</v>
       </c>
+      <c r="G41" t="s">
+        <v>795</v>
+      </c>
       <c r="H41" t="s">
-        <v>797</v>
-      </c>
-      <c r="I41" t="s">
-        <v>803</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9">
+        <v>801</v>
+      </c>
+    </row>
+    <row r="42" spans="1:8">
       <c r="A42" t="s">
         <v>66</v>
       </c>
@@ -17497,20 +17875,20 @@
       <c r="D42" t="s">
         <v>68</v>
       </c>
+      <c r="E42">
+        <v>41.523431613458399</v>
+      </c>
       <c r="F42">
-        <v>41.523431613458399</v>
-      </c>
-      <c r="G42">
         <v>2.5409768902508598</v>
       </c>
+      <c r="G42" t="s">
+        <v>804</v>
+      </c>
       <c r="H42" t="s">
-        <v>806</v>
-      </c>
-      <c r="I42" t="s">
-        <v>805</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9">
+        <v>803</v>
+      </c>
+    </row>
+    <row r="43" spans="1:8">
       <c r="A43" t="s">
         <v>156</v>
       </c>
@@ -17523,25 +17901,25 @@
       <c r="D43" t="s">
         <v>158</v>
       </c>
+      <c r="E43">
+        <v>48.973399886181802</v>
+      </c>
       <c r="F43">
-        <v>48.973399886181802</v>
-      </c>
-      <c r="G43">
         <v>2.30468277539183</v>
       </c>
+      <c r="G43" t="s">
+        <v>806</v>
+      </c>
       <c r="H43" t="s">
+        <v>805</v>
+      </c>
+    </row>
+    <row r="44" spans="1:8">
+      <c r="A44" t="s">
+        <v>807</v>
+      </c>
+      <c r="B44" t="s">
         <v>808</v>
-      </c>
-      <c r="I43" t="s">
-        <v>807</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9">
-      <c r="A44" t="s">
-        <v>809</v>
-      </c>
-      <c r="B44" t="s">
-        <v>810</v>
       </c>
       <c r="C44" t="s">
         <v>88</v>
@@ -17549,48 +17927,48 @@
       <c r="D44" t="s">
         <v>158</v>
       </c>
+      <c r="E44">
+        <v>43.771369444886702</v>
+      </c>
       <c r="F44">
-        <v>43.771369444886702</v>
-      </c>
-      <c r="G44">
         <v>7.2646827520436696</v>
       </c>
+      <c r="G44" t="s">
+        <v>810</v>
+      </c>
       <c r="H44" t="s">
+        <v>809</v>
+      </c>
+    </row>
+    <row r="45" spans="1:8">
+      <c r="A45" t="s">
+        <v>814</v>
+      </c>
+      <c r="B45" t="s">
         <v>812</v>
-      </c>
-      <c r="I44" t="s">
-        <v>811</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9">
-      <c r="A45" t="s">
-        <v>816</v>
-      </c>
-      <c r="B45" t="s">
-        <v>814</v>
       </c>
       <c r="C45" t="s">
         <v>88</v>
       </c>
       <c r="D45" t="s">
-        <v>828</v>
+        <v>826</v>
+      </c>
+      <c r="E45">
+        <v>52.711779660655402</v>
       </c>
       <c r="F45">
-        <v>52.711779660655402</v>
-      </c>
-      <c r="G45">
         <v>-2.7544210462605099</v>
       </c>
+      <c r="G45" t="s">
+        <v>813</v>
+      </c>
       <c r="H45" t="s">
+        <v>811</v>
+      </c>
+    </row>
+    <row r="46" spans="1:8">
+      <c r="A46" t="s">
         <v>815</v>
-      </c>
-      <c r="I45" t="s">
-        <v>813</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9">
-      <c r="A46" t="s">
-        <v>817</v>
       </c>
       <c r="B46" t="s">
         <v>101</v>
@@ -17599,48 +17977,48 @@
         <v>88</v>
       </c>
       <c r="D46" t="s">
-        <v>828</v>
+        <v>826</v>
+      </c>
+      <c r="E46">
+        <v>52.131304915221598</v>
       </c>
       <c r="F46">
-        <v>52.131304915221598</v>
-      </c>
-      <c r="G46">
         <v>2.3116018557096701E-2</v>
       </c>
+      <c r="G46" t="s">
+        <v>817</v>
+      </c>
       <c r="H46" t="s">
+        <v>816</v>
+      </c>
+    </row>
+    <row r="47" spans="1:8">
+      <c r="A47" t="s">
+        <v>818</v>
+      </c>
+      <c r="B47" t="s">
         <v>819</v>
-      </c>
-      <c r="I46" t="s">
-        <v>818</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9">
-      <c r="A47" t="s">
-        <v>820</v>
-      </c>
-      <c r="B47" t="s">
-        <v>821</v>
       </c>
       <c r="C47" t="s">
         <v>88</v>
       </c>
       <c r="D47" t="s">
-        <v>828</v>
+        <v>826</v>
+      </c>
+      <c r="E47">
+        <v>50.824919945324702</v>
       </c>
       <c r="F47">
-        <v>50.824919945324702</v>
-      </c>
-      <c r="G47">
         <v>-0.14456399091611599</v>
       </c>
+      <c r="G47" t="s">
+        <v>821</v>
+      </c>
       <c r="H47" t="s">
-        <v>823</v>
-      </c>
-      <c r="I47" t="s">
-        <v>822</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9">
+        <v>820</v>
+      </c>
+    </row>
+    <row r="48" spans="1:8">
       <c r="A48" t="s">
         <v>458</v>
       </c>
@@ -17651,22 +18029,22 @@
         <v>88</v>
       </c>
       <c r="D48" t="s">
-        <v>828</v>
+        <v>826</v>
+      </c>
+      <c r="E48">
+        <v>51.544533375625001</v>
       </c>
       <c r="F48">
-        <v>51.544533375625001</v>
-      </c>
-      <c r="G48">
         <v>-0.14992233319881601</v>
       </c>
+      <c r="G48" t="s">
+        <v>823</v>
+      </c>
       <c r="H48" t="s">
-        <v>825</v>
-      </c>
-      <c r="I48" t="s">
-        <v>824</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9">
+        <v>822</v>
+      </c>
+    </row>
+    <row r="49" spans="1:8">
       <c r="A49" t="s">
         <v>458</v>
       </c>
@@ -17677,22 +18055,22 @@
         <v>88</v>
       </c>
       <c r="D49" t="s">
-        <v>828</v>
+        <v>826</v>
+      </c>
+      <c r="E49">
+        <v>51.513388843156498</v>
       </c>
       <c r="F49">
-        <v>51.513388843156498</v>
-      </c>
-      <c r="G49">
         <v>-0.13013037045387099</v>
       </c>
+      <c r="G49" t="s">
+        <v>823</v>
+      </c>
       <c r="H49" t="s">
-        <v>825</v>
-      </c>
-      <c r="I49" t="s">
-        <v>826</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9">
+        <v>824</v>
+      </c>
+    </row>
+    <row r="50" spans="1:8">
       <c r="A50" t="s">
         <v>458</v>
       </c>
@@ -17703,27 +18081,27 @@
         <v>88</v>
       </c>
       <c r="D50" t="s">
-        <v>828</v>
+        <v>826</v>
+      </c>
+      <c r="E50">
+        <v>51.495996583316597</v>
       </c>
       <c r="F50">
-        <v>51.495996583316597</v>
-      </c>
-      <c r="G50">
         <v>-0.14526540078824099</v>
+      </c>
+      <c r="G50" t="s">
+        <v>823</v>
       </c>
       <c r="H50" t="s">
         <v>825</v>
       </c>
-      <c r="I50" t="s">
+    </row>
+    <row r="51" spans="1:8">
+      <c r="A51" t="s">
         <v>827</v>
       </c>
-    </row>
-    <row r="51" spans="1:9">
-      <c r="A51" t="s">
+      <c r="B51" t="s">
         <v>829</v>
-      </c>
-      <c r="B51" t="s">
-        <v>831</v>
       </c>
       <c r="C51" t="s">
         <v>88</v>
@@ -17731,20 +18109,20 @@
       <c r="D51" t="s">
         <v>649</v>
       </c>
+      <c r="E51">
+        <v>52.378198062539497</v>
+      </c>
       <c r="F51">
-        <v>52.378198062539497</v>
-      </c>
-      <c r="G51">
         <v>4.5170594911307704</v>
       </c>
+      <c r="G51" t="s">
+        <v>830</v>
+      </c>
       <c r="H51" t="s">
-        <v>832</v>
-      </c>
-      <c r="I51" t="s">
-        <v>830</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9">
+        <v>828</v>
+      </c>
+    </row>
+    <row r="52" spans="1:8">
       <c r="A52" t="s">
         <v>526</v>
       </c>
@@ -17757,22 +18135,22 @@
       <c r="D52" t="s">
         <v>649</v>
       </c>
+      <c r="E52">
+        <v>52.375070075125102</v>
+      </c>
       <c r="F52">
-        <v>52.375070075125102</v>
-      </c>
-      <c r="G52">
         <v>4.8883119454223003</v>
       </c>
+      <c r="G52" t="s">
+        <v>832</v>
+      </c>
       <c r="H52" t="s">
-        <v>834</v>
-      </c>
-      <c r="I52" t="s">
+        <v>831</v>
+      </c>
+    </row>
+    <row r="53" spans="1:8">
+      <c r="A53" t="s">
         <v>833</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9">
-      <c r="A53" t="s">
-        <v>835</v>
       </c>
       <c r="B53" t="s">
         <v>524</v>
@@ -17783,19 +18161,19 @@
       <c r="D53" t="s">
         <v>649</v>
       </c>
+      <c r="E53">
+        <v>52.370196721388403</v>
+      </c>
       <c r="F53">
-        <v>52.370196721388403</v>
-      </c>
-      <c r="G53">
         <v>4.8920884957162798</v>
       </c>
-      <c r="I53" t="s">
+      <c r="H53" t="s">
+        <v>834</v>
+      </c>
+    </row>
+    <row r="54" spans="1:8">
+      <c r="A54" t="s">
         <v>836</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9">
-      <c r="A54" t="s">
-        <v>838</v>
       </c>
       <c r="B54" t="s">
         <v>524</v>
@@ -17806,19 +18184,19 @@
       <c r="D54" t="s">
         <v>649</v>
       </c>
+      <c r="E54">
+        <v>52.371873634966299</v>
+      </c>
       <c r="F54">
-        <v>52.371873634966299</v>
-      </c>
-      <c r="G54">
         <v>4.89612253807576</v>
       </c>
-      <c r="I54" t="s">
-        <v>837</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9">
+      <c r="H54" t="s">
+        <v>835</v>
+      </c>
+    </row>
+    <row r="55" spans="1:8">
       <c r="A55" t="s">
-        <v>835</v>
+        <v>833</v>
       </c>
       <c r="B55" t="s">
         <v>524</v>
@@ -17829,22 +18207,22 @@
       <c r="D55" t="s">
         <v>649</v>
       </c>
+      <c r="E55">
+        <v>52.375594059638097</v>
+      </c>
       <c r="F55">
-        <v>52.375594059638097</v>
-      </c>
-      <c r="G55">
         <v>4.9023881783362304</v>
       </c>
-      <c r="I55" t="s">
-        <v>839</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9">
+      <c r="H55" t="s">
+        <v>837</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8">
       <c r="A56" t="s">
+        <v>838</v>
+      </c>
+      <c r="B56" t="s">
         <v>840</v>
-      </c>
-      <c r="B56" t="s">
-        <v>842</v>
       </c>
       <c r="C56" t="s">
         <v>88</v>
@@ -17852,25 +18230,25 @@
       <c r="D56" t="s">
         <v>649</v>
       </c>
+      <c r="E56">
+        <v>50.853174792217501</v>
+      </c>
       <c r="F56">
-        <v>50.853174792217501</v>
-      </c>
-      <c r="G56">
         <v>5.69135731114772</v>
       </c>
+      <c r="G56" t="s">
+        <v>841</v>
+      </c>
       <c r="H56" t="s">
-        <v>843</v>
-      </c>
-      <c r="I56" t="s">
-        <v>841</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9">
+        <v>839</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8">
       <c r="A57" t="s">
+        <v>842</v>
+      </c>
+      <c r="B57" t="s">
         <v>844</v>
-      </c>
-      <c r="B57" t="s">
-        <v>846</v>
       </c>
       <c r="C57" t="s">
         <v>88</v>
@@ -17878,22 +18256,22 @@
       <c r="D57" t="s">
         <v>571</v>
       </c>
+      <c r="E57">
+        <v>51.878187806059799</v>
+      </c>
       <c r="F57">
-        <v>51.878187806059799</v>
-      </c>
-      <c r="G57">
         <v>6.6960724324398102</v>
       </c>
+      <c r="G57" t="s">
+        <v>845</v>
+      </c>
       <c r="H57" t="s">
-        <v>847</v>
-      </c>
-      <c r="I57" t="s">
-        <v>845</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9">
+        <v>843</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8">
       <c r="A58" t="s">
-        <v>848</v>
+        <v>846</v>
       </c>
       <c r="B58" t="s">
         <v>570</v>
@@ -17904,22 +18282,22 @@
       <c r="D58" t="s">
         <v>571</v>
       </c>
+      <c r="E58">
+        <v>48.137221333880603</v>
+      </c>
       <c r="F58">
-        <v>48.137221333880603</v>
-      </c>
-      <c r="G58">
         <v>11.4690853303973</v>
       </c>
-      <c r="I58" t="s">
-        <v>849</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9">
+      <c r="H58" t="s">
+        <v>847</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8">
       <c r="A59" t="s">
+        <v>848</v>
+      </c>
+      <c r="B59" t="s">
         <v>850</v>
-      </c>
-      <c r="B59" t="s">
-        <v>852</v>
       </c>
       <c r="C59" t="s">
         <v>88</v>
@@ -17927,403 +18305,403 @@
       <c r="D59" t="s">
         <v>571</v>
       </c>
+      <c r="E59">
+        <v>52.545502086676898</v>
+      </c>
       <c r="F59">
-        <v>52.545502086676898</v>
-      </c>
-      <c r="G59">
         <v>13.355599788077599</v>
       </c>
-      <c r="I59" t="s">
+      <c r="H59" t="s">
+        <v>849</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8">
+      <c r="A60" t="s">
         <v>851</v>
       </c>
-    </row>
-    <row r="60" spans="1:9">
-      <c r="A60" t="s">
-        <v>853</v>
-      </c>
       <c r="B60" t="s">
-        <v>857</v>
+        <v>855</v>
       </c>
       <c r="C60" t="s">
         <v>88</v>
       </c>
       <c r="D60" t="s">
+        <v>852</v>
+      </c>
+      <c r="E60">
+        <v>55.6774230496355</v>
+      </c>
+      <c r="F60">
+        <v>12.568158381159201</v>
+      </c>
+      <c r="G60" t="s">
+        <v>853</v>
+      </c>
+      <c r="H60" t="s">
         <v>854</v>
       </c>
-      <c r="F60">
-        <v>55.6774230496355</v>
-      </c>
-      <c r="G60">
-        <v>12.568158381159201</v>
-      </c>
-      <c r="H60" t="s">
-        <v>855</v>
-      </c>
-      <c r="I60" t="s">
+    </row>
+    <row r="61" spans="1:8">
+      <c r="A61" t="s">
         <v>856</v>
       </c>
-    </row>
-    <row r="61" spans="1:9">
-      <c r="A61" t="s">
-        <v>858</v>
-      </c>
       <c r="B61" t="s">
-        <v>859</v>
+        <v>857</v>
       </c>
       <c r="C61" t="s">
         <v>88</v>
       </c>
       <c r="D61" t="s">
+        <v>858</v>
+      </c>
+      <c r="E61">
+        <v>59.442348826981799</v>
+      </c>
+      <c r="F61">
+        <v>24.7429114165996</v>
+      </c>
+      <c r="G61" t="s">
         <v>860</v>
       </c>
-      <c r="F61">
-        <v>59.442348826981799</v>
-      </c>
-      <c r="G61">
-        <v>24.7429114165996</v>
-      </c>
       <c r="H61" t="s">
-        <v>862</v>
-      </c>
-      <c r="I61" t="s">
+        <v>859</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8">
+      <c r="A62" t="s">
         <v>861</v>
       </c>
-    </row>
-    <row r="62" spans="1:9">
-      <c r="A62" t="s">
+      <c r="B62" t="s">
         <v>863</v>
-      </c>
-      <c r="B62" t="s">
-        <v>865</v>
       </c>
       <c r="C62" t="s">
         <v>88</v>
       </c>
       <c r="D62" t="s">
+        <v>864</v>
+      </c>
+      <c r="E62">
+        <v>53.918879037622801</v>
+      </c>
+      <c r="F62">
+        <v>14.2528957989717</v>
+      </c>
+      <c r="H62" t="s">
+        <v>862</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8">
+      <c r="A63" t="s">
+        <v>865</v>
+      </c>
+      <c r="B63" t="s">
         <v>866</v>
-      </c>
-      <c r="F62">
-        <v>53.918879037622801</v>
-      </c>
-      <c r="G62">
-        <v>14.2528957989717</v>
-      </c>
-      <c r="I62" t="s">
-        <v>864</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9">
-      <c r="A63" t="s">
-        <v>867</v>
-      </c>
-      <c r="B63" t="s">
-        <v>868</v>
       </c>
       <c r="C63" t="s">
         <v>88</v>
       </c>
       <c r="D63" t="s">
-        <v>866</v>
+        <v>864</v>
+      </c>
+      <c r="E63">
+        <v>50.062293158228499</v>
       </c>
       <c r="F63">
-        <v>50.062293158228499</v>
-      </c>
-      <c r="G63">
         <v>19.9349083318201</v>
       </c>
+      <c r="G63" t="s">
+        <v>867</v>
+      </c>
       <c r="H63" t="s">
+        <v>868</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8">
+      <c r="A64" t="s">
         <v>869</v>
       </c>
-      <c r="I63" t="s">
+      <c r="B64" t="s">
         <v>870</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9">
-      <c r="A64" t="s">
-        <v>871</v>
-      </c>
-      <c r="B64" t="s">
-        <v>872</v>
       </c>
       <c r="C64" t="s">
         <v>88</v>
       </c>
       <c r="D64" t="s">
-        <v>866</v>
+        <v>864</v>
+      </c>
+      <c r="E64">
+        <v>49.299704517398801</v>
       </c>
       <c r="F64">
-        <v>49.299704517398801</v>
-      </c>
-      <c r="G64">
         <v>19.955287727156101</v>
       </c>
+      <c r="G64" t="s">
+        <v>872</v>
+      </c>
       <c r="H64" t="s">
+        <v>871</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8">
+      <c r="A65" t="s">
+        <v>873</v>
+      </c>
+      <c r="B65" t="s">
         <v>874</v>
-      </c>
-      <c r="I64" t="s">
-        <v>873</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9">
-      <c r="A65" t="s">
-        <v>875</v>
-      </c>
-      <c r="B65" t="s">
-        <v>876</v>
       </c>
       <c r="C65" t="s">
         <v>88</v>
       </c>
       <c r="D65" t="s">
+        <v>875</v>
+      </c>
+      <c r="E65">
+        <v>47.493781030775899</v>
+      </c>
+      <c r="F65">
+        <v>19.056194687097499</v>
+      </c>
+      <c r="G65" t="s">
         <v>877</v>
       </c>
-      <c r="F65">
-        <v>47.493781030775899</v>
-      </c>
-      <c r="G65">
-        <v>19.056194687097499</v>
-      </c>
       <c r="H65" t="s">
+        <v>876</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8">
+      <c r="A66" t="s">
+        <v>878</v>
+      </c>
+      <c r="B66" t="s">
         <v>879</v>
-      </c>
-      <c r="I65" t="s">
-        <v>878</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9">
-      <c r="A66" t="s">
-        <v>880</v>
-      </c>
-      <c r="B66" t="s">
-        <v>881</v>
       </c>
       <c r="C66" t="s">
         <v>88</v>
       </c>
       <c r="D66" t="s">
+        <v>880</v>
+      </c>
+      <c r="E66">
+        <v>44.450794263639096</v>
+      </c>
+      <c r="F66">
+        <v>26.086394058725201</v>
+      </c>
+      <c r="G66" t="s">
         <v>882</v>
       </c>
-      <c r="F66">
-        <v>44.450794263639096</v>
-      </c>
-      <c r="G66">
-        <v>26.086394058725201</v>
-      </c>
       <c r="H66" t="s">
+        <v>881</v>
+      </c>
+    </row>
+    <row r="67" spans="1:8">
+      <c r="A67" t="s">
+        <v>883</v>
+      </c>
+      <c r="B67" t="s">
         <v>884</v>
-      </c>
-      <c r="I66" t="s">
-        <v>883</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9">
-      <c r="A67" t="s">
-        <v>885</v>
-      </c>
-      <c r="B67" t="s">
-        <v>886</v>
       </c>
       <c r="C67" t="s">
         <v>88</v>
       </c>
       <c r="D67" t="s">
+        <v>885</v>
+      </c>
+      <c r="E67">
+        <v>37.977628330785301</v>
+      </c>
+      <c r="F67">
+        <v>23.724571665283101</v>
+      </c>
+      <c r="G67" t="s">
         <v>887</v>
       </c>
-      <c r="F67">
-        <v>37.977628330785301</v>
-      </c>
-      <c r="G67">
-        <v>23.724571665283101</v>
-      </c>
       <c r="H67" t="s">
+        <v>886</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8">
+      <c r="A68" t="s">
+        <v>888</v>
+      </c>
+      <c r="B68" t="s">
         <v>889</v>
-      </c>
-      <c r="I67" t="s">
-        <v>888</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9">
-      <c r="A68" t="s">
-        <v>890</v>
-      </c>
-      <c r="B68" t="s">
-        <v>891</v>
       </c>
       <c r="C68" t="s">
         <v>88</v>
       </c>
       <c r="D68" t="s">
+        <v>890</v>
+      </c>
+      <c r="E68">
+        <v>42.640669732898502</v>
+      </c>
+      <c r="F68">
+        <v>18.1088954965102</v>
+      </c>
+      <c r="G68" t="s">
         <v>892</v>
       </c>
-      <c r="F68">
-        <v>42.640669732898502</v>
-      </c>
-      <c r="G68">
-        <v>18.1088954965102</v>
-      </c>
       <c r="H68" t="s">
+        <v>891</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8">
+      <c r="A69" t="s">
+        <v>893</v>
+      </c>
+      <c r="B69" t="s">
         <v>894</v>
-      </c>
-      <c r="I68" t="s">
-        <v>893</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9">
-      <c r="A69" t="s">
-        <v>895</v>
-      </c>
-      <c r="B69" t="s">
-        <v>896</v>
       </c>
       <c r="C69" t="s">
         <v>88</v>
       </c>
       <c r="D69" t="s">
-        <v>892</v>
+        <v>890</v>
+      </c>
+      <c r="E69">
+        <v>43.509153771859999</v>
       </c>
       <c r="F69">
-        <v>43.509153771859999</v>
-      </c>
-      <c r="G69">
         <v>16.439297745722001</v>
       </c>
+      <c r="G69" t="s">
+        <v>896</v>
+      </c>
       <c r="H69" t="s">
+        <v>895</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8">
+      <c r="A70" t="s">
+        <v>897</v>
+      </c>
+      <c r="B70" t="s">
         <v>898</v>
-      </c>
-      <c r="I69" t="s">
-        <v>897</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9">
-      <c r="A70" t="s">
-        <v>899</v>
-      </c>
-      <c r="B70" t="s">
-        <v>900</v>
       </c>
       <c r="C70" t="s">
         <v>88</v>
       </c>
       <c r="D70" t="s">
-        <v>892</v>
+        <v>890</v>
+      </c>
+      <c r="E70">
+        <v>44.113881823968498</v>
       </c>
       <c r="F70">
-        <v>44.113881823968498</v>
-      </c>
-      <c r="G70">
         <v>15.226994459353801</v>
       </c>
-      <c r="I70" t="s">
-        <v>901</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9">
+      <c r="H70" t="s">
+        <v>899</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8">
       <c r="A71" t="s">
-        <v>902</v>
+        <v>900</v>
       </c>
       <c r="B71" t="s">
-        <v>896</v>
+        <v>894</v>
       </c>
       <c r="C71" t="s">
         <v>88</v>
       </c>
       <c r="D71" t="s">
+        <v>890</v>
+      </c>
+      <c r="E71">
+        <v>43.508491462566703</v>
+      </c>
+      <c r="F71">
+        <v>16.438738703728799</v>
+      </c>
+      <c r="G71" t="s">
         <v>892</v>
       </c>
-      <c r="F71">
-        <v>43.508491462566703</v>
-      </c>
-      <c r="G71">
-        <v>16.438738703728799</v>
-      </c>
       <c r="H71" t="s">
-        <v>894</v>
-      </c>
-      <c r="I71" t="s">
-        <v>903</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9">
+        <v>901</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8">
       <c r="A72" t="s">
-        <v>890</v>
+        <v>888</v>
       </c>
       <c r="B72" t="s">
-        <v>891</v>
+        <v>889</v>
       </c>
       <c r="C72" t="s">
         <v>88</v>
       </c>
       <c r="D72" t="s">
+        <v>890</v>
+      </c>
+      <c r="E72">
+        <v>42.641448880157299</v>
+      </c>
+      <c r="F72">
+        <v>18.108708858081901</v>
+      </c>
+      <c r="G72" t="s">
         <v>892</v>
       </c>
-      <c r="F72">
-        <v>42.641448880157299</v>
-      </c>
-      <c r="G72">
-        <v>18.108708858081901</v>
-      </c>
       <c r="H72" t="s">
-        <v>894</v>
-      </c>
-      <c r="I72" t="s">
+        <v>902</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8">
+      <c r="A73" t="s">
+        <v>903</v>
+      </c>
+      <c r="B73" t="s">
         <v>904</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9">
-      <c r="A73" t="s">
-        <v>905</v>
-      </c>
-      <c r="B73" t="s">
-        <v>906</v>
       </c>
       <c r="C73" t="s">
         <v>88</v>
       </c>
       <c r="D73" t="s">
-        <v>892</v>
+        <v>890</v>
+      </c>
+      <c r="E73">
+        <v>45.815999034471403</v>
       </c>
       <c r="F73">
-        <v>45.815999034471403</v>
-      </c>
-      <c r="G73">
         <v>15.9757907599175</v>
       </c>
+      <c r="G73" t="s">
+        <v>906</v>
+      </c>
       <c r="H73" t="s">
+        <v>905</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8">
+      <c r="A74" t="s">
+        <v>907</v>
+      </c>
+      <c r="B74" t="s">
         <v>908</v>
-      </c>
-      <c r="I73" t="s">
-        <v>907</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9">
-      <c r="A74" t="s">
-        <v>909</v>
-      </c>
-      <c r="B74" t="s">
-        <v>910</v>
       </c>
       <c r="C74" t="s">
         <v>88</v>
       </c>
       <c r="D74" t="s">
+        <v>909</v>
+      </c>
+      <c r="E74">
+        <v>46.052500560187703</v>
+      </c>
+      <c r="F74">
+        <v>14.5051018908164</v>
+      </c>
+      <c r="H74" t="s">
+        <v>910</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8">
+      <c r="A75" t="s">
         <v>911</v>
       </c>
-      <c r="F74">
-        <v>46.052500560187703</v>
-      </c>
-      <c r="G74">
-        <v>14.5051018908164</v>
-      </c>
-      <c r="I74" t="s">
+      <c r="B75" t="s">
         <v>912</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9">
-      <c r="A75" t="s">
-        <v>913</v>
-      </c>
-      <c r="B75" t="s">
-        <v>914</v>
       </c>
       <c r="C75" t="s">
         <v>88</v>
@@ -18331,20 +18709,20 @@
       <c r="D75" t="s">
         <v>314</v>
       </c>
+      <c r="E75">
+        <v>45.459955873306903</v>
+      </c>
       <c r="F75">
-        <v>45.459955873306903</v>
-      </c>
-      <c r="G75">
         <v>9.1817341590042698</v>
       </c>
+      <c r="G75" t="s">
+        <v>914</v>
+      </c>
       <c r="H75" t="s">
-        <v>916</v>
-      </c>
-      <c r="I75" t="s">
-        <v>915</v>
-      </c>
-    </row>
-    <row r="76" spans="1:9">
+        <v>913</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8">
       <c r="A76" t="s">
         <v>318</v>
       </c>
@@ -18357,20 +18735,20 @@
       <c r="D76" t="s">
         <v>314</v>
       </c>
+      <c r="E76">
+        <v>45.437711653191698</v>
+      </c>
       <c r="F76">
-        <v>45.437711653191698</v>
-      </c>
-      <c r="G76">
         <v>12.3372600700623</v>
       </c>
+      <c r="G76" t="s">
+        <v>916</v>
+      </c>
       <c r="H76" t="s">
-        <v>918</v>
-      </c>
-      <c r="I76" t="s">
-        <v>917</v>
-      </c>
-    </row>
-    <row r="77" spans="1:9">
+        <v>915</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8">
       <c r="A77" t="s">
         <v>318</v>
       </c>
@@ -18383,20 +18761,20 @@
       <c r="D77" t="s">
         <v>314</v>
       </c>
+      <c r="E77">
+        <v>45.4357857236336</v>
+      </c>
       <c r="F77">
-        <v>45.4357857236336</v>
-      </c>
-      <c r="G77">
         <v>12.338114341246699</v>
       </c>
+      <c r="G77" t="s">
+        <v>916</v>
+      </c>
       <c r="H77" t="s">
-        <v>918</v>
-      </c>
-      <c r="I77" t="s">
-        <v>919</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9">
+        <v>917</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8">
       <c r="A78" t="s">
         <v>318</v>
       </c>
@@ -18409,25 +18787,25 @@
       <c r="D78" t="s">
         <v>314</v>
       </c>
+      <c r="E78">
+        <v>45.440782321598597</v>
+      </c>
       <c r="F78">
-        <v>45.440782321598597</v>
-      </c>
-      <c r="G78">
         <v>12.3352324126277</v>
+      </c>
+      <c r="G78" t="s">
+        <v>916</v>
       </c>
       <c r="H78" t="s">
         <v>918</v>
       </c>
-      <c r="I78" t="s">
+    </row>
+    <row r="79" spans="1:8">
+      <c r="A79" t="s">
+        <v>919</v>
+      </c>
+      <c r="B79" t="s">
         <v>920</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9">
-      <c r="A79" t="s">
-        <v>921</v>
-      </c>
-      <c r="B79" t="s">
-        <v>922</v>
       </c>
       <c r="C79" t="s">
         <v>88</v>
@@ -18435,25 +18813,25 @@
       <c r="D79" t="s">
         <v>314</v>
       </c>
+      <c r="E79">
+        <v>43.770867429289197</v>
+      </c>
       <c r="F79">
-        <v>43.770867429289197</v>
-      </c>
-      <c r="G79">
         <v>11.2554047899725</v>
       </c>
+      <c r="G79" t="s">
+        <v>922</v>
+      </c>
       <c r="H79" t="s">
+        <v>921</v>
+      </c>
+    </row>
+    <row r="80" spans="1:8">
+      <c r="A80" t="s">
+        <v>923</v>
+      </c>
+      <c r="B80" t="s">
         <v>924</v>
-      </c>
-      <c r="I79" t="s">
-        <v>923</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9">
-      <c r="A80" t="s">
-        <v>925</v>
-      </c>
-      <c r="B80" t="s">
-        <v>926</v>
       </c>
       <c r="C80" t="s">
         <v>88</v>
@@ -18461,22 +18839,22 @@
       <c r="D80" t="s">
         <v>314</v>
       </c>
+      <c r="E80">
+        <v>43.935609314633197</v>
+      </c>
       <c r="F80">
-        <v>43.935609314633197</v>
-      </c>
-      <c r="G80">
         <v>12.446803482111701</v>
       </c>
+      <c r="G80" t="s">
+        <v>926</v>
+      </c>
       <c r="H80" t="s">
-        <v>928</v>
-      </c>
-      <c r="I80" t="s">
+        <v>925</v>
+      </c>
+    </row>
+    <row r="81" spans="1:8">
+      <c r="A81" t="s">
         <v>927</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9">
-      <c r="A81" t="s">
-        <v>929</v>
       </c>
       <c r="B81" t="s">
         <v>325</v>
@@ -18487,20 +18865,20 @@
       <c r="D81" t="s">
         <v>314</v>
       </c>
+      <c r="E81">
+        <v>41.904766191071197</v>
+      </c>
       <c r="F81">
-        <v>41.904766191071197</v>
-      </c>
-      <c r="G81">
         <v>12.478982679078699</v>
       </c>
+      <c r="G81" t="s">
+        <v>929</v>
+      </c>
       <c r="H81" t="s">
-        <v>931</v>
-      </c>
-      <c r="I81" t="s">
-        <v>930</v>
-      </c>
-    </row>
-    <row r="82" spans="1:9">
+        <v>928</v>
+      </c>
+    </row>
+    <row r="82" spans="1:8">
       <c r="A82" t="s">
         <v>327</v>
       </c>
@@ -18513,25 +18891,25 @@
       <c r="D82" t="s">
         <v>314</v>
       </c>
+      <c r="E82">
+        <v>41.900532853153301</v>
+      </c>
       <c r="F82">
-        <v>41.900532853153301</v>
-      </c>
-      <c r="G82">
         <v>12.468392352353</v>
       </c>
+      <c r="G82" t="s">
+        <v>931</v>
+      </c>
       <c r="H82" t="s">
+        <v>930</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8">
+      <c r="A83" t="s">
         <v>933</v>
       </c>
-      <c r="I82" t="s">
-        <v>932</v>
-      </c>
-    </row>
-    <row r="83" spans="1:9">
-      <c r="A83" t="s">
-        <v>935</v>
-      </c>
       <c r="B83" t="s">
-        <v>936</v>
+        <v>934</v>
       </c>
       <c r="C83" t="s">
         <v>88</v>
@@ -18539,19 +18917,19 @@
       <c r="D83" t="s">
         <v>134</v>
       </c>
+      <c r="E83">
+        <v>32.922455623738799</v>
+      </c>
       <c r="F83">
-        <v>32.922455623738799</v>
-      </c>
-      <c r="G83">
         <v>35.070240555908498</v>
       </c>
-      <c r="I83" t="s">
-        <v>934</v>
-      </c>
-    </row>
-    <row r="84" spans="1:9">
+      <c r="H83" t="s">
+        <v>932</v>
+      </c>
+    </row>
+    <row r="84" spans="1:8">
       <c r="A84" t="s">
-        <v>937</v>
+        <v>935</v>
       </c>
       <c r="B84" t="s">
         <v>133</v>
@@ -18562,25 +18940,25 @@
       <c r="D84" t="s">
         <v>134</v>
       </c>
+      <c r="E84">
+        <v>32.070936261991797</v>
+      </c>
       <c r="F84">
-        <v>32.070936261991797</v>
-      </c>
-      <c r="G84">
         <v>34.772256917509203</v>
       </c>
+      <c r="G84" t="s">
+        <v>936</v>
+      </c>
       <c r="H84" t="s">
-        <v>938</v>
-      </c>
-      <c r="I84" t="s">
+        <v>937</v>
+      </c>
+    </row>
+    <row r="85" spans="1:8">
+      <c r="A85" t="s">
         <v>939</v>
       </c>
-    </row>
-    <row r="85" spans="1:9">
-      <c r="A85" t="s">
-        <v>941</v>
-      </c>
       <c r="B85" t="s">
-        <v>942</v>
+        <v>940</v>
       </c>
       <c r="C85" t="s">
         <v>88</v>
@@ -18588,69 +18966,144 @@
       <c r="D85" t="s">
         <v>134</v>
       </c>
+      <c r="E85">
+        <v>31.241277726774001</v>
+      </c>
       <c r="F85">
-        <v>31.241277726774001</v>
-      </c>
-      <c r="G85">
         <v>34.796193268741902</v>
       </c>
+      <c r="G85" t="s">
+        <v>941</v>
+      </c>
       <c r="H85" t="s">
-        <v>943</v>
-      </c>
-      <c r="I85" t="s">
-        <v>940</v>
-      </c>
-    </row>
-    <row r="86" spans="1:9">
+        <v>938</v>
+      </c>
+    </row>
+    <row r="86" spans="1:8">
       <c r="A86" t="s">
-        <v>944</v>
+        <v>942</v>
       </c>
       <c r="B86" t="s">
-        <v>948</v>
+        <v>946</v>
       </c>
       <c r="C86" t="s">
         <v>88</v>
       </c>
       <c r="D86" t="s">
+        <v>945</v>
+      </c>
+      <c r="E86">
+        <v>30.020802135695298</v>
+      </c>
+      <c r="F86">
+        <v>31.0030222660539</v>
+      </c>
+      <c r="G86" t="s">
+        <v>944</v>
+      </c>
+      <c r="H86" t="s">
+        <v>943</v>
+      </c>
+    </row>
+    <row r="87" spans="1:8">
+      <c r="A87" t="s">
         <v>947</v>
       </c>
-      <c r="F86">
-        <v>30.020802135695298</v>
-      </c>
-      <c r="G86">
-        <v>31.0030222660539</v>
-      </c>
-      <c r="H86" t="s">
-        <v>946</v>
-      </c>
-      <c r="I86" t="s">
-        <v>945</v>
-      </c>
-    </row>
-    <row r="87" spans="1:9">
-      <c r="A87" t="s">
-        <v>949</v>
-      </c>
       <c r="B87" t="s">
-        <v>950</v>
+        <v>948</v>
       </c>
       <c r="C87" t="s">
         <v>88</v>
       </c>
       <c r="D87" t="s">
+        <v>949</v>
+      </c>
+      <c r="E87">
+        <v>25.215850937399502</v>
+      </c>
+      <c r="F87">
+        <v>55.250893152761897</v>
+      </c>
+      <c r="G87" t="s">
         <v>951</v>
       </c>
-      <c r="F87">
-        <v>25.215850937399502</v>
-      </c>
-      <c r="G87">
-        <v>55.250893152761897</v>
-      </c>
       <c r="H87" t="s">
+        <v>950</v>
+      </c>
+    </row>
+    <row r="88" spans="1:8">
+      <c r="A88" t="s">
+        <v>952</v>
+      </c>
+      <c r="B88" t="s">
+        <v>524</v>
+      </c>
+      <c r="C88" t="s">
+        <v>88</v>
+      </c>
+      <c r="D88" t="s">
+        <v>649</v>
+      </c>
+      <c r="E88">
+        <v>52.366857518563002</v>
+      </c>
+      <c r="F88">
+        <v>4.8953030348517501</v>
+      </c>
+      <c r="G88" t="s">
         <v>953</v>
       </c>
-      <c r="I87" t="s">
-        <v>952</v>
+      <c r="H88" t="s">
+        <v>954</v>
+      </c>
+    </row>
+    <row r="89" spans="1:8">
+      <c r="A89" t="s">
+        <v>955</v>
+      </c>
+      <c r="B89" t="s">
+        <v>957</v>
+      </c>
+      <c r="C89" t="s">
+        <v>88</v>
+      </c>
+      <c r="D89" t="s">
+        <v>826</v>
+      </c>
+      <c r="E89">
+        <v>51.279214386945199</v>
+      </c>
+      <c r="F89">
+        <v>1.0811299370738801</v>
+      </c>
+      <c r="H89" t="s">
+        <v>956</v>
+      </c>
+    </row>
+    <row r="90" spans="1:8">
+      <c r="A90" t="s">
+        <v>960</v>
+      </c>
+      <c r="B90" t="s">
+        <v>958</v>
+      </c>
+      <c r="C90" t="s">
+        <v>88</v>
+      </c>
+      <c r="D90" t="s">
+        <v>961</v>
+      </c>
+      <c r="E90">
+        <v>52.062570092405103</v>
+      </c>
+      <c r="F90">
+        <v>-9.5108505116264705</v>
+      </c>
+      <c r="G90" t="s">
+        <v>962</v>
+      </c>
+      <c r="H90" t="s">
+        <v>959</v>
       </c>
     </row>
   </sheetData>
@@ -18664,7 +19117,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{54904E20-3C5D-490F-BCF5-E5014AEEFD29}">
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="12.33203125" customWidth="1"/>
@@ -18672,7 +19125,7 @@
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
-        <v>702</v>
+        <v>701</v>
       </c>
     </row>
     <row r="2" spans="1:1">
@@ -18687,12 +19140,12 @@
     </row>
     <row r="4" spans="1:1">
       <c r="A4" t="s">
-        <v>703</v>
+        <v>702</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" t="s">
-        <v>295</v>
+        <v>972</v>
       </c>
     </row>
     <row r="6" spans="1:1">
@@ -18702,7 +19155,12 @@
     </row>
     <row r="7" spans="1:1">
       <c r="A7" t="s">
-        <v>740</v>
+        <v>738</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>973</v>
       </c>
     </row>
   </sheetData>

</xml_diff>